<commit_message>
Add external recovery and cruise guards
</commit_message>
<xml_diff>
--- a/Database/eBay_listing.xlsx
+++ b/Database/eBay_listing.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH283"/>
+  <dimension ref="A1:AJ283"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -590,6 +590,16 @@
           <t>Metadata_Sync_Status</t>
         </is>
       </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>SEO_Strike_Timestamp</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>SEO_Strike_Group</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -7733,12 +7743,12 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Celestial Koi Constellation 4pc 6x6 Kiss-Cut Sticker Zen Aesthetic Laptop Vinyl</t>
+          <t>Deep Work Sticker Set Celestial Koi Constellation 4pc 6x6 Vinyl Laptop Journal</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>&lt;h2&gt;Celestial Koi Constellation Kiss-Cut Sticker&lt;/h2&gt;&lt;p&gt;Bring calm and balance into your daily routine with this Celestial Koi Constellation zen aesthetic kiss-cut sticker.&lt;/p&gt;&lt;p&gt;Designed for study rooms, creative workspaces, shelves, gallery walls, and collectible aesthetic decor, this sticker blends niche aesthetic appeal with collectible mentor-grade artwork.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 6x6 kiss-cut sheet with 4 individual sticker designs.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; Durable kiss-cut vinyl sticker sheet with waterproof finish.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Size:&lt;/strong&gt; 6x6 kiss-cut sheet with four coordinated designs.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Zen Mentor-Grade; Zen aesthetic.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;DNA Profile:&lt;/strong&gt; A cosmic koi fish swimming through space, body constructed from translucent moonstone scales with imperial jade fins, ink-wash nebula trailing from tail, floating Daoist Fulu talisman fragments following its path, ethereal bioluminescence along spine, zen-mythic aesthetic, , , , , , person, text, watermark&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Best For:&lt;/strong&gt; mindfulness lovers, minimalists, journal keepers, yoga enthusiasts, and peaceful room setups.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;SEO Keywords:&lt;/strong&gt; koi fish sticker, celestial koi, moonstone fish, jade koi, zen fish, cosmic creature, spiritual koi, translucent scales, Daoist symbol, bioluminescent fish&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the actual product customers receive. Additional images are bonus concept/detail reference images and do not represent extra products or selectable variations.&lt;/p&gt;&lt;p&gt;Complete the collection with matching Alchemy pieces.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Sticker-Zen-0072&lt;/small&gt;&lt;/p&gt;</t>
+          <t>&lt;h2&gt;Deep Work Sticker Set Celestial Koi Constellation 4pc 6x6 Vinyl Laptop Journal&lt;/h2&gt;&lt;p&gt;This is part of a fast A/B traffic test built around higher-intent buyer scenes: laptops, journals, planners, reading notebooks, book nooks, and focused desk setups. The style leans into smoky jade accents, quiet desk mood, sharp die-cut presentation, and giftable detail, avoiding generic mass-market wording.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One physical 4pc 6x6 kiss-cut vinyl sticker sheet, produced on demand through Printify.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Visual Lane:&lt;/strong&gt; A Deep Work Sticker Set&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Zen with Quiet Jade / Deep Work positioning.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the physical product customers receive. Additional gallery images are concept, detail, or collection-reference views and are not extra products or selectable variations.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Sticker-Zen-0072&lt;/small&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -7794,6 +7804,21 @@
       <c r="Q73" t="inlineStr">
         <is>
           <t>69f26281feceb0d66c042ce7</t>
+        </is>
+      </c>
+      <c r="AH73" t="inlineStr">
+        <is>
+          <t>SEO_STRIKE_SYNCED_PRINTIFY_DRAFT</t>
+        </is>
+      </c>
+      <c r="AI73" t="inlineStr">
+        <is>
+          <t>2026-05-07 02:06:35 -0400</t>
+        </is>
+      </c>
+      <c r="AJ73" t="inlineStr">
+        <is>
+          <t>A_DEEP_WORK_STICKER_SET</t>
         </is>
       </c>
     </row>
@@ -7820,12 +7845,12 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Sacred Singing Bowl Mindful Zen 4pc 6x6 Vinyl Sticker Yoga Minimalist Gift Gift</t>
+          <t>Book Nook Laptop Decals Sacred Singing Bowl Yoga Minimalist 4pc 6x6 Kiss-Cut</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>&lt;h2&gt;Sacred Singing Bowl | Kiss-Cut Sticker&lt;/h2&gt;&lt;p&gt;Add a quiet mindful accent to your workspace with this Sacred Singing Bowl kiss-cut sticker. The artwork is built around a focused visual DNA profile, so each piece feels like part of a coherent small-batch collection.&lt;/p&gt;&lt;p&gt;Use it for laptops, notebooks, reading corners, desk setups, gallery shelves, and gift bundles. The composition favors readable detail, strong mood, and giftable niche appeal without generic mass-market styling.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 6x6 kiss-cut sheet with 4 individual sticker designs.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; Durable kiss-cut vinyl sticker sheet with waterproof finish.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Size:&lt;/strong&gt; 6x6 kiss-cut sheet with four coordinated designs.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Zen Mentor-Grade; Zen aesthetic.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;DNA Profile:&lt;/strong&gt; A ceremonial Tibetan singing bowl made of imperial jade with translucent moonstone rim, sound waves visualized as ink-wash nebula emanating outward, floating Daoist Fulu talisman fragments suspended above, ethereal bioluminescence pulsing from bowl interior, zen-mythic aesthetic, , , , , , person, text, watermark&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Best For:&lt;/strong&gt; meditation fans, calm desk setups, notebook collectors, and gift buyers who like clean aesthetics.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;SEO Keywords:&lt;/strong&gt; singing bowl, meditation bowl, jade bowl, ritual instrument, zen bowl, spiritual tool, moonstone rim, Daoist ceremony, bioluminescent sound, sacred artifact&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the actual product customers receive. Additional images are bonus concept/detail reference images and do not represent extra products or selectable variations.&lt;/p&gt;&lt;p&gt;Pair it with related OpenClaw pieces for a coordinated collection.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Sticker-Zen-0073&lt;/small&gt;&lt;/p&gt;</t>
+          <t>&lt;h2&gt;Book Nook Laptop Decals Sacred Singing Bowl Yoga Minimalist 4pc 6x6 Kiss-Cut&lt;/h2&gt;&lt;p&gt;This is part of a fast A/B traffic test built around higher-intent buyer scenes: laptops, journals, planners, reading notebooks, book nooks, and focused desk setups. The style leans into smoky jade accents, quiet desk mood, sharp die-cut presentation, and giftable detail, avoiding generic mass-market wording.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One physical 4pc 6x6 kiss-cut vinyl sticker sheet, produced on demand through Printify.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Visual Lane:&lt;/strong&gt; B Book Nook Laptop Decals&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Zen with Quiet Jade / Deep Work positioning.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the physical product customers receive. Additional gallery images are concept, detail, or collection-reference views and are not extra products or selectable variations.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Sticker-Zen-0073&lt;/small&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -7881,6 +7906,21 @@
       <c r="Q74" t="inlineStr">
         <is>
           <t>69f262db5269e3325904b893</t>
+        </is>
+      </c>
+      <c r="AH74" t="inlineStr">
+        <is>
+          <t>SEO_STRIKE_SYNCED_PRINTIFY_DRAFT</t>
+        </is>
+      </c>
+      <c r="AI74" t="inlineStr">
+        <is>
+          <t>2026-05-07 02:06:35 -0400</t>
+        </is>
+      </c>
+      <c r="AJ74" t="inlineStr">
+        <is>
+          <t>B_BOOK_NOOK_LAPTOP_DECALS</t>
         </is>
       </c>
     </row>
@@ -7907,12 +7947,12 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Minimal Zen Bamboo Pagoda Relic 4pc 6x6 Sticker Sheet Serene Mindful Clean Gift</t>
+          <t>Deep Work Sticker Set Bamboo Pagoda Relic Serene Clean 4pc 6x6 Vinyl Laptop</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>&lt;h2&gt;Bamboo Pagoda Relic - Kiss-Cut Sticker&lt;/h2&gt;&lt;p&gt;A polished Zen aesthetic piece for students, remote workers, yoga lovers, and anyone building a serene everyday space. Designed for peaceful desks, journals, and small rituals, this Bamboo Pagoda Relic kiss-cut sticker carries a clean Zen mood.&lt;/p&gt;&lt;p&gt;The design works well across journal spreads, library shelves, dorm rooms, studio desks, and cozy personal collections, while the title, material notes, and DNA profile stay specific for easy comparison.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 6x6 kiss-cut sheet with 4 individual sticker designs.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; Durable kiss-cut vinyl sticker sheet with waterproof finish.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Size:&lt;/strong&gt; 6x6 kiss-cut sheet with four coordinated designs.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Zen Mentor-Grade; Zen aesthetic.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;DNA Profile:&lt;/strong&gt; A miniature five-tier pagoda structure crafted from imperial jade beams and translucent moonstone panels, ink-wash nebula swirling around base, floating Daoist Fulu talisman fragments at each tier level, ethereal bioluminescence glowing from windows, zen-mythic aesthetic, , , , , , person, text, watermark&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Best For:&lt;/strong&gt; students, remote workers, yoga lovers, and anyone building a serene everyday space.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;SEO Keywords:&lt;/strong&gt; pagoda sticker, jade pagoda, moonstone architecture, zen temple, spiritual building, celestial pagoda, architectural relic, Daoist shrine, bioluminescent tower, sacred structure&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the actual product customers receive. Additional images are bonus concept/detail reference images and do not represent extra products or selectable variations.&lt;/p&gt;&lt;p&gt;Saved under the reference SKU below for easy collector matching.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Sticker-Zen-0074&lt;/small&gt;&lt;/p&gt;</t>
+          <t>&lt;h2&gt;Deep Work Sticker Set Bamboo Pagoda Relic Serene Clean 4pc 6x6 Vinyl Laptop&lt;/h2&gt;&lt;p&gt;This is part of a fast A/B traffic test built around higher-intent buyer scenes: laptops, journals, planners, reading notebooks, book nooks, and focused desk setups. The style leans into smoky jade accents, quiet desk mood, sharp die-cut presentation, and giftable detail, avoiding generic mass-market wording.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One physical 4pc 6x6 kiss-cut vinyl sticker sheet, produced on demand through Printify.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Visual Lane:&lt;/strong&gt; A Deep Work Sticker Set&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Zen with Quiet Jade / Deep Work positioning.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the physical product customers receive. Additional gallery images are concept, detail, or collection-reference views and are not extra products or selectable variations.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Sticker-Zen-0074&lt;/small&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -7968,6 +8008,21 @@
       <c r="Q75" t="inlineStr">
         <is>
           <t>69f263729b469f716d0e7409</t>
+        </is>
+      </c>
+      <c r="AH75" t="inlineStr">
+        <is>
+          <t>SEO_STRIKE_SYNCED_PRINTIFY_DRAFT</t>
+        </is>
+      </c>
+      <c r="AI75" t="inlineStr">
+        <is>
+          <t>2026-05-07 02:06:35 -0400</t>
+        </is>
+      </c>
+      <c r="AJ75" t="inlineStr">
+        <is>
+          <t>A_DEEP_WORK_STICKER_SET</t>
         </is>
       </c>
     </row>
@@ -7994,12 +8049,12 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Mindful Zen Dragon Pearl Talisman 4pc 6x6 Vinyl Sticker Laptop Journal Gift</t>
+          <t>Book Nook Laptop Decals Dragon Pearl Talisman 4pc 6x6 Kiss-Cut Sticker Set Gift</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>&lt;h2&gt;Dragon Pearl Talisman | Kiss-Cut Sticker&lt;/h2&gt;&lt;p&gt;Add a quiet mindful accent to your workspace with this Dragon Pearl Talisman kiss-cut sticker. The artwork is built around a focused visual DNA profile, so each piece feels like part of a coherent small-batch collection.&lt;/p&gt;&lt;p&gt;Use it for laptops, notebooks, reading corners, desk setups, gallery shelves, and gift bundles. The composition favors readable detail, strong mood, and giftable niche appeal without generic mass-market styling.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 6x6 kiss-cut sheet with 4 individual sticker designs.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; Durable kiss-cut vinyl sticker sheet with waterproof finish.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Size:&lt;/strong&gt; 6x6 kiss-cut sheet with four coordinated designs.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Zen Mentor-Grade; Zen aesthetic.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;DNA Profile:&lt;/strong&gt; An ancient dragon pearl talisman seal with imperial jade dragon coiled around translucent moonstone sphere, ink-wash nebula contained within the orb, floating Daoist Fulu talisman fragments forming protective circle, ethereal bioluminescence radiating from pearl core, zen-mythic aesthetic, , , , , , person, text, watermark&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Best For:&lt;/strong&gt; meditation fans, calm desk setups, notebook collectors, and gift buyers who like clean aesthetics.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;SEO Keywords:&lt;/strong&gt; dragon pearl, jade talisman, moonstone orb, spiritual seal, zen amulet, celestial talisman, dragon artifact, Daoist seal, bioluminescent pearl, protection charm&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the actual product customers receive. Additional images are bonus concept/detail reference images and do not represent extra products or selectable variations.&lt;/p&gt;&lt;p&gt;Pair it with related OpenClaw pieces for a coordinated collection.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Sticker-Zen-0075&lt;/small&gt;&lt;/p&gt;</t>
+          <t>&lt;h2&gt;Book Nook Laptop Decals Dragon Pearl Talisman 4pc 6x6 Kiss-Cut Sticker Set Gift&lt;/h2&gt;&lt;p&gt;This is part of a fast A/B traffic test built around higher-intent buyer scenes: laptops, journals, planners, reading notebooks, book nooks, and focused desk setups. The style leans into smoky jade accents, quiet desk mood, sharp die-cut presentation, and giftable detail, avoiding generic mass-market wording.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One physical 4pc 6x6 kiss-cut vinyl sticker sheet, produced on demand through Printify.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Visual Lane:&lt;/strong&gt; B Book Nook Laptop Decals&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Zen with Quiet Jade / Deep Work positioning.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the physical product customers receive. Additional gallery images are concept, detail, or collection-reference views and are not extra products or selectable variations.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Sticker-Zen-0075&lt;/small&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -8055,6 +8110,21 @@
       <c r="Q76" t="inlineStr">
         <is>
           <t>69f26426671cc7c7960b3f3d</t>
+        </is>
+      </c>
+      <c r="AH76" t="inlineStr">
+        <is>
+          <t>SEO_STRIKE_SYNCED_PRINTIFY_DRAFT</t>
+        </is>
+      </c>
+      <c r="AI76" t="inlineStr">
+        <is>
+          <t>2026-05-07 02:06:35 -0400</t>
+        </is>
+      </c>
+      <c r="AJ76" t="inlineStr">
+        <is>
+          <t>B_BOOK_NOOK_LAPTOP_DECALS</t>
         </is>
       </c>
     </row>
@@ -8081,12 +8151,12 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Moonlit Mountain Shrine Mindful Zen 4pc 6x6 Vinyl Sticker Yoga Minimalist Gift</t>
+          <t>Deep Work Sticker Set Moonlit Mountain Shrine Yoga Minimalist 4pc 6x6 Vinyl</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>&lt;h2&gt;Moonlit Mountain Shrine | Kiss-Cut Sticker&lt;/h2&gt;&lt;p&gt;Add a quiet mindful accent to your workspace with this Moonlit Mountain Shrine kiss-cut sticker. The artwork is built around a focused visual DNA profile, so each piece feels like part of a coherent small-batch collection.&lt;/p&gt;&lt;p&gt;Use it for laptops, notebooks, reading corners, desk setups, gallery shelves, and gift bundles. The composition favors readable detail, strong mood, and giftable niche appeal without generic mass-market styling.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 6x6 kiss-cut sheet with 4 individual sticker designs.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; Durable kiss-cut vinyl sticker sheet with waterproof finish.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Size:&lt;/strong&gt; 6x6 kiss-cut sheet with four coordinated designs.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Zen Mentor-Grade; Zen aesthetic.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;DNA Profile:&lt;/strong&gt; A miniature mountain landscape with imperial jade peaks and translucent moonstone mist layers, tiny shrine structure at summit, ink-wash nebula forming clouds, floating Daoist Fulu talisman fragments drifting through scene, ethereal bioluminescence from mountain caves, zen-mythic aesthetic, , , , , , person, text, watermark&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Best For:&lt;/strong&gt; meditation fans, calm desk setups, notebook collectors, and gift buyers who like clean aesthetics.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;SEO Keywords:&lt;/strong&gt; mountain shrine, jade landscape, moonstone mist, zen scenery, spiritual mountain, celestial landscape, micro scene, Daoist shrine, bioluminescent caves, sacred geography&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the actual product customers receive. Additional images are bonus concept/detail reference images and do not represent extra products or selectable variations.&lt;/p&gt;&lt;p&gt;Pair it with related OpenClaw pieces for a coordinated collection.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Sticker-Zen-0076&lt;/small&gt;&lt;/p&gt;</t>
+          <t>&lt;h2&gt;Deep Work Sticker Set Moonlit Mountain Shrine Yoga Minimalist 4pc 6x6 Vinyl&lt;/h2&gt;&lt;p&gt;This is part of a fast A/B traffic test built around higher-intent buyer scenes: laptops, journals, planners, reading notebooks, book nooks, and focused desk setups. The style leans into smoky jade accents, quiet desk mood, sharp die-cut presentation, and giftable detail, avoiding generic mass-market wording.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One physical 4pc 6x6 kiss-cut vinyl sticker sheet, produced on demand through Printify.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Visual Lane:&lt;/strong&gt; A Deep Work Sticker Set&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Zen with Quiet Jade / Deep Work positioning.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the physical product customers receive. Additional gallery images are concept, detail, or collection-reference views and are not extra products or selectable variations.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Sticker-Zen-0076&lt;/small&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -8142,6 +8212,21 @@
       <c r="Q77" t="inlineStr">
         <is>
           <t>69f264df357398ded80f6a3a</t>
+        </is>
+      </c>
+      <c r="AH77" t="inlineStr">
+        <is>
+          <t>SEO_STRIKE_SYNCED_PRINTIFY_DRAFT</t>
+        </is>
+      </c>
+      <c r="AI77" t="inlineStr">
+        <is>
+          <t>2026-05-07 02:06:35 -0400</t>
+        </is>
+      </c>
+      <c r="AJ77" t="inlineStr">
+        <is>
+          <t>A_DEEP_WORK_STICKER_SET</t>
         </is>
       </c>
     </row>
@@ -8414,12 +8499,12 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Celestial Koi Ascension Minimal Zen 4pc 6x6 Kiss-Cut Vinyl Desk Collector Decor</t>
+          <t>Deep Work Sticker Set Celestial Koi Ascension Collector 4pc 6x6 Vinyl Laptop</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>&lt;h2&gt;Celestial Koi Ascension - Kiss-Cut Sticker&lt;/h2&gt;&lt;p&gt;A polished Zen aesthetic piece for students, remote workers, yoga lovers, and anyone building a serene everyday space. Designed for peaceful desks, journals, and small rituals, this Celestial Koi Ascension kiss-cut sticker carries a clean Zen mood.&lt;/p&gt;&lt;p&gt;The design works well across journal spreads, library shelves, dorm rooms, studio desks, and cozy personal collections, while the title, material notes, and DNA profile stay specific for easy comparison.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 6x6 kiss-cut sheet with 4 individual sticker designs.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; Durable kiss-cut vinyl sticker sheet with waterproof finish.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Size:&lt;/strong&gt; 6x6 kiss-cut sheet with four coordinated designs.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Zen Mentor-Grade; Zen aesthetic.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;DNA Profile:&lt;/strong&gt; A luminous koi fish leaping upward formed from Peach Moonstone and Rose Jade, soft pink ink-wash nebula flowing around body, coral talisman fragments orbiting fins, spring blossom bioluminescence trailing from tail, zen-mythic aesthetic, , , , , , person, text, watermark&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Best For:&lt;/strong&gt; students, remote workers, yoga lovers, and anyone building a serene everyday space.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;SEO Keywords:&lt;/strong&gt; zen koi sticker, peach moonstone fish, celestial koi art, rose jade aquatic, pink nebula design, coral talisman decor, bioluminescent sticker, premium fish sticker, mystical koi, Japanese zen art&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the actual product customers receive. Additional images are bonus concept/detail reference images and do not represent extra products or selectable variations.&lt;/p&gt;&lt;p&gt;Saved under the reference SKU below for easy collector matching.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Sticker-Zen-0081&lt;/small&gt;&lt;/p&gt;</t>
+          <t>&lt;h2&gt;Deep Work Sticker Set Celestial Koi Ascension Collector 4pc 6x6 Vinyl Laptop&lt;/h2&gt;&lt;p&gt;This is part of a fast A/B traffic test built around higher-intent buyer scenes: laptops, journals, planners, reading notebooks, book nooks, and focused desk setups. The style leans into smoky jade accents, quiet desk mood, sharp die-cut presentation, and giftable detail, avoiding generic mass-market wording.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One physical 4pc 6x6 kiss-cut vinyl sticker sheet, produced on demand through Printify.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Visual Lane:&lt;/strong&gt; A Deep Work Sticker Set&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Zen with Quiet Jade / Deep Work positioning.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the physical product customers receive. Additional gallery images are concept, detail, or collection-reference views and are not extra products or selectable variations.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Sticker-Zen-0081&lt;/small&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -8475,6 +8560,21 @@
       <c r="Q81" t="inlineStr">
         <is>
           <t>69f26782c326d7da170c1498</t>
+        </is>
+      </c>
+      <c r="AH81" t="inlineStr">
+        <is>
+          <t>SEO_STRIKE_SYNCED_PRINTIFY_DRAFT</t>
+        </is>
+      </c>
+      <c r="AI81" t="inlineStr">
+        <is>
+          <t>2026-05-07 02:06:35 -0400</t>
+        </is>
+      </c>
+      <c r="AJ81" t="inlineStr">
+        <is>
+          <t>A_DEEP_WORK_STICKER_SET</t>
         </is>
       </c>
     </row>
@@ -8583,12 +8683,12 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Phoenix Wing Fragment 4pc 6x6 Kiss-Cut Sticker Zen Aesthetic Laptop Journal</t>
+          <t>Deep Work Sticker Set Phoenix Wing Fragment 4pc 6x6 Vinyl Laptop Journal Decor</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>&lt;h2&gt;Phoenix Wing Fragment Kiss-Cut Sticker&lt;/h2&gt;&lt;p&gt;Bring calm and balance into your daily routine with this Phoenix Wing Fragment zen aesthetic kiss-cut sticker.&lt;/p&gt;&lt;p&gt;Designed for study rooms, creative workspaces, shelves, gallery walls, and collectible aesthetic decor, this sticker blends niche aesthetic appeal with collectible mentor-grade artwork.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 6x6 kiss-cut sheet with 4 individual sticker designs.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; Durable kiss-cut vinyl sticker sheet with waterproof finish.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Size:&lt;/strong&gt; 6x6 kiss-cut sheet with four coordinated designs.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Zen Mentor-Grade; Zen aesthetic.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;DNA Profile:&lt;/strong&gt; A single majestic phoenix wing unfurled formed from Peach Moonstone and Rose Jade, soft pink ink-wash nebula flowing between feathers, coral talisman fragments embedded in plumage, spring blossom bioluminescence glowing from wing tips, zen-mythic aesthetic, , , , , , person, text, watermark&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Best For:&lt;/strong&gt; mindfulness lovers, minimalists, journal keepers, yoga enthusiasts, and peaceful room setups.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;SEO Keywords:&lt;/strong&gt; phoenix wing sticker, peach moonstone feather, celestial bird art, rose jade wing, mythical phoenix design, coral talisman decor, bioluminescent wing, premium fantasy sticker, zen phoenix, sacred bird art&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the actual product customers receive. Additional images are bonus concept/detail reference images and do not represent extra products or selectable variations.&lt;/p&gt;&lt;p&gt;Complete the collection with matching Alchemy pieces.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Sticker-Zen-0083&lt;/small&gt;&lt;/p&gt;</t>
+          <t>&lt;h2&gt;Deep Work Sticker Set Phoenix Wing Fragment 4pc 6x6 Vinyl Laptop Journal Decor&lt;/h2&gt;&lt;p&gt;This is part of a fast A/B traffic test built around higher-intent buyer scenes: laptops, journals, planners, reading notebooks, book nooks, and focused desk setups. The style leans into smoky jade accents, quiet desk mood, sharp die-cut presentation, and giftable detail, avoiding generic mass-market wording.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One physical 4pc 6x6 kiss-cut vinyl sticker sheet, produced on demand through Printify.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Visual Lane:&lt;/strong&gt; A Deep Work Sticker Set&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Zen with Quiet Jade / Deep Work positioning.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the physical product customers receive. Additional gallery images are concept, detail, or collection-reference views and are not extra products or selectable variations.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Sticker-Zen-0083&lt;/small&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -8644,6 +8744,21 @@
       <c r="Q83" t="inlineStr">
         <is>
           <t>69f2683ecaeb1241880b7fcb</t>
+        </is>
+      </c>
+      <c r="AH83" t="inlineStr">
+        <is>
+          <t>SEO_STRIKE_SYNCED_PRINTIFY_DRAFT</t>
+        </is>
+      </c>
+      <c r="AI83" t="inlineStr">
+        <is>
+          <t>2026-05-07 02:06:35 -0400</t>
+        </is>
+      </c>
+      <c r="AJ83" t="inlineStr">
+        <is>
+          <t>A_DEEP_WORK_STICKER_SET</t>
         </is>
       </c>
     </row>
@@ -20667,6 +20782,43 @@
           <t>69f86a3d25819cdf3d0563b6</t>
         </is>
       </c>
+      <c r="S203" t="inlineStr">
+        <is>
+          <t>406909215172</t>
+        </is>
+      </c>
+      <c r="T203" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909215172</t>
+        </is>
+      </c>
+      <c r="U203" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V203" s="1" t="n">
+        <v>46149.07897425926</v>
+      </c>
+      <c r="Y203" s="1" t="n">
+        <v>46149.07897425926</v>
+      </c>
+      <c r="Z203" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA203" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB203" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909215172 handle=https://www.ebay.com/itm/406909215172</t>
+        </is>
+      </c>
+      <c r="AC203" s="1" t="n">
+        <v>46149.07897425926</v>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -20754,6 +20906,43 @@
           <t>69f86b8e83a8608fd80f1341</t>
         </is>
       </c>
+      <c r="S204" t="inlineStr">
+        <is>
+          <t>406909219066</t>
+        </is>
+      </c>
+      <c r="T204" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909219066</t>
+        </is>
+      </c>
+      <c r="U204" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V204" s="1" t="n">
+        <v>46149.07898653935</v>
+      </c>
+      <c r="Y204" s="1" t="n">
+        <v>46149.07898653935</v>
+      </c>
+      <c r="Z204" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA204" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB204" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909219066 handle=https://www.ebay.com/itm/406909219066</t>
+        </is>
+      </c>
+      <c r="AC204" s="1" t="n">
+        <v>46149.07898653935</v>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -20841,6 +21030,43 @@
           <t>69f86d3709f3b730240200b7</t>
         </is>
       </c>
+      <c r="S205" t="inlineStr">
+        <is>
+          <t>406909222169</t>
+        </is>
+      </c>
+      <c r="T205" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909222169</t>
+        </is>
+      </c>
+      <c r="U205" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V205" s="1" t="n">
+        <v>46149.0790015625</v>
+      </c>
+      <c r="Y205" s="1" t="n">
+        <v>46149.0790015625</v>
+      </c>
+      <c r="Z205" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA205" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB205" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909222169 handle=https://www.ebay.com/itm/406909222169</t>
+        </is>
+      </c>
+      <c r="AC205" s="1" t="n">
+        <v>46149.0790015625</v>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -20928,6 +21154,43 @@
           <t>69f86f6c2810b52a940a4161</t>
         </is>
       </c>
+      <c r="S206" t="inlineStr">
+        <is>
+          <t>406909223875</t>
+        </is>
+      </c>
+      <c r="T206" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909223875</t>
+        </is>
+      </c>
+      <c r="U206" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V206" s="1" t="n">
+        <v>46149.07901393519</v>
+      </c>
+      <c r="Y206" s="1" t="n">
+        <v>46149.07901393519</v>
+      </c>
+      <c r="Z206" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA206" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB206" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909223875 handle=https://www.ebay.com/itm/406909223875</t>
+        </is>
+      </c>
+      <c r="AC206" s="1" t="n">
+        <v>46149.07901393519</v>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -21015,6 +21278,43 @@
           <t>69f8807a011b67ecf80761ae</t>
         </is>
       </c>
+      <c r="S207" t="inlineStr">
+        <is>
+          <t>406909225478</t>
+        </is>
+      </c>
+      <c r="T207" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909225478</t>
+        </is>
+      </c>
+      <c r="U207" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V207" s="1" t="n">
+        <v>46149.07902600695</v>
+      </c>
+      <c r="Y207" s="1" t="n">
+        <v>46149.07902600695</v>
+      </c>
+      <c r="Z207" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA207" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB207" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909225478 handle=https://www.ebay.com/itm/406909225478</t>
+        </is>
+      </c>
+      <c r="AC207" s="1" t="n">
+        <v>46149.07902600695</v>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -21102,6 +21402,43 @@
           <t>69f8818abe136844f0003e48</t>
         </is>
       </c>
+      <c r="S208" t="inlineStr">
+        <is>
+          <t>406909226531</t>
+        </is>
+      </c>
+      <c r="T208" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909226531</t>
+        </is>
+      </c>
+      <c r="U208" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V208" s="1" t="n">
+        <v>46149.079038125</v>
+      </c>
+      <c r="Y208" s="1" t="n">
+        <v>46149.079038125</v>
+      </c>
+      <c r="Z208" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA208" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB208" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909226531 handle=https://www.ebay.com/itm/406909226531</t>
+        </is>
+      </c>
+      <c r="AC208" s="1" t="n">
+        <v>46149.079038125</v>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -21189,6 +21526,43 @@
           <t>69f882a1be136844f0003eed</t>
         </is>
       </c>
+      <c r="S209" t="inlineStr">
+        <is>
+          <t>406909228840</t>
+        </is>
+      </c>
+      <c r="T209" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909228840</t>
+        </is>
+      </c>
+      <c r="U209" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V209" s="1" t="n">
+        <v>46149.07905042824</v>
+      </c>
+      <c r="Y209" s="1" t="n">
+        <v>46149.07905042824</v>
+      </c>
+      <c r="Z209" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA209" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB209" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909228840 handle=https://www.ebay.com/itm/406909228840</t>
+        </is>
+      </c>
+      <c r="AC209" s="1" t="n">
+        <v>46149.07905042824</v>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -21276,6 +21650,43 @@
           <t>69f8836c5da263f75f04fad5</t>
         </is>
       </c>
+      <c r="S210" t="inlineStr">
+        <is>
+          <t>406909231370</t>
+        </is>
+      </c>
+      <c r="T210" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909231370</t>
+        </is>
+      </c>
+      <c r="U210" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V210" s="1" t="n">
+        <v>46149.07906267361</v>
+      </c>
+      <c r="Y210" s="1" t="n">
+        <v>46149.07906267361</v>
+      </c>
+      <c r="Z210" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA210" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB210" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909231370 handle=https://www.ebay.com/itm/406909231370</t>
+        </is>
+      </c>
+      <c r="AC210" s="1" t="n">
+        <v>46149.07906267361</v>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -21363,6 +21774,43 @@
           <t>69f883f3be136844f0003ff9</t>
         </is>
       </c>
+      <c r="S211" t="inlineStr">
+        <is>
+          <t>406909232068</t>
+        </is>
+      </c>
+      <c r="T211" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909232068</t>
+        </is>
+      </c>
+      <c r="U211" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V211" s="1" t="n">
+        <v>46149.07907480324</v>
+      </c>
+      <c r="Y211" s="1" t="n">
+        <v>46149.07907480324</v>
+      </c>
+      <c r="Z211" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA211" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB211" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909232068 handle=https://www.ebay.com/itm/406909232068</t>
+        </is>
+      </c>
+      <c r="AC211" s="1" t="n">
+        <v>46149.07907480324</v>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -21450,6 +21898,43 @@
           <t>69f88472ffbc831dea086941</t>
         </is>
       </c>
+      <c r="S212" t="inlineStr">
+        <is>
+          <t>406909232951</t>
+        </is>
+      </c>
+      <c r="T212" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909232951</t>
+        </is>
+      </c>
+      <c r="U212" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V212" s="1" t="n">
+        <v>46149.07908722222</v>
+      </c>
+      <c r="Y212" s="1" t="n">
+        <v>46149.07908722222</v>
+      </c>
+      <c r="Z212" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA212" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB212" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909232951 handle=https://www.ebay.com/itm/406909232951</t>
+        </is>
+      </c>
+      <c r="AC212" s="1" t="n">
+        <v>46149.07908722222</v>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -21537,6 +22022,43 @@
           <t>69f884ed83a8608fd80f239c</t>
         </is>
       </c>
+      <c r="S213" t="inlineStr">
+        <is>
+          <t>406909233684</t>
+        </is>
+      </c>
+      <c r="T213" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909233684</t>
+        </is>
+      </c>
+      <c r="U213" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V213" s="1" t="n">
+        <v>46149.0790996875</v>
+      </c>
+      <c r="Y213" s="1" t="n">
+        <v>46149.0790996875</v>
+      </c>
+      <c r="Z213" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA213" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB213" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909233684 handle=https://www.ebay.com/itm/406909233684</t>
+        </is>
+      </c>
+      <c r="AC213" s="1" t="n">
+        <v>46149.0790996875</v>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -21624,6 +22146,43 @@
           <t>69f88562be136844f00040a3</t>
         </is>
       </c>
+      <c r="S214" t="inlineStr">
+        <is>
+          <t>406909234435</t>
+        </is>
+      </c>
+      <c r="T214" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909234435</t>
+        </is>
+      </c>
+      <c r="U214" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V214" s="1" t="n">
+        <v>46149.07911322916</v>
+      </c>
+      <c r="Y214" s="1" t="n">
+        <v>46149.07911322916</v>
+      </c>
+      <c r="Z214" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA214" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB214" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909234435 handle=https://www.ebay.com/itm/406909234435</t>
+        </is>
+      </c>
+      <c r="AC214" s="1" t="n">
+        <v>46149.07911322916</v>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -21711,6 +22270,43 @@
           <t>69f886005da263f75f04fc9d</t>
         </is>
       </c>
+      <c r="S215" t="inlineStr">
+        <is>
+          <t>406909235356</t>
+        </is>
+      </c>
+      <c r="T215" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909235356</t>
+        </is>
+      </c>
+      <c r="U215" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V215" s="1" t="n">
+        <v>46149.07912559028</v>
+      </c>
+      <c r="Y215" s="1" t="n">
+        <v>46149.07912559028</v>
+      </c>
+      <c r="Z215" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA215" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB215" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909235356 handle=https://www.ebay.com/itm/406909235356</t>
+        </is>
+      </c>
+      <c r="AC215" s="1" t="n">
+        <v>46149.07912559028</v>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -21798,6 +22394,43 @@
           <t>69f88ee825819cdf3d057c87</t>
         </is>
       </c>
+      <c r="S216" t="inlineStr">
+        <is>
+          <t>406909236640</t>
+        </is>
+      </c>
+      <c r="T216" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909236640</t>
+        </is>
+      </c>
+      <c r="U216" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V216" s="1" t="n">
+        <v>46149.07913774306</v>
+      </c>
+      <c r="Y216" s="1" t="n">
+        <v>46149.07913774306</v>
+      </c>
+      <c r="Z216" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA216" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB216" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909236640 handle=https://www.ebay.com/itm/406909236640</t>
+        </is>
+      </c>
+      <c r="AC216" s="1" t="n">
+        <v>46149.07913774306</v>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -21885,6 +22518,43 @@
           <t>69f88fd4feed9979d10d0ce7</t>
         </is>
       </c>
+      <c r="S217" t="inlineStr">
+        <is>
+          <t>406909238227</t>
+        </is>
+      </c>
+      <c r="T217" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909238227</t>
+        </is>
+      </c>
+      <c r="U217" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V217" s="1" t="n">
+        <v>46149.07914980324</v>
+      </c>
+      <c r="Y217" s="1" t="n">
+        <v>46149.07914980324</v>
+      </c>
+      <c r="Z217" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA217" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB217" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909238227 handle=https://www.ebay.com/itm/406909238227</t>
+        </is>
+      </c>
+      <c r="AC217" s="1" t="n">
+        <v>46149.07914980324</v>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -21972,6 +22642,43 @@
           <t>69f8904bc1f268dee601c34f</t>
         </is>
       </c>
+      <c r="S218" t="inlineStr">
+        <is>
+          <t>406909240724</t>
+        </is>
+      </c>
+      <c r="T218" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909240724</t>
+        </is>
+      </c>
+      <c r="U218" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V218" s="1" t="n">
+        <v>46149.0791625</v>
+      </c>
+      <c r="Y218" s="1" t="n">
+        <v>46149.0791625</v>
+      </c>
+      <c r="Z218" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA218" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB218" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909240724 handle=https://www.ebay.com/itm/406909240724</t>
+        </is>
+      </c>
+      <c r="AC218" s="1" t="n">
+        <v>46149.0791625</v>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -22059,6 +22766,43 @@
           <t>69f890b8c1f268dee601c394</t>
         </is>
       </c>
+      <c r="S219" t="inlineStr">
+        <is>
+          <t>406909242546</t>
+        </is>
+      </c>
+      <c r="T219" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909242546</t>
+        </is>
+      </c>
+      <c r="U219" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V219" s="1" t="n">
+        <v>46149.07917508102</v>
+      </c>
+      <c r="Y219" s="1" t="n">
+        <v>46149.07917508102</v>
+      </c>
+      <c r="Z219" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA219" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB219" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909242546 handle=https://www.ebay.com/itm/406909242546</t>
+        </is>
+      </c>
+      <c r="AC219" s="1" t="n">
+        <v>46149.07917508102</v>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -22146,6 +22890,43 @@
           <t>69f89116b051b8a0e90b9662</t>
         </is>
       </c>
+      <c r="S220" t="inlineStr">
+        <is>
+          <t>406909243824</t>
+        </is>
+      </c>
+      <c r="T220" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909243824</t>
+        </is>
+      </c>
+      <c r="U220" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V220" s="1" t="n">
+        <v>46149.0791871875</v>
+      </c>
+      <c r="Y220" s="1" t="n">
+        <v>46149.0791871875</v>
+      </c>
+      <c r="Z220" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA220" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB220" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909243824 handle=https://www.ebay.com/itm/406909243824</t>
+        </is>
+      </c>
+      <c r="AC220" s="1" t="n">
+        <v>46149.0791871875</v>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -22233,6 +23014,43 @@
           <t>69f8918925819cdf3d057e2d</t>
         </is>
       </c>
+      <c r="S221" t="inlineStr">
+        <is>
+          <t>406909244688</t>
+        </is>
+      </c>
+      <c r="T221" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909244688</t>
+        </is>
+      </c>
+      <c r="U221" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V221" s="1" t="n">
+        <v>46149.07919978009</v>
+      </c>
+      <c r="Y221" s="1" t="n">
+        <v>46149.07919978009</v>
+      </c>
+      <c r="Z221" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA221" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB221" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909244688 handle=https://www.ebay.com/itm/406909244688</t>
+        </is>
+      </c>
+      <c r="AC221" s="1" t="n">
+        <v>46149.07919978009</v>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -22320,6 +23138,43 @@
           <t>69f892035da263f75f05059e</t>
         </is>
       </c>
+      <c r="S222" t="inlineStr">
+        <is>
+          <t>406909247161</t>
+        </is>
+      </c>
+      <c r="T222" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909247161</t>
+        </is>
+      </c>
+      <c r="U222" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V222" s="1" t="n">
+        <v>46149.07921200232</v>
+      </c>
+      <c r="Y222" s="1" t="n">
+        <v>46149.07921200232</v>
+      </c>
+      <c r="Z222" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA222" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB222" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909247161 handle=https://www.ebay.com/itm/406909247161</t>
+        </is>
+      </c>
+      <c r="AC222" s="1" t="n">
+        <v>46149.07921200232</v>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -22344,12 +23199,12 @@
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t>Rose Quartz Chapel Soul Lantern Grimdark 5x7 Acrylic Art Gothic Collectible</t>
+          <t>Quiet Luxury Desk Relic Rose Quartz Chapel Soul Lantern 5x7 Acrylic Block Decor</t>
         </is>
       </c>
       <c r="F223" t="inlineStr">
         <is>
-          <t>&lt;p&gt;This Rose Quartz Chapel Soul Lantern captures a grimdark artifact aesthetic with a pink-white spirit flame suspended within wrought iron chapel gates. The imperial jade glass panels feature ink-wash nebula patterns and rose quartz inlays, creating a soft rose glow that evokes a soul vessel from a forgotten gothic archive.&lt;/p&gt;&lt;p&gt;Printed on premium 5x7 acrylic, this piece offers a luminous, museum-grade presence for a study desk, altar shelf, or dark academia reading nook. The transparent substrate enhances the layered depth and subtle bioluminescent effect, making it ideal for collectors of mentor-grade gothic artifacts or those seeking a unique gift for a book lover or occult enthusiast.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 5x7 acrylic print, ready to display on included easel stand or wall mount&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; High-gloss clear acrylic with UV-resistant inks, 5mm thickness&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Size:&lt;/strong&gt; 5x7 inches (12.7 x 17.8 cm)&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Grimdark Mentor-Grade with rose quartz, wrought iron, and jade glass motifs&lt;/li&gt;&lt;li&gt;&lt;strong&gt;DNA Profile:&lt;/strong&gt; Grimdark artifact, rose quartz inlay, chapel gate frame, pink-white flame, ink-wash nebula, imperial jade glass, talisman fragments, kintsugi vein logic, bioluminescent glow, micro-engraved relief&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Use Cases:&lt;/strong&gt; Gothic decor, dark academia study, witchy altar, collector display, gift for occult or fantasy enthusiasts&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the actual product customers receive. Additional images are bonus concept/detail reference images and do not represent extra products or selectable variations.&lt;/p&gt;&lt;p&gt;&lt;em&gt;Image Note: &lt;/em&gt;&lt;/p&gt;</t>
+          <t>&lt;h2&gt;Quiet Luxury Desk Relic Rose Quartz Chapel Soul Lantern 5x7 Acrylic Block Decor&lt;/h2&gt;&lt;p&gt;This is part of a fast A/B traffic test built around higher-intent buyer scenes: quiet luxury apartment shelves, gothic study desks, collector corners, and deep-work rooms. The style leans into smoky jade glow, acrylic depth, refractive light, and gallery-object presence, avoiding generic mass-market wording.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 5x7 vertical acrylic photo block, produced on demand through Printify.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Visual Lane:&lt;/strong&gt; A Quiet Luxury Desk Object&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Grimdark with Quiet Jade / Deep Work positioning.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the physical product customers receive. Additional gallery images are concept, detail, or collection-reference views and are not extra products or selectable variations.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Acrylic-Grimdark-0038&lt;/small&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="G223" t="inlineStr">
@@ -22394,7 +23249,7 @@
       </c>
       <c r="O223" t="inlineStr">
         <is>
-          <t>Printify_UI_Mockups4</t>
+          <t>Printify_Published_Mockups4</t>
         </is>
       </c>
       <c r="P223" t="inlineStr">
@@ -22405,6 +23260,42 @@
       <c r="Q223" t="inlineStr">
         <is>
           <t>69f8928b25819cdf3d057ef7</t>
+        </is>
+      </c>
+      <c r="R223" s="1" t="n">
+        <v>46149.08978430011</v>
+      </c>
+      <c r="S223" t="inlineStr">
+        <is>
+          <t>406910074365</t>
+        </is>
+      </c>
+      <c r="T223" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406910074365</t>
+        </is>
+      </c>
+      <c r="U223" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V223" s="1" t="n">
+        <v>46149.09008196864</v>
+      </c>
+      <c r="AH223" t="inlineStr">
+        <is>
+          <t>SEO_STRIKE_SYNCED_PRINTIFY_DRAFT</t>
+        </is>
+      </c>
+      <c r="AI223" t="inlineStr">
+        <is>
+          <t>2026-05-07 02:06:35 -0400</t>
+        </is>
+      </c>
+      <c r="AJ223" t="inlineStr">
+        <is>
+          <t>A_QUIET_LUXURY_DESK_OBJECT</t>
         </is>
       </c>
     </row>
@@ -22431,12 +23322,12 @@
       </c>
       <c r="E224" t="inlineStr">
         <is>
-          <t>Sapphire Temple Soul Lantern Grimdark 5x7 Acrylic Display Gothic Artifact Shelf</t>
+          <t>Smoky Jade Gothic Object Sapphire Temple Soul Lantern Artifact 5x7 Acrylic Gift</t>
         </is>
       </c>
       <c r="F224" t="inlineStr">
         <is>
-          <t>&lt;p&gt;This 5x7 acrylic display presents the Sapphire Temple Soul Lantern, a gothic artifact from the Grimdark Mentor-Grade collection. The design features a wrought iron temple archway frame with sapphire inlays, enclosing a deep-blue spirit flame and floating talisman fragments against imperial jade glass panels. The ink-wash nebula patterns and soft sapphire glow create a balanced, collector-focused aesthetic.&lt;/p&gt;&lt;p&gt;Ideal for study desks, bookshelves, or altars, this piece brings dark academia and mystical decor to any space. The high-gloss acrylic surface enhances the layered translucent depth and micro-engraved relief, while the internal bioluminescent glow adds a subtle, refined presence. Use it as a meditation focal point, a gothic room accent, or a premium gift for artifact enthusiasts.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 5x7 acrylic print with protective film&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; High-gloss acrylic, 0.25-inch thick, with beveled edges&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Size:&lt;/strong&gt; 5x7 inches (portrait orientation)&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Grimdark Mentor-Grade, gothic artifact, dark academia&lt;/li&gt;&lt;li&gt;&lt;strong&gt;DNA Profile:&lt;/strong&gt; Wrought iron frame, sapphire inlays, deep-blue spirit flame, floating talisman fragments, imperial jade glass panels, ink-wash nebula patterns, micro-engraved surface relief, kintsugi-like vein logic, internal bioluminescent glow, cinematic rim lighting&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Use Cases:&lt;/strong&gt; Study desk decor, bookshelf accent, altar piece, gothic room decor, collector display, dark academia gift, meditation focal point&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the actual product customers receive. Additional images are bonus concept/detail reference images and do not represent extra products or selectable variations.&lt;/p&gt;&lt;p&gt;&lt;em&gt;Image Note: &lt;/em&gt;&lt;/p&gt;</t>
+          <t>&lt;h2&gt;Smoky Jade Gothic Object Sapphire Temple Soul Lantern Artifact 5x7 Acrylic Gift&lt;/h2&gt;&lt;p&gt;This is part of a fast A/B traffic test built around higher-intent buyer scenes: quiet luxury apartment shelves, gothic study desks, collector corners, and deep-work rooms. The style leans into smoky jade glow, acrylic depth, refractive light, and gallery-object presence, avoiding generic mass-market wording.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 5x7 vertical acrylic photo block, produced on demand through Printify.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Visual Lane:&lt;/strong&gt; B Gothic Collector Shelf&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Grimdark with Quiet Jade / Deep Work positioning.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the physical product customers receive. Additional gallery images are concept, detail, or collection-reference views and are not extra products or selectable variations.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Acrylic-Grimdark-0039&lt;/small&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="G224" t="inlineStr">
@@ -22481,7 +23372,7 @@
       </c>
       <c r="O224" t="inlineStr">
         <is>
-          <t>Printify_UI_Mockups4</t>
+          <t>Printify_Published_Mockups4</t>
         </is>
       </c>
       <c r="P224" t="inlineStr">
@@ -22492,6 +23383,42 @@
       <c r="Q224" t="inlineStr">
         <is>
           <t>69f8931cb051b8a0e90b97c7</t>
+        </is>
+      </c>
+      <c r="R224" s="1" t="n">
+        <v>46149.09025860706</v>
+      </c>
+      <c r="S224" t="inlineStr">
+        <is>
+          <t>406910075457</t>
+        </is>
+      </c>
+      <c r="T224" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406910075457</t>
+        </is>
+      </c>
+      <c r="U224" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V224" s="1" t="n">
+        <v>46149.09070339654</v>
+      </c>
+      <c r="AH224" t="inlineStr">
+        <is>
+          <t>SEO_STRIKE_SYNCED_PRINTIFY_DRAFT</t>
+        </is>
+      </c>
+      <c r="AI224" t="inlineStr">
+        <is>
+          <t>2026-05-07 02:06:35 -0400</t>
+        </is>
+      </c>
+      <c r="AJ224" t="inlineStr">
+        <is>
+          <t>B_GOTHIC_COLLECTOR_SHELF</t>
         </is>
       </c>
     </row>
@@ -22518,12 +23445,12 @@
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t>Silver Moon Gate Soul Lantern Grimdark 5x7 Acrylic Art Gothic Mentor-Grade Gift</t>
+          <t>Smoky Jade Gothic Object Silver Moon Gate Soul Lantern 5x7 Acrylic Display Gift</t>
         </is>
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t>&lt;p&gt;This Silver Moon Gate Soul Lantern captures a grimdark mentor-grade aesthetic, blending a wrought iron moon gate silhouette with moonstone inlays and imperial jade glass panels. The swirling silver-white spirit flame and floating talisman fragments evoke a gothic, collectible artifact mood, perfect for dark academia or occult-inspired spaces.&lt;/p&gt;&lt;p&gt;Printed on premium 5x7 acrylic, this piece offers a luminous, translucent depth with micro-engraved surface relief and a subtle internal glow. Ideal for display on a study desk, bookshelf, or altar, it serves as a conversation-starting decor accent or a thoughtful gift for lovers of gothic fantasy and dark art.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 5x7 acrylic art panel, ready to hang or stand&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; High-gloss acrylic with UV-resistant print&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Size:&lt;/strong&gt; 5x7 inches (12.7 x 17.8 cm)&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Grimdark Mentor-Grade, with wrought iron, moonstone, jade glass, talisman fragments, and silver-white flame motifs&lt;/li&gt;&lt;li&gt;&lt;strong&gt;DNA Profile:&lt;/strong&gt; Ethereal gothic lantern, moon gate silhouette, spirit flame, talisman fragments, ink-wash nebula patterns, imperial jade glass, soft lunar glow, hyper-detailed object design, micro-engraved relief, handcrafted edge bevels, layered translucent depth, internal bioluminescent glow, kintsugi-like vein logic, floating accent fragments, cinematic rim lighting, museum-grade overhead fill, crisp silhouette, centered composition, high-end collectible artifact aesthetic&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Use Cases:&lt;/strong&gt; Gothic decor, dark academia study, occult art collection, mentor-grade display, gift for fantasy enthusiasts&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the actual product customers receive. Additional images are bonus concept/detail reference images and do not represent extra products or selectable variations.&lt;/p&gt;&lt;p&gt;&lt;em&gt;Image Note: &lt;/em&gt;&lt;/p&gt;</t>
+          <t>&lt;h2&gt;Smoky Jade Gothic Object Silver Moon Gate Soul Lantern 5x7 Acrylic Display Gift&lt;/h2&gt;&lt;p&gt;This is part of a fast A/B traffic test built around higher-intent buyer scenes: quiet luxury apartment shelves, gothic study desks, collector corners, and deep-work rooms. The style leans into smoky jade glow, acrylic depth, refractive light, and gallery-object presence, avoiding generic mass-market wording.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 5x7 vertical acrylic photo block, produced on demand through Printify.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Visual Lane:&lt;/strong&gt; B Gothic Collector Shelf&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Grimdark with Quiet Jade / Deep Work positioning.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the physical product customers receive. Additional gallery images are concept, detail, or collection-reference views and are not extra products or selectable variations.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Acrylic-Grimdark-0040&lt;/small&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="G225" t="inlineStr">
@@ -22568,7 +23495,7 @@
       </c>
       <c r="O225" t="inlineStr">
         <is>
-          <t>Printify_UI_Mockups4</t>
+          <t>Printify_Published_Mockups4</t>
         </is>
       </c>
       <c r="P225" t="inlineStr">
@@ -22579,6 +23506,42 @@
       <c r="Q225" t="inlineStr">
         <is>
           <t>69f8937bbe136844f0004b36</t>
+        </is>
+      </c>
+      <c r="R225" s="1" t="n">
+        <v>46149.09086501994</v>
+      </c>
+      <c r="S225" t="inlineStr">
+        <is>
+          <t>406910076542</t>
+        </is>
+      </c>
+      <c r="T225" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406910076542</t>
+        </is>
+      </c>
+      <c r="U225" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V225" s="1" t="n">
+        <v>46149.09116347688</v>
+      </c>
+      <c r="AH225" t="inlineStr">
+        <is>
+          <t>SEO_STRIKE_SYNCED_PRINTIFY_DRAFT</t>
+        </is>
+      </c>
+      <c r="AI225" t="inlineStr">
+        <is>
+          <t>2026-05-07 02:06:35 -0400</t>
+        </is>
+      </c>
+      <c r="AJ225" t="inlineStr">
+        <is>
+          <t>B_GOTHIC_COLLECTOR_SHELF</t>
         </is>
       </c>
     </row>
@@ -22668,6 +23631,43 @@
           <t>69f89a94c1f268dee601cb9d</t>
         </is>
       </c>
+      <c r="S226" t="inlineStr">
+        <is>
+          <t>406903730229</t>
+        </is>
+      </c>
+      <c r="T226" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903730229</t>
+        </is>
+      </c>
+      <c r="U226" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V226" s="1" t="n">
+        <v>46149.07922526621</v>
+      </c>
+      <c r="Y226" s="1" t="n">
+        <v>46149.07922526621</v>
+      </c>
+      <c r="Z226" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA226" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB226" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406903730229 handle=https://www.ebay.com/itm/406903730229</t>
+        </is>
+      </c>
+      <c r="AC226" s="1" t="n">
+        <v>46149.07922526621</v>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -22755,6 +23755,43 @@
           <t>69f89b9ca70f06579a00a708</t>
         </is>
       </c>
+      <c r="S227" t="inlineStr">
+        <is>
+          <t>406903744471</t>
+        </is>
+      </c>
+      <c r="T227" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903744471</t>
+        </is>
+      </c>
+      <c r="U227" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V227" s="1" t="n">
+        <v>46149.07923866898</v>
+      </c>
+      <c r="Y227" s="1" t="n">
+        <v>46149.07923866898</v>
+      </c>
+      <c r="Z227" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA227" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB227" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406903744471 handle=https://www.ebay.com/itm/406903744471</t>
+        </is>
+      </c>
+      <c r="AC227" s="1" t="n">
+        <v>46149.07923866898</v>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -22842,6 +23879,43 @@
           <t>69f89c6f09f3b730240221b8</t>
         </is>
       </c>
+      <c r="S228" t="inlineStr">
+        <is>
+          <t>406903748661</t>
+        </is>
+      </c>
+      <c r="T228" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903748661</t>
+        </is>
+      </c>
+      <c r="U228" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V228" s="1" t="n">
+        <v>46149.07925134259</v>
+      </c>
+      <c r="Y228" s="1" t="n">
+        <v>46149.07925134259</v>
+      </c>
+      <c r="Z228" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA228" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB228" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406903748661 handle=https://www.ebay.com/itm/406903748661</t>
+        </is>
+      </c>
+      <c r="AC228" s="1" t="n">
+        <v>46149.07925134259</v>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -22929,6 +24003,43 @@
           <t>69f89da69f68ab7cf001f531</t>
         </is>
       </c>
+      <c r="S229" t="inlineStr">
+        <is>
+          <t>406903754696</t>
+        </is>
+      </c>
+      <c r="T229" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903754696</t>
+        </is>
+      </c>
+      <c r="U229" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V229" s="1" t="n">
+        <v>46149.07926362268</v>
+      </c>
+      <c r="Y229" s="1" t="n">
+        <v>46149.07926362268</v>
+      </c>
+      <c r="Z229" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA229" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB229" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406903754696 handle=https://www.ebay.com/itm/406903754696</t>
+        </is>
+      </c>
+      <c r="AC229" s="1" t="n">
+        <v>46149.07926362268</v>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -23016,6 +24127,43 @@
           <t>69f89eac011b67ecf8077844</t>
         </is>
       </c>
+      <c r="S230" t="inlineStr">
+        <is>
+          <t>406903758348</t>
+        </is>
+      </c>
+      <c r="T230" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406903758348</t>
+        </is>
+      </c>
+      <c r="U230" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V230" s="1" t="n">
+        <v>46149.07927614584</v>
+      </c>
+      <c r="Y230" s="1" t="n">
+        <v>46149.07927614584</v>
+      </c>
+      <c r="Z230" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA230" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB230" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406903758348 handle=https://www.ebay.com/itm/406903758348</t>
+        </is>
+      </c>
+      <c r="AC230" s="1" t="n">
+        <v>46149.07927614584</v>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -23103,6 +24251,43 @@
           <t>69f89fda2592a8ad8e0f2e79</t>
         </is>
       </c>
+      <c r="S231" t="inlineStr">
+        <is>
+          <t>406909147173</t>
+        </is>
+      </c>
+      <c r="T231" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909147173</t>
+        </is>
+      </c>
+      <c r="U231" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V231" s="1" t="n">
+        <v>46149.07928880787</v>
+      </c>
+      <c r="Y231" s="1" t="n">
+        <v>46149.07928880787</v>
+      </c>
+      <c r="Z231" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA231" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB231" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909147173 handle=https://www.ebay.com/itm/406909147173</t>
+        </is>
+      </c>
+      <c r="AC231" s="1" t="n">
+        <v>46149.07928880787</v>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -23190,6 +24375,43 @@
           <t>69f8a454c1f268dee601d3ad</t>
         </is>
       </c>
+      <c r="S232" t="inlineStr">
+        <is>
+          <t>406909150037</t>
+        </is>
+      </c>
+      <c r="T232" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909150037</t>
+        </is>
+      </c>
+      <c r="U232" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V232" s="1" t="n">
+        <v>46149.07930130787</v>
+      </c>
+      <c r="Y232" s="1" t="n">
+        <v>46149.07930130787</v>
+      </c>
+      <c r="Z232" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA232" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB232" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909150037 handle=https://www.ebay.com/itm/406909150037</t>
+        </is>
+      </c>
+      <c r="AC232" s="1" t="n">
+        <v>46149.07930130787</v>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -23277,6 +24499,43 @@
           <t>69f903dec1f268dee601f679</t>
         </is>
       </c>
+      <c r="S233" t="inlineStr">
+        <is>
+          <t>406909153504</t>
+        </is>
+      </c>
+      <c r="T233" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909153504</t>
+        </is>
+      </c>
+      <c r="U233" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V233" s="1" t="n">
+        <v>46149.07931458333</v>
+      </c>
+      <c r="Y233" s="1" t="n">
+        <v>46149.07931458333</v>
+      </c>
+      <c r="Z233" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA233" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB233" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909153504 handle=https://www.ebay.com/itm/406909153504</t>
+        </is>
+      </c>
+      <c r="AC233" s="1" t="n">
+        <v>46149.07931458333</v>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -23364,6 +24623,43 @@
           <t>69f904df97d964f736006a48</t>
         </is>
       </c>
+      <c r="S234" t="inlineStr">
+        <is>
+          <t>406909164941</t>
+        </is>
+      </c>
+      <c r="T234" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909164941</t>
+        </is>
+      </c>
+      <c r="U234" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V234" s="1" t="n">
+        <v>46149.07932724537</v>
+      </c>
+      <c r="Y234" s="1" t="n">
+        <v>46149.07932724537</v>
+      </c>
+      <c r="Z234" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA234" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB234" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909164941 handle=https://www.ebay.com/itm/406909164941</t>
+        </is>
+      </c>
+      <c r="AC234" s="1" t="n">
+        <v>46149.07932724537</v>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -23451,6 +24747,43 @@
           <t>69f90607feed9979d10d40e7</t>
         </is>
       </c>
+      <c r="S235" t="inlineStr">
+        <is>
+          <t>406909216787</t>
+        </is>
+      </c>
+      <c r="T235" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909216787</t>
+        </is>
+      </c>
+      <c r="U235" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V235" s="1" t="n">
+        <v>46149.07933987268</v>
+      </c>
+      <c r="Y235" s="1" t="n">
+        <v>46149.07933987268</v>
+      </c>
+      <c r="Z235" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA235" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB235" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909216787 handle=https://www.ebay.com/itm/406909216787</t>
+        </is>
+      </c>
+      <c r="AC235" s="1" t="n">
+        <v>46149.07933987268</v>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -23538,6 +24871,43 @@
           <t>69f907b49f68ab7cf0022003</t>
         </is>
       </c>
+      <c r="S236" t="inlineStr">
+        <is>
+          <t>406909220927</t>
+        </is>
+      </c>
+      <c r="T236" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909220927</t>
+        </is>
+      </c>
+      <c r="U236" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V236" s="1" t="n">
+        <v>46149.07935664352</v>
+      </c>
+      <c r="Y236" s="1" t="n">
+        <v>46149.07935664352</v>
+      </c>
+      <c r="Z236" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA236" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB236" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909220927 handle=https://www.ebay.com/itm/406909220927</t>
+        </is>
+      </c>
+      <c r="AC236" s="1" t="n">
+        <v>46149.07935664352</v>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -23625,6 +24995,43 @@
           <t>69f90c957f4b346c8a0c603f</t>
         </is>
       </c>
+      <c r="S237" t="inlineStr">
+        <is>
+          <t>406909264998</t>
+        </is>
+      </c>
+      <c r="T237" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909264998</t>
+        </is>
+      </c>
+      <c r="U237" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V237" s="1" t="n">
+        <v>46149.0793691088</v>
+      </c>
+      <c r="Y237" s="1" t="n">
+        <v>46149.0793691088</v>
+      </c>
+      <c r="Z237" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA237" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB237" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909264998 handle=https://www.ebay.com/itm/406909264998</t>
+        </is>
+      </c>
+      <c r="AC237" s="1" t="n">
+        <v>46149.0793691088</v>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -23712,6 +25119,43 @@
           <t>69fba23409770f1d9306b86d</t>
         </is>
       </c>
+      <c r="S238" t="inlineStr">
+        <is>
+          <t>406909266188</t>
+        </is>
+      </c>
+      <c r="T238" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909266188</t>
+        </is>
+      </c>
+      <c r="U238" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V238" s="1" t="n">
+        <v>46149.07938283565</v>
+      </c>
+      <c r="Y238" s="1" t="n">
+        <v>46149.07938283565</v>
+      </c>
+      <c r="Z238" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA238" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB238" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909266188 handle=https://www.ebay.com/itm/406909266188</t>
+        </is>
+      </c>
+      <c r="AC238" s="1" t="n">
+        <v>46149.07938283565</v>
+      </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -23799,6 +25243,43 @@
           <t>69fba266489d5635ab0e6504</t>
         </is>
       </c>
+      <c r="S239" t="inlineStr">
+        <is>
+          <t>406909268494</t>
+        </is>
+      </c>
+      <c r="T239" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909268494</t>
+        </is>
+      </c>
+      <c r="U239" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V239" s="1" t="n">
+        <v>46149.07939530093</v>
+      </c>
+      <c r="Y239" s="1" t="n">
+        <v>46149.07939530093</v>
+      </c>
+      <c r="Z239" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA239" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB239" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909268494 handle=https://www.ebay.com/itm/406909268494</t>
+        </is>
+      </c>
+      <c r="AC239" s="1" t="n">
+        <v>46149.07939530093</v>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -23886,6 +25367,43 @@
           <t>69fba28a6d07bd21600e1684</t>
         </is>
       </c>
+      <c r="S240" t="inlineStr">
+        <is>
+          <t>406909269321</t>
+        </is>
+      </c>
+      <c r="T240" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909269321</t>
+        </is>
+      </c>
+      <c r="U240" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V240" s="1" t="n">
+        <v>46149.07940789352</v>
+      </c>
+      <c r="Y240" s="1" t="n">
+        <v>46149.07940789352</v>
+      </c>
+      <c r="Z240" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA240" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB240" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909269321 handle=https://www.ebay.com/itm/406909269321</t>
+        </is>
+      </c>
+      <c r="AC240" s="1" t="n">
+        <v>46149.07940789352</v>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -23973,6 +25491,43 @@
           <t>69fbbffef60a24b6d1034e4d</t>
         </is>
       </c>
+      <c r="S241" t="inlineStr">
+        <is>
+          <t>406909467980</t>
+        </is>
+      </c>
+      <c r="T241" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909467980</t>
+        </is>
+      </c>
+      <c r="U241" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V241" s="1" t="n">
+        <v>46149.07942113426</v>
+      </c>
+      <c r="Y241" s="1" t="n">
+        <v>46149.07942113426</v>
+      </c>
+      <c r="Z241" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA241" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB241" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909467980 handle=https://www.ebay.com/itm/406909467980</t>
+        </is>
+      </c>
+      <c r="AC241" s="1" t="n">
+        <v>46149.07942113426</v>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -24125,6 +25680,43 @@
           <t>69fb7e754ce71ea8ae0c7af1</t>
         </is>
       </c>
+      <c r="S243" t="inlineStr">
+        <is>
+          <t>406909061109</t>
+        </is>
+      </c>
+      <c r="T243" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909061109</t>
+        </is>
+      </c>
+      <c r="U243" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V243" s="1" t="n">
+        <v>46149.07943375</v>
+      </c>
+      <c r="Y243" s="1" t="n">
+        <v>46149.07943375</v>
+      </c>
+      <c r="Z243" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA243" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB243" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909061109 handle=https://www.ebay.com/itm/406909061109</t>
+        </is>
+      </c>
+      <c r="AC243" s="1" t="n">
+        <v>46149.07943375</v>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -24212,6 +25804,43 @@
           <t>69fb804bff28e7d4030aa67d</t>
         </is>
       </c>
+      <c r="S244" t="inlineStr">
+        <is>
+          <t>406909095974</t>
+        </is>
+      </c>
+      <c r="T244" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909095974</t>
+        </is>
+      </c>
+      <c r="U244" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V244" s="1" t="n">
+        <v>46149.07944618056</v>
+      </c>
+      <c r="Y244" s="1" t="n">
+        <v>46149.07944618056</v>
+      </c>
+      <c r="Z244" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA244" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB244" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909095974 handle=https://www.ebay.com/itm/406909095974</t>
+        </is>
+      </c>
+      <c r="AC244" s="1" t="n">
+        <v>46149.07944618056</v>
+      </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -24299,6 +25928,43 @@
           <t>69fb819d4c6544084c0f8370</t>
         </is>
       </c>
+      <c r="S245" t="inlineStr">
+        <is>
+          <t>406909097469</t>
+        </is>
+      </c>
+      <c r="T245" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909097469</t>
+        </is>
+      </c>
+      <c r="U245" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V245" s="1" t="n">
+        <v>46149.07945979167</v>
+      </c>
+      <c r="Y245" s="1" t="n">
+        <v>46149.07945979167</v>
+      </c>
+      <c r="Z245" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA245" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB245" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909097469 handle=https://www.ebay.com/itm/406909097469</t>
+        </is>
+      </c>
+      <c r="AC245" s="1" t="n">
+        <v>46149.07945979167</v>
+      </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -24386,6 +26052,43 @@
           <t>69fb82e64c6544084c0f83d5</t>
         </is>
       </c>
+      <c r="S246" t="inlineStr">
+        <is>
+          <t>406909100892</t>
+        </is>
+      </c>
+      <c r="T246" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909100892</t>
+        </is>
+      </c>
+      <c r="U246" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V246" s="1" t="n">
+        <v>46149.07947209491</v>
+      </c>
+      <c r="Y246" s="1" t="n">
+        <v>46149.07947209491</v>
+      </c>
+      <c r="Z246" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA246" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB246" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909100892 handle=https://www.ebay.com/itm/406909100892</t>
+        </is>
+      </c>
+      <c r="AC246" s="1" t="n">
+        <v>46149.07947209491</v>
+      </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -24473,6 +26176,43 @@
           <t>69fb868dc5114ecf420d2b93</t>
         </is>
       </c>
+      <c r="S247" t="inlineStr">
+        <is>
+          <t>406909114799</t>
+        </is>
+      </c>
+      <c r="T247" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909114799</t>
+        </is>
+      </c>
+      <c r="U247" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V247" s="1" t="n">
+        <v>46149.07948486111</v>
+      </c>
+      <c r="Y247" s="1" t="n">
+        <v>46149.07948486111</v>
+      </c>
+      <c r="Z247" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA247" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB247" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909114799 handle=https://www.ebay.com/itm/406909114799</t>
+        </is>
+      </c>
+      <c r="AC247" s="1" t="n">
+        <v>46149.07948486111</v>
+      </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -24560,6 +26300,43 @@
           <t>69fb8749a7afceb9f70f1956</t>
         </is>
       </c>
+      <c r="S248" t="inlineStr">
+        <is>
+          <t>406909116716</t>
+        </is>
+      </c>
+      <c r="T248" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909116716</t>
+        </is>
+      </c>
+      <c r="U248" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V248" s="1" t="n">
+        <v>46149.07949722222</v>
+      </c>
+      <c r="Y248" s="1" t="n">
+        <v>46149.07949722222</v>
+      </c>
+      <c r="Z248" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA248" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB248" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909116716 handle=https://www.ebay.com/itm/406909116716</t>
+        </is>
+      </c>
+      <c r="AC248" s="1" t="n">
+        <v>46149.07949722222</v>
+      </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -24647,6 +26424,43 @@
           <t>69fb87aca7afceb9f70f1982</t>
         </is>
       </c>
+      <c r="S249" t="inlineStr">
+        <is>
+          <t>406909118000</t>
+        </is>
+      </c>
+      <c r="T249" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909118000</t>
+        </is>
+      </c>
+      <c r="U249" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V249" s="1" t="n">
+        <v>46149.07950961806</v>
+      </c>
+      <c r="Y249" s="1" t="n">
+        <v>46149.07950961806</v>
+      </c>
+      <c r="Z249" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA249" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB249" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909118000 handle=https://www.ebay.com/itm/406909118000</t>
+        </is>
+      </c>
+      <c r="AC249" s="1" t="n">
+        <v>46149.07950961806</v>
+      </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -24734,6 +26548,43 @@
           <t>69fb87efc5114ecf420d2c5a</t>
         </is>
       </c>
+      <c r="S250" t="inlineStr">
+        <is>
+          <t>406909119544</t>
+        </is>
+      </c>
+      <c r="T250" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909119544</t>
+        </is>
+      </c>
+      <c r="U250" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V250" s="1" t="n">
+        <v>46149.07952208333</v>
+      </c>
+      <c r="Y250" s="1" t="n">
+        <v>46149.07952208333</v>
+      </c>
+      <c r="Z250" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA250" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB250" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909119544 handle=https://www.ebay.com/itm/406909119544</t>
+        </is>
+      </c>
+      <c r="AC250" s="1" t="n">
+        <v>46149.07952208333</v>
+      </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -24821,6 +26672,43 @@
           <t>69fb8805ee663532c8017f4f</t>
         </is>
       </c>
+      <c r="S251" t="inlineStr">
+        <is>
+          <t>406909121336</t>
+        </is>
+      </c>
+      <c r="T251" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909121336</t>
+        </is>
+      </c>
+      <c r="U251" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V251" s="1" t="n">
+        <v>46149.07953444444</v>
+      </c>
+      <c r="Y251" s="1" t="n">
+        <v>46149.07953444444</v>
+      </c>
+      <c r="Z251" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA251" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB251" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909121336 handle=https://www.ebay.com/itm/406909121336</t>
+        </is>
+      </c>
+      <c r="AC251" s="1" t="n">
+        <v>46149.07953444444</v>
+      </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -24908,6 +26796,43 @@
           <t>69fb8811e5402c478e03108f</t>
         </is>
       </c>
+      <c r="S252" t="inlineStr">
+        <is>
+          <t>406909122790</t>
+        </is>
+      </c>
+      <c r="T252" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909122790</t>
+        </is>
+      </c>
+      <c r="U252" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V252" s="1" t="n">
+        <v>46149.07954709491</v>
+      </c>
+      <c r="Y252" s="1" t="n">
+        <v>46149.07954709491</v>
+      </c>
+      <c r="Z252" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA252" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB252" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909122790 handle=https://www.ebay.com/itm/406909122790</t>
+        </is>
+      </c>
+      <c r="AC252" s="1" t="n">
+        <v>46149.07954709491</v>
+      </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -24995,6 +26920,43 @@
           <t>69fb881f2b1da07362014876</t>
         </is>
       </c>
+      <c r="S253" t="inlineStr">
+        <is>
+          <t>406909124585</t>
+        </is>
+      </c>
+      <c r="T253" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909124585</t>
+        </is>
+      </c>
+      <c r="U253" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V253" s="1" t="n">
+        <v>46149.07955925926</v>
+      </c>
+      <c r="Y253" s="1" t="n">
+        <v>46149.07955925926</v>
+      </c>
+      <c r="Z253" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA253" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB253" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909124585 handle=https://www.ebay.com/itm/406909124585</t>
+        </is>
+      </c>
+      <c r="AC253" s="1" t="n">
+        <v>46149.07955925926</v>
+      </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -25082,6 +27044,43 @@
           <t>69fb882c54fd3fbacf051371</t>
         </is>
       </c>
+      <c r="S254" t="inlineStr">
+        <is>
+          <t>406909125700</t>
+        </is>
+      </c>
+      <c r="T254" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909125700</t>
+        </is>
+      </c>
+      <c r="U254" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V254" s="1" t="n">
+        <v>46149.07957320602</v>
+      </c>
+      <c r="Y254" s="1" t="n">
+        <v>46149.07957320602</v>
+      </c>
+      <c r="Z254" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA254" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB254" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909125700 handle=https://www.ebay.com/itm/406909125700</t>
+        </is>
+      </c>
+      <c r="AC254" s="1" t="n">
+        <v>46149.07957320602</v>
+      </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -25169,6 +27168,43 @@
           <t>69fb883cce0d8cb5570fa7cc</t>
         </is>
       </c>
+      <c r="S255" t="inlineStr">
+        <is>
+          <t>406909126789</t>
+        </is>
+      </c>
+      <c r="T255" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909126789</t>
+        </is>
+      </c>
+      <c r="U255" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V255" s="1" t="n">
+        <v>46149.07958537037</v>
+      </c>
+      <c r="Y255" s="1" t="n">
+        <v>46149.07958537037</v>
+      </c>
+      <c r="Z255" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA255" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB255" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909126789 handle=https://www.ebay.com/itm/406909126789</t>
+        </is>
+      </c>
+      <c r="AC255" s="1" t="n">
+        <v>46149.07958537037</v>
+      </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -25256,6 +27292,43 @@
           <t>69fb8849e5402c478e0310af</t>
         </is>
       </c>
+      <c r="S256" t="inlineStr">
+        <is>
+          <t>406909127704</t>
+        </is>
+      </c>
+      <c r="T256" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909127704</t>
+        </is>
+      </c>
+      <c r="U256" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V256" s="1" t="n">
+        <v>46149.07959787037</v>
+      </c>
+      <c r="Y256" s="1" t="n">
+        <v>46149.07959787037</v>
+      </c>
+      <c r="Z256" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA256" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB256" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909127704 handle=https://www.ebay.com/itm/406909127704</t>
+        </is>
+      </c>
+      <c r="AC256" s="1" t="n">
+        <v>46149.07959787037</v>
+      </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -25343,6 +27416,43 @@
           <t>69fbae614c6544084c0f95ec</t>
         </is>
       </c>
+      <c r="S257" t="inlineStr">
+        <is>
+          <t>406909342825</t>
+        </is>
+      </c>
+      <c r="T257" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909342825</t>
+        </is>
+      </c>
+      <c r="U257" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V257" s="1" t="n">
+        <v>46149.07961042824</v>
+      </c>
+      <c r="Y257" s="1" t="n">
+        <v>46149.07961042824</v>
+      </c>
+      <c r="Z257" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA257" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB257" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909342825 handle=https://www.ebay.com/itm/406909342825</t>
+        </is>
+      </c>
+      <c r="AC257" s="1" t="n">
+        <v>46149.07961042824</v>
+      </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -25430,6 +27540,43 @@
           <t>69fbae7da7afceb9f70f2982</t>
         </is>
       </c>
+      <c r="S258" t="inlineStr">
+        <is>
+          <t>406909344491</t>
+        </is>
+      </c>
+      <c r="T258" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909344491</t>
+        </is>
+      </c>
+      <c r="U258" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V258" s="1" t="n">
+        <v>46149.07962293982</v>
+      </c>
+      <c r="Y258" s="1" t="n">
+        <v>46149.07962293982</v>
+      </c>
+      <c r="Z258" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA258" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB258" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909344491 handle=https://www.ebay.com/itm/406909344491</t>
+        </is>
+      </c>
+      <c r="AC258" s="1" t="n">
+        <v>46149.07962293982</v>
+      </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -25517,6 +27664,43 @@
           <t>69fbae974c6544084c0f9610</t>
         </is>
       </c>
+      <c r="S259" t="inlineStr">
+        <is>
+          <t>406909345291</t>
+        </is>
+      </c>
+      <c r="T259" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909345291</t>
+        </is>
+      </c>
+      <c r="U259" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V259" s="1" t="n">
+        <v>46149.07963510416</v>
+      </c>
+      <c r="Y259" s="1" t="n">
+        <v>46149.07963510416</v>
+      </c>
+      <c r="Z259" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA259" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB259" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909345291 handle=https://www.ebay.com/itm/406909345291</t>
+        </is>
+      </c>
+      <c r="AC259" s="1" t="n">
+        <v>46149.07963510416</v>
+      </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -25604,6 +27788,43 @@
           <t>69fbaea961c4aefdea04aaaf</t>
         </is>
       </c>
+      <c r="S260" t="inlineStr">
+        <is>
+          <t>406909353931</t>
+        </is>
+      </c>
+      <c r="T260" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909353931</t>
+        </is>
+      </c>
+      <c r="U260" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V260" s="1" t="n">
+        <v>46149.07964733796</v>
+      </c>
+      <c r="Y260" s="1" t="n">
+        <v>46149.07964733796</v>
+      </c>
+      <c r="Z260" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA260" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB260" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909353931 handle=https://www.ebay.com/itm/406909353931</t>
+        </is>
+      </c>
+      <c r="AC260" s="1" t="n">
+        <v>46149.07964733796</v>
+      </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -25691,6 +27912,43 @@
           <t>69fbaeb9f60a24b6d1034575</t>
         </is>
       </c>
+      <c r="S261" t="inlineStr">
+        <is>
+          <t>406909354903</t>
+        </is>
+      </c>
+      <c r="T261" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909354903</t>
+        </is>
+      </c>
+      <c r="U261" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V261" s="1" t="n">
+        <v>46149.07965949074</v>
+      </c>
+      <c r="Y261" s="1" t="n">
+        <v>46149.07965949074</v>
+      </c>
+      <c r="Z261" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA261" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB261" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909354903 handle=https://www.ebay.com/itm/406909354903</t>
+        </is>
+      </c>
+      <c r="AC261" s="1" t="n">
+        <v>46149.07965949074</v>
+      </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -25778,6 +28036,43 @@
           <t>69fbaecbb8dd7e2bb0094b7c</t>
         </is>
       </c>
+      <c r="S262" t="inlineStr">
+        <is>
+          <t>406909355853</t>
+        </is>
+      </c>
+      <c r="T262" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909355853</t>
+        </is>
+      </c>
+      <c r="U262" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V262" s="1" t="n">
+        <v>46149.07967215278</v>
+      </c>
+      <c r="Y262" s="1" t="n">
+        <v>46149.07967215278</v>
+      </c>
+      <c r="Z262" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA262" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB262" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909355853 handle=https://www.ebay.com/itm/406909355853</t>
+        </is>
+      </c>
+      <c r="AC262" s="1" t="n">
+        <v>46149.07967215278</v>
+      </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -25865,6 +28160,43 @@
           <t>69fbaedb4c6544084c0f9620</t>
         </is>
       </c>
+      <c r="S263" t="inlineStr">
+        <is>
+          <t>406909359949</t>
+        </is>
+      </c>
+      <c r="T263" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909359949</t>
+        </is>
+      </c>
+      <c r="U263" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V263" s="1" t="n">
+        <v>46149.07968435185</v>
+      </c>
+      <c r="Y263" s="1" t="n">
+        <v>46149.07968435185</v>
+      </c>
+      <c r="Z263" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA263" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB263" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909359949 handle=https://www.ebay.com/itm/406909359949</t>
+        </is>
+      </c>
+      <c r="AC263" s="1" t="n">
+        <v>46149.07968435185</v>
+      </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -25952,6 +28284,43 @@
           <t>69fbaeebce0d8cb5570fb7dc</t>
         </is>
       </c>
+      <c r="S264" t="inlineStr">
+        <is>
+          <t>406909364977</t>
+        </is>
+      </c>
+      <c r="T264" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909364977</t>
+        </is>
+      </c>
+      <c r="U264" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V264" s="1" t="n">
+        <v>46149.07969721065</v>
+      </c>
+      <c r="Y264" s="1" t="n">
+        <v>46149.07969721065</v>
+      </c>
+      <c r="Z264" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA264" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB264" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909364977 handle=https://www.ebay.com/itm/406909364977</t>
+        </is>
+      </c>
+      <c r="AC264" s="1" t="n">
+        <v>46149.07969721065</v>
+      </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -26039,6 +28408,43 @@
           <t>69fbaefcc6dfbcc11107aa91</t>
         </is>
       </c>
+      <c r="S265" t="inlineStr">
+        <is>
+          <t>406909368739</t>
+        </is>
+      </c>
+      <c r="T265" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909368739</t>
+        </is>
+      </c>
+      <c r="U265" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V265" s="1" t="n">
+        <v>46149.07971039352</v>
+      </c>
+      <c r="Y265" s="1" t="n">
+        <v>46149.07971039352</v>
+      </c>
+      <c r="Z265" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA265" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB265" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909368739 handle=https://www.ebay.com/itm/406909368739</t>
+        </is>
+      </c>
+      <c r="AC265" s="1" t="n">
+        <v>46149.07971039352</v>
+      </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -26126,6 +28532,43 @@
           <t>69fbaf12ff28e7d4030aba2d</t>
         </is>
       </c>
+      <c r="S266" t="inlineStr">
+        <is>
+          <t>406909373586</t>
+        </is>
+      </c>
+      <c r="T266" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909373586</t>
+        </is>
+      </c>
+      <c r="U266" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V266" s="1" t="n">
+        <v>46149.07972332176</v>
+      </c>
+      <c r="Y266" s="1" t="n">
+        <v>46149.07972332176</v>
+      </c>
+      <c r="Z266" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA266" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB266" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909373586 handle=https://www.ebay.com/itm/406909373586</t>
+        </is>
+      </c>
+      <c r="AC266" s="1" t="n">
+        <v>46149.07972332176</v>
+      </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -26213,6 +28656,43 @@
           <t>69fbc023f60a24b6d1034e5c</t>
         </is>
       </c>
+      <c r="S267" t="inlineStr">
+        <is>
+          <t>406909471020</t>
+        </is>
+      </c>
+      <c r="T267" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909471020</t>
+        </is>
+      </c>
+      <c r="U267" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V267" s="1" t="n">
+        <v>46149.07973618055</v>
+      </c>
+      <c r="Y267" s="1" t="n">
+        <v>46149.07973618055</v>
+      </c>
+      <c r="Z267" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA267" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB267" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909471020 handle=https://www.ebay.com/itm/406909471020</t>
+        </is>
+      </c>
+      <c r="AC267" s="1" t="n">
+        <v>46149.07973618055</v>
+      </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -26300,6 +28780,43 @@
           <t>69fbc0482b1da073620161ad</t>
         </is>
       </c>
+      <c r="S268" t="inlineStr">
+        <is>
+          <t>406909472775</t>
+        </is>
+      </c>
+      <c r="T268" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406909472775</t>
+        </is>
+      </c>
+      <c r="U268" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V268" s="1" t="n">
+        <v>46149.07974864583</v>
+      </c>
+      <c r="Y268" s="1" t="n">
+        <v>46149.07974864583</v>
+      </c>
+      <c r="Z268" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA268" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB268" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406909472775 handle=https://www.ebay.com/itm/406909472775</t>
+        </is>
+      </c>
+      <c r="AC268" s="1" t="n">
+        <v>46149.07974864583</v>
+      </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -26479,7 +28996,7 @@
       </c>
       <c r="O270" t="inlineStr">
         <is>
-          <t>Printify_PublishExternalPending_Mockups8</t>
+          <t>Printify_Published_Mockups8</t>
         </is>
       </c>
       <c r="P270" t="inlineStr">
@@ -26493,10 +29010,44 @@
         </is>
       </c>
       <c r="R270" s="1" t="n">
-        <v>46148.84302734954</v>
+        <v>46149.08054959491</v>
+      </c>
+      <c r="S270" t="inlineStr">
+        <is>
+          <t>406910056059</t>
+        </is>
+      </c>
+      <c r="T270" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406910056059</t>
+        </is>
+      </c>
+      <c r="U270" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="V270" s="1" t="n">
-        <v>46148.84259488426</v>
+        <v>46149.08084729167</v>
+      </c>
+      <c r="Y270" s="1" t="n">
+        <v>46149.07976099537</v>
+      </c>
+      <c r="Z270" t="n">
+        <v>5</v>
+      </c>
+      <c r="AA270" t="inlineStr">
+        <is>
+          <t>DELAY_POLL</t>
+        </is>
+      </c>
+      <c r="AB270" t="inlineStr">
+        <is>
+          <t>still within delayed propagation envelope age=381m attempts=4</t>
+        </is>
+      </c>
+      <c r="AC270" s="1" t="n">
+        <v>46149.07976099537</v>
       </c>
     </row>
     <row r="271">
@@ -26572,7 +29123,7 @@
       </c>
       <c r="O271" t="inlineStr">
         <is>
-          <t>Printify_PublishExternalPending_Mockups8</t>
+          <t>Printify_Published_Mockups8</t>
         </is>
       </c>
       <c r="P271" t="inlineStr">
@@ -26586,10 +29137,44 @@
         </is>
       </c>
       <c r="R271" s="1" t="n">
-        <v>46148.80971548611</v>
+        <v>46149.08102733796</v>
+      </c>
+      <c r="S271" t="inlineStr">
+        <is>
+          <t>406910057355</t>
+        </is>
+      </c>
+      <c r="T271" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406910057355</t>
+        </is>
+      </c>
+      <c r="U271" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="V271" s="1" t="n">
-        <v>46148.84261596065</v>
+        <v>46149.08132538194</v>
+      </c>
+      <c r="Y271" s="1" t="n">
+        <v>46149.07977336805</v>
+      </c>
+      <c r="Z271" t="n">
+        <v>5</v>
+      </c>
+      <c r="AA271" t="inlineStr">
+        <is>
+          <t>DELAY_POLL</t>
+        </is>
+      </c>
+      <c r="AB271" t="inlineStr">
+        <is>
+          <t>still within delayed propagation envelope age=381m attempts=4</t>
+        </is>
+      </c>
+      <c r="AC271" s="1" t="n">
+        <v>46149.07977336805</v>
       </c>
     </row>
     <row r="272">
@@ -26665,7 +29250,7 @@
       </c>
       <c r="O272" t="inlineStr">
         <is>
-          <t>Printify_PublishExternalPending_Mockups8</t>
+          <t>Printify_Published_Mockups8</t>
         </is>
       </c>
       <c r="P272" t="inlineStr">
@@ -26679,10 +29264,44 @@
         </is>
       </c>
       <c r="R272" s="1" t="n">
-        <v>46148.81078710648</v>
+        <v>46149.08149414352</v>
+      </c>
+      <c r="S272" t="inlineStr">
+        <is>
+          <t>406910058626</t>
+        </is>
+      </c>
+      <c r="T272" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406910058626</t>
+        </is>
+      </c>
+      <c r="U272" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="V272" s="1" t="n">
-        <v>46148.84263555556</v>
+        <v>46149.0817916088</v>
+      </c>
+      <c r="Y272" s="1" t="n">
+        <v>46149.07978571759</v>
+      </c>
+      <c r="Z272" t="n">
+        <v>5</v>
+      </c>
+      <c r="AA272" t="inlineStr">
+        <is>
+          <t>DELAY_POLL</t>
+        </is>
+      </c>
+      <c r="AB272" t="inlineStr">
+        <is>
+          <t>still within delayed propagation envelope age=381m attempts=4</t>
+        </is>
+      </c>
+      <c r="AC272" s="1" t="n">
+        <v>46149.07978571759</v>
       </c>
     </row>
     <row r="273">
@@ -26758,7 +29377,7 @@
       </c>
       <c r="O273" t="inlineStr">
         <is>
-          <t>Printify_PublishExternalPending_Mockups8</t>
+          <t>Printify_Published_Mockups8</t>
         </is>
       </c>
       <c r="P273" t="inlineStr">
@@ -26772,10 +29391,44 @@
         </is>
       </c>
       <c r="R273" s="1" t="n">
-        <v>46148.81192653935</v>
+        <v>46149.08194987269</v>
+      </c>
+      <c r="S273" t="inlineStr">
+        <is>
+          <t>406910059060</t>
+        </is>
+      </c>
+      <c r="T273" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406910059060</t>
+        </is>
+      </c>
+      <c r="U273" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="V273" s="1" t="n">
-        <v>46148.84265912037</v>
+        <v>46149.08224751157</v>
+      </c>
+      <c r="Y273" s="1" t="n">
+        <v>46149.07979824074</v>
+      </c>
+      <c r="Z273" t="n">
+        <v>5</v>
+      </c>
+      <c r="AA273" t="inlineStr">
+        <is>
+          <t>DELAY_POLL</t>
+        </is>
+      </c>
+      <c r="AB273" t="inlineStr">
+        <is>
+          <t>still within delayed propagation envelope age=381m attempts=4</t>
+        </is>
+      </c>
+      <c r="AC273" s="1" t="n">
+        <v>46149.07979824074</v>
       </c>
     </row>
     <row r="274">
@@ -26851,7 +29504,7 @@
       </c>
       <c r="O274" t="inlineStr">
         <is>
-          <t>Printify_PublishExternalPending_Mockups8</t>
+          <t>Printify_Published_Mockups8</t>
         </is>
       </c>
       <c r="P274" t="inlineStr">
@@ -26865,10 +29518,44 @@
         </is>
       </c>
       <c r="R274" s="1" t="n">
-        <v>46148.81309128472</v>
+        <v>46149.08243599537</v>
+      </c>
+      <c r="S274" t="inlineStr">
+        <is>
+          <t>406910060084</t>
+        </is>
+      </c>
+      <c r="T274" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406910060084</t>
+        </is>
+      </c>
+      <c r="U274" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="V274" s="1" t="n">
-        <v>46148.84267935185</v>
+        <v>46149.08288788194</v>
+      </c>
+      <c r="Y274" s="1" t="n">
+        <v>46149.07981099537</v>
+      </c>
+      <c r="Z274" t="n">
+        <v>5</v>
+      </c>
+      <c r="AA274" t="inlineStr">
+        <is>
+          <t>DELAY_POLL</t>
+        </is>
+      </c>
+      <c r="AB274" t="inlineStr">
+        <is>
+          <t>still within delayed propagation envelope age=381m attempts=4</t>
+        </is>
+      </c>
+      <c r="AC274" s="1" t="n">
+        <v>46149.07981099537</v>
       </c>
     </row>
     <row r="275">

</xml_diff>

<commit_message>
Execute first multi-track copy batch
</commit_message>
<xml_diff>
--- a/Database/eBay_listing.xlsx
+++ b/Database/eBay_listing.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ283"/>
+  <dimension ref="A1:AN283"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -600,6 +600,26 @@
           <t>SEO_Strike_Group</t>
         </is>
       </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>Multi_Track_Timestamp</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>Multi_Track_Track</t>
+        </is>
+      </c>
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>Multi_Track_Primary_Intent</t>
+        </is>
+      </c>
+      <c r="AN1" t="inlineStr">
+        <is>
+          <t>Multi_Track_Mockup_Mood</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -16986,12 +17006,12 @@
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>Zen Mentor-Grade Jade Phoenix Incense Altar 5x7 Acrylic Block for Meditation</t>
+          <t>Meditation Room Jade Relic Phoenix 5x7 Acrylic Block Shelf Decor Gift Study</t>
         </is>
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Elevate your meditation space with this Zen Mentor-Grade Jade Phoenix Incense Altar, a museum-quality acrylic block that captures the serene balance of ceremonial art. The imperial jade phoenix, with moonstone feather inlays and kintsugi vein detail, appears to float against an ink-wash nebula backdrop, while soft bioluminescent glow and floating lotus fragments evoke mindful tranquility. This piece transforms any desk, altar, or shelf into a focal point for daily reflection and aesthetic harmony.&lt;/p&gt;&lt;p&gt;Perfect for the collector or mindfulness practitioner, this 5x7 acrylic block offers a luminous, translucent depth that shifts with ambient light. Whether placed on a study desk, a meditation altar, or a minimalist shelf, its refined composition supports a calm, focused atmosphere. The solid white background ensures the phoenix and celestial details remain crisp and prominent, making it an ideal gift for mentors, Zen enthusiasts, or anyone seeking a unique decorative object.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 5x7 acrylic block with printed design&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; Premium clear acrylic with UV-resistant print, edge bevels for refined finish&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Size:&lt;/strong&gt; 5x7 inches (vertical orientation)&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Zen Mentor-Grade, inspired by imperial jade, moonstone, raku pottery, and ink-wash aesthetics&lt;/li&gt;&lt;li&gt;&lt;strong&gt;DNA Profile:&lt;/strong&gt; Ceremonial phoenix sculpture, floating incense altar, moonstone inlay, kintsugi vein detail, bioluminescent glow, lotus fragments, ink-wash nebula, bamboo silhouette, negative space composition, museum-grade collectible artifact&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Use Cases:&lt;/strong&gt; Meditation desk decor, altar accent, study shelf display, mindful gift for Zen practitioners, minimalist home decor, mentor appreciation gift&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the actual product customers receive. Additional images are bonus concept/detail reference images and do not represent extra products or selectable variations.&lt;/p&gt;</t>
+          <t>&lt;h2&gt;Meditation Room Jade Relic Phoenix 5x7 Acrylic Block Shelf Decor Gift Study&lt;/h2&gt;&lt;p&gt;This listing is part of a focused search-intent experiment for tea room accent. It is written for buyers decorating quiet shelves, meditation corners, gothic study desks, collector rooms, and deep-work apartments, not for generic wall-art browsing.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 5x7 vertical acrylic photo block, produced on demand through Printify.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Visual Mood:&lt;/strong&gt; Reading Nook Warm Lamp.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Design Language:&lt;/strong&gt; refractive depth, smoky jade color, internal glow, and premium desk-object presence.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Search Lane:&lt;/strong&gt; reading nook decor, meditation room wall art, tea room accent, quiet corner decor, dorm desk calm art, deep work visual.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; This is a single printed acrylic display block. The main artwork is the product customers receive; any additional gallery images are concept/detail references.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Acrylic-Zen-0006. Prior title: Meditation Room Jade Relic Jade Phoenix Incense Altar for 5x7 Acrylic Block&lt;/small&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="G173" t="inlineStr">
@@ -17066,6 +17086,31 @@
       </c>
       <c r="V173" s="1" t="n">
         <v>46148.85826324074</v>
+      </c>
+      <c r="AH173" t="inlineStr">
+        <is>
+          <t>MULTI_TRACK_SYNCED_PRINTIFY_PUBLISH</t>
+        </is>
+      </c>
+      <c r="AK173" t="inlineStr">
+        <is>
+          <t>2026-05-07 02:48:12 -0400</t>
+        </is>
+      </c>
+      <c r="AL173" t="inlineStr">
+        <is>
+          <t>A_LOW_COMPETITION_NICHE</t>
+        </is>
+      </c>
+      <c r="AM173" t="inlineStr">
+        <is>
+          <t>tea room accent</t>
+        </is>
+      </c>
+      <c r="AN173" t="inlineStr">
+        <is>
+          <t>reading_nook_warm_lamp</t>
+        </is>
       </c>
     </row>
     <row r="174">
@@ -17091,12 +17136,12 @@
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>Quiet Luxury Shelf Decor Sacred Lotus Meditation Bell for 5x7 Acrylic Photo</t>
+          <t>Meditation Room Jade Relic Quiet Luxury 5x7 Acrylic Block Shelf Decor Gift Wall</t>
         </is>
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>&lt;h2&gt;Quiet Luxury Shelf Decor Sacred Lotus Meditation Bell for 5x7 Acrylic Photo&lt;/h2&gt;&lt;p&gt;A Quiet Jade collection piece built for desks, bookshelves, altar corners, office focus spaces, and collector displays. The visual direction leans into smoky jade tones, quiet luxury decor language, kintsugi detail, and deep-work atmosphere instead of generic mass-market wall art.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 5x7 vertical acrylic photo block.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; Acrylic block display with depth, gloss, and light-reflective finish.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Zen collector aesthetic; smoky jade, wabi-sabi, scholar-room mood.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Best For:&lt;/strong&gt; apartment decor, reading nook styling, focused workspaces, collectors, and giftable room accents.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the physical product customers receive. Additional gallery images are concept, detail, or collection-reference views and are not extra products or selectable variations.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Search Themes:&lt;/strong&gt; Sacred Lotus Meditation Bell for, Smoky Jade, Quiet Luxury Decor, Deep Work Visuals, Reading Nook Decor, Wabi Sabi Decor, Scholar Room, Apartment Decor, Jade Art, Kintsugi Aesthetic, Collector Gift, Meditation Decor, Calm Desk Art&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Acrylic-Zen-0007; Subject: Sacred Lotus Meditation Bell for&lt;/small&gt;&lt;/p&gt;</t>
+          <t>&lt;h2&gt;Meditation Room Jade Relic Quiet Luxury 5x7 Acrylic Block Shelf Decor Gift Wall&lt;/h2&gt;&lt;p&gt;This listing is part of a focused search-intent experiment for meditation room wall art. It is written for buyers decorating quiet shelves, meditation corners, gothic study desks, collector rooms, and deep-work apartments, not for generic wall-art browsing.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 5x7 vertical acrylic photo block, produced on demand through Printify.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Visual Mood:&lt;/strong&gt; Reading Nook Warm Lamp.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Design Language:&lt;/strong&gt; refractive depth, smoky jade color, internal glow, and premium desk-object presence.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Search Lane:&lt;/strong&gt; reading nook decor, meditation room wall art, tea room accent, quiet corner decor, dorm desk calm art, deep work visual.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; This is a single printed acrylic display block. The main artwork is the product customers receive; any additional gallery images are concept/detail references.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Acrylic-Zen-0007. Prior title: Meditation Room Jade Relic Quiet Luxury Sacred Lotus Meditation 5x7 Acrylic&lt;/small&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="G174" t="inlineStr">
@@ -17194,7 +17239,27 @@
       </c>
       <c r="AH174" t="inlineStr">
         <is>
-          <t>QUIET_JADE_SYNCED_PRINTIFY_PUBLISH</t>
+          <t>MULTI_TRACK_SYNCED_PRINTIFY_PUBLISH</t>
+        </is>
+      </c>
+      <c r="AK174" t="inlineStr">
+        <is>
+          <t>2026-05-07 02:48:12 -0400</t>
+        </is>
+      </c>
+      <c r="AL174" t="inlineStr">
+        <is>
+          <t>A_LOW_COMPETITION_NICHE</t>
+        </is>
+      </c>
+      <c r="AM174" t="inlineStr">
+        <is>
+          <t>meditation room wall art</t>
+        </is>
+      </c>
+      <c r="AN174" t="inlineStr">
+        <is>
+          <t>reading_nook_warm_lamp</t>
         </is>
       </c>
     </row>
@@ -17741,12 +17806,12 @@
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>Gallery Desk Art Alchemist Divination Compass Occult 5x7 Acrylic Photo Block</t>
+          <t>Dark Study Smoky Jade Alchemist Divination Compass 5x7 Acrylic Block Shelf Gift</t>
         </is>
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t>&lt;h2&gt;Gallery Desk Art Alchemist Divination Compass Occult 5x7 Acrylic Photo Block&lt;/h2&gt;&lt;p&gt;A Quiet Jade collection piece built for desks, bookshelves, altar corners, office focus spaces, and collector displays. The visual direction leans into smoky jade tones, quiet luxury decor language, kintsugi detail, and deep-work atmosphere instead of generic mass-market wall art.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 5x7 vertical acrylic photo block.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; Acrylic block display with depth, gloss, and light-reflective finish.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Grimdark collector aesthetic; smoky jade, wabi-sabi, scholar-room mood.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Best For:&lt;/strong&gt; apartment decor, reading nook styling, focused workspaces, collectors, and giftable room accents.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the physical product customers receive. Additional gallery images are concept, detail, or collection-reference views and are not extra products or selectable variations.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Search Themes:&lt;/strong&gt; Alchemist Divination Compass Occult, Smoky Jade, Quiet Luxury Decor, Deep Work Visuals, Reading Nook Decor, Wabi Sabi Decor, Scholar Room, Apartment Decor, Jade Art, Kintsugi Aesthetic, Collector Gift, Gothic Study Decor, Alchemy Decor&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Acrylic-Grimdark-0085; Subject: Alchemist Divination Compass Occult&lt;/small&gt;&lt;/p&gt;</t>
+          <t>&lt;h2&gt;Dark Study Smoky Jade Alchemist Divination Compass 5x7 Acrylic Block Shelf Gift&lt;/h2&gt;&lt;p&gt;This listing is part of a focused search-intent experiment for dark study room decor. It is written for buyers decorating quiet shelves, meditation corners, gothic study desks, collector rooms, and deep-work apartments, not for generic wall-art browsing.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 5x7 vertical acrylic photo block, produced on demand through Printify.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Visual Mood:&lt;/strong&gt; Reading Nook Warm Lamp.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Design Language:&lt;/strong&gt; refractive depth, smoky jade color, internal glow, and premium desk-object presence.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Search Lane:&lt;/strong&gt; gothic shelf decor, moody desk display, occult library art, dark study room decor, collector shelf object, smoky jade relic.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; This is a single printed acrylic display block. The main artwork is the product customers receive; any additional gallery images are concept/detail references.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Acrylic-Grimdark-0085. Prior title: Dark Study Smoky Jade Alchemist Divination Compass Occult 5x7 Acrylic Block&lt;/small&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="G179" t="inlineStr">
@@ -17844,7 +17909,27 @@
       </c>
       <c r="AH179" t="inlineStr">
         <is>
-          <t>QUIET_JADE_SYNCED_PRINTIFY_PUBLISH</t>
+          <t>MULTI_TRACK_SYNCED_PRINTIFY_PUBLISH</t>
+        </is>
+      </c>
+      <c r="AK179" t="inlineStr">
+        <is>
+          <t>2026-05-07 02:48:12 -0400</t>
+        </is>
+      </c>
+      <c r="AL179" t="inlineStr">
+        <is>
+          <t>A_LOW_COMPETITION_NICHE</t>
+        </is>
+      </c>
+      <c r="AM179" t="inlineStr">
+        <is>
+          <t>dark study room decor</t>
+        </is>
+      </c>
+      <c r="AN179" t="inlineStr">
+        <is>
+          <t>reading_nook_warm_lamp</t>
         </is>
       </c>
     </row>
@@ -20471,12 +20556,12 @@
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>Soulbound Harbinger Torch Grimdark Gothic Lantern 5x7 Acrylic Print Dark Decor</t>
+          <t>Quiet Luxury Jade Relic Soulbound 5x7 Acrylic Block Shelf Decor Gift Study Wall</t>
         </is>
       </c>
       <c r="F201" t="inlineStr">
         <is>
-          <t>&lt;p&gt;This 5x7 acrylic print captures the &lt;strong&gt;Soulbound Harbinger's Torch&lt;/strong&gt;, a grimdark mentor-grade artifact where a magenta spirit flame swirls within cracked ghostly rose quartz glass, framed by ornate wrought iron wings. The refractive internal glow and high-contrast shadows create a premium collectible aesthetic for gothic or dark academia interiors.&lt;/p&gt;&lt;p&gt;Display this piece on a study desk, shelf, or altar to evoke themes of spirit vessels and forbidden knowledge. The durable acrylic surface with a glossy finish enhances the layered depth and bioluminescent details, making it a striking focal point in low-light settings.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 5x7 acrylic print with a clear stand for tabletop display.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; High-gloss acrylic with a rigid, scratch-resistant surface.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Size:&lt;/strong&gt; 5x7 inches (12.7 x 17.8 cm).&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Grimdark Mentor-Grade with wrought iron, ghostly rose quartz glass, and magenta spirit flame motifs.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;DNA Profile:&lt;/strong&gt; Wrought iron filigree, cracked translucent quartz, internal bioluminescent glow, kintsugi-like vein logic, floating accent fragments, refractive lighting, high-contrast shadows, museum-grade overhead fill.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Use Cases:&lt;/strong&gt; Gothic decor, dark academia study, spirit vessel collection, occult-inspired room accent, gift for grimdark enthusiasts.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the actual product customers receive. Additional images are bonus concept/detail reference images and do not represent extra products or selectable variations.&lt;/p&gt;&lt;p&gt;&lt;em&gt;Image Note: &lt;/em&gt;&lt;/p&gt;</t>
+          <t>&lt;h2&gt;Quiet Luxury Jade Relic Soulbound 5x7 Acrylic Block Shelf Decor Gift Study Wall&lt;/h2&gt;&lt;p&gt;This listing is part of a focused search-intent experiment for smoky jade relic. It is written for buyers decorating quiet shelves, meditation corners, gothic study desks, collector rooms, and deep-work apartments, not for generic wall-art browsing.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 5x7 vertical acrylic photo block, produced on demand through Printify.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Visual Mood:&lt;/strong&gt; Quiet Luxury Apartment.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Design Language:&lt;/strong&gt; refractive depth, smoky jade color, internal glow, and premium desk-object presence.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Search Lane:&lt;/strong&gt; gothic shelf decor, moody desk display, occult library art, dark study room decor, collector shelf object, smoky jade relic.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; This is a single printed acrylic display block. The main artwork is the product customers receive; any additional gallery images are concept/detail references.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Acrylic-Grimdark-0014. Prior title: Quiet Luxury Jade Relic Soulbound Harbinger Torch Lantern Print 5x7 Acrylic&lt;/small&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="G201" t="inlineStr">
@@ -20570,6 +20655,31 @@
       </c>
       <c r="AC201" s="1" t="n">
         <v>46149.00210729166</v>
+      </c>
+      <c r="AH201" t="inlineStr">
+        <is>
+          <t>MULTI_TRACK_SYNCED_PRINTIFY_PUBLISH</t>
+        </is>
+      </c>
+      <c r="AK201" t="inlineStr">
+        <is>
+          <t>2026-05-07 02:48:12 -0400</t>
+        </is>
+      </c>
+      <c r="AL201" t="inlineStr">
+        <is>
+          <t>A_LOW_COMPETITION_NICHE</t>
+        </is>
+      </c>
+      <c r="AM201" t="inlineStr">
+        <is>
+          <t>smoky jade relic</t>
+        </is>
+      </c>
+      <c r="AN201" t="inlineStr">
+        <is>
+          <t>quiet_luxury_apartment</t>
+        </is>
       </c>
     </row>
     <row r="202">
@@ -21091,12 +21201,12 @@
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>Abyssal Watcher Eternal Eye Grimdark Gothic Acrylic 5x7 Spirit Beacon Artifact</t>
+          <t>Quiet Luxury Jade Relic Abyssal 5x7 Acrylic Block Shelf Decor Gift Study Wall</t>
         </is>
       </c>
       <c r="F206" t="inlineStr">
         <is>
-          <t>&lt;p&gt;This grimdark acrylic print captures the Abyssal Watcher's Eternal Eye, a gothic lantern of wrought iron and ghostly aqua glass, its cyan spirit flame glowing with bioluminescent intensity. A premium artifact for collectors of dark fantasy and occult decor.&lt;/p&gt;&lt;p&gt;Display this 5x7 piece on a study desk, altar, or shelf to evoke a spirit beacon's watchful presence. The refractive lighting and high-contrast shadows create a museum-grade visual depth, perfect for adding a mentor-grade aesthetic to any room.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 5x7 acrylic print, ready to hang or stand&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; High-gloss acrylic with UV-resistant ink&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Size:&lt;/strong&gt; 5x7 inches (12.7 x 17.8 cm)&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Grimdark Mentor-Grade, gothic filigree, bioluminescent glow&lt;/li&gt;&lt;li&gt;&lt;strong&gt;DNA Profile:&lt;/strong&gt; Wrought iron, ghostly aqua glass, cyan spirit flame, micro-engraved surface relief, kintsugi-like vein logic&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Use Cases:&lt;/strong&gt; Gothic collectible display, altar decor, study desk accent, dark fantasy gift, spirit beacon aesthetic&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the actual product customers receive. Additional images are bonus concept/detail reference images and do not represent extra products or selectable variations.&lt;/p&gt;</t>
+          <t>&lt;h2&gt;Quiet Luxury Jade Relic Abyssal 5x7 Acrylic Block Shelf Decor Gift Study Wall&lt;/h2&gt;&lt;p&gt;This listing is part of a focused search-intent experiment for moody desk display. It is written for buyers decorating quiet shelves, meditation corners, gothic study desks, collector rooms, and deep-work apartments, not for generic wall-art browsing.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 5x7 vertical acrylic photo block, produced on demand through Printify.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Visual Mood:&lt;/strong&gt; Quiet Luxury Apartment.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Design Language:&lt;/strong&gt; refractive depth, smoky jade color, internal glow, and premium desk-object presence.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Search Lane:&lt;/strong&gt; gothic shelf decor, moody desk display, occult library art, dark study room decor, collector shelf object, smoky jade relic.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; This is a single printed acrylic display block. The main artwork is the product customers receive; any additional gallery images are concept/detail references.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Acrylic-Grimdark-0019. Prior title: Quiet Luxury Jade Relic Abyssal Watcher Eternal Eye Spirit 5x7 Acrylic Block&lt;/small&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="G206" t="inlineStr">
@@ -21190,6 +21300,31 @@
       </c>
       <c r="AC206" s="1" t="n">
         <v>46149.07901393519</v>
+      </c>
+      <c r="AH206" t="inlineStr">
+        <is>
+          <t>MULTI_TRACK_SYNCED_PRINTIFY_PUBLISH</t>
+        </is>
+      </c>
+      <c r="AK206" t="inlineStr">
+        <is>
+          <t>2026-05-07 02:48:12 -0400</t>
+        </is>
+      </c>
+      <c r="AL206" t="inlineStr">
+        <is>
+          <t>A_LOW_COMPETITION_NICHE</t>
+        </is>
+      </c>
+      <c r="AM206" t="inlineStr">
+        <is>
+          <t>moody desk display</t>
+        </is>
+      </c>
+      <c r="AN206" t="inlineStr">
+        <is>
+          <t>quiet_luxury_apartment</t>
+        </is>
       </c>
     </row>
     <row r="207">
@@ -21959,12 +22094,12 @@
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>Magenta Malice Lantern Grimdark Mentor-Grade 5x7 Acrylic Decor Dark Fantasy</t>
+          <t>Quiet Luxury Jade Relic Magenta 5x7 Acrylic Block Shelf Decor Gift Study Wall</t>
         </is>
       </c>
       <c r="F213" t="inlineStr">
         <is>
-          <t>&lt;p&gt;This 5x7 acrylic print captures the &lt;strong&gt;Magenta Malice Lantern&lt;/strong&gt;, a corrupted gothic artifact forged from blackened wrought iron with razor-sharp filigree. A violent magenta spirit flame thrashes against frosted rose-tinted glass, embodying a grimdark mentor-grade aesthetic. The piece balances corrupted elegance with vibrant bioluminescent depth, making it a striking focal point for dark fantasy collections.&lt;/p&gt;&lt;p&gt;Perfect for study desks, gothic libraries, or minimalist shelves, this print brings a touch of corrupted romance to your space. The high-gloss acrylic surface enhances the layered translucent depth and internal glow, while the 5x7 size fits neatly into any room. Use it as a conversation starter in a home office or as a bold accent in a bedroom gallery wall.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 5x7 acrylic print, ready to hang with a built-in easel stand&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; High-gloss acrylic with vivid UV-resistant inks&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Size:&lt;/strong&gt; 5x7 inches (12.7 x 17.8 cm)&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Grimdark Mentor-Grade – corrupted gothic, bioluminescent magenta, blackened iron filigree&lt;/li&gt;&lt;li&gt;&lt;strong&gt;DNA Profile:&lt;/strong&gt; Blackened Wrought Iron, Rose-Tinted Glass, Magenta Spirit Flame, Sharp Filigree, micro-engraved surface relief, layered translucent depth, subtle internal bioluminescent glow&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Use Cases:&lt;/strong&gt; Gothic decor, dark fantasy collection, mentor gift, study desk accent, bedroom wall art&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the actual product customers receive. Additional images are bonus concept/detail reference images and do not represent extra products or selectable variations.&lt;/p&gt;&lt;p&gt;&lt;em&gt;Image Note: &lt;/em&gt;&lt;/p&gt;</t>
+          <t>&lt;h2&gt;Quiet Luxury Jade Relic Magenta 5x7 Acrylic Block Shelf Decor Gift Study Wall&lt;/h2&gt;&lt;p&gt;This listing is part of a focused search-intent experiment for occult library art. It is written for buyers decorating quiet shelves, meditation corners, gothic study desks, collector rooms, and deep-work apartments, not for generic wall-art browsing.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 5x7 vertical acrylic photo block, produced on demand through Printify.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Visual Mood:&lt;/strong&gt; Quiet Luxury Apartment.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Design Language:&lt;/strong&gt; refractive depth, smoky jade color, internal glow, and premium desk-object presence.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Search Lane:&lt;/strong&gt; gothic shelf decor, moody desk display, occult library art, dark study room decor, collector shelf object, smoky jade relic.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; This is a single printed acrylic display block. The main artwork is the product customers receive; any additional gallery images are concept/detail references.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Acrylic-Grimdark-0027. Prior title: Quiet Luxury Jade Relic Magenta Malice Lantern Fantasy 5x7 Acrylic Block Desk&lt;/small&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="G213" t="inlineStr">
@@ -22058,6 +22193,31 @@
       </c>
       <c r="AC213" s="1" t="n">
         <v>46149.0790996875</v>
+      </c>
+      <c r="AH213" t="inlineStr">
+        <is>
+          <t>MULTI_TRACK_SYNCED_PRINTIFY_PUBLISH</t>
+        </is>
+      </c>
+      <c r="AK213" t="inlineStr">
+        <is>
+          <t>2026-05-07 02:48:12 -0400</t>
+        </is>
+      </c>
+      <c r="AL213" t="inlineStr">
+        <is>
+          <t>A_LOW_COMPETITION_NICHE</t>
+        </is>
+      </c>
+      <c r="AM213" t="inlineStr">
+        <is>
+          <t>occult library art</t>
+        </is>
+      </c>
+      <c r="AN213" t="inlineStr">
+        <is>
+          <t>quiet_luxury_apartment</t>
+        </is>
       </c>
     </row>
     <row r="214">
@@ -22579,12 +22739,12 @@
       </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t>Grimdark Ethereal Archway Soul Lantern 5x7 Acrylic Display Gothic Artifact Gift</t>
+          <t>Dark Study Smoky Jade Ethereal Archway Soul 5x7 Acrylic Block Shelf Decor Gift</t>
         </is>
       </c>
       <c r="F218" t="inlineStr">
         <is>
-          <t>&lt;p&gt;This grimdark mentor-grade acrylic display presents the Ethereal Archway Soul Lantern, a gothic artifact rendered in a 5x7 format. The design centers on a wrought iron archway silhouette framing a selenite-inlaid vessel, with a pearl-white spirit flame and floating talisman fragments against imperial jade glass panels. The ink-wash nebula patterns and soft ethereal glow evoke a collector-focused aesthetic, perfect for dark academia or gothic decor.&lt;/p&gt;&lt;p&gt;Ideal for study desks, bookshelves, or ritual spaces, this piece brings a mood of ancient mystery and intellectual depth. The micro-engraved surface relief and layered translucent depth mimic handcrafted edge bevels, while the refined kintsugi-like vein logic adds subtle texture. Use it as a conversation starter in a home library, or as a unique gift for lovers of grimdark fantasy and occult artifacts.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 5x7 acrylic print, ready to display&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; Premium acrylic with glossy finish&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Size:&lt;/strong&gt; 5x7 inches (12.7 x 17.8 cm)&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Grimdark Mentor-Grade, gothic collectible&lt;/li&gt;&lt;li&gt;&lt;strong&gt;DNA Profile:&lt;/strong&gt; Wrought iron archway, selenite inlays, pearl-white flame, talisman fragments, imperial jade glass, ink-wash nebula, soft ethereal glow, micro-engraved relief, kintsugi vein logic, floating accent fragments, cinematic rim lighting, museum-grade overhead fill&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Use Cases:&lt;/strong&gt; Study desk decor, bookshelf accent, gothic home art, dark academia gift, occult display, ritual space adornment&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the actual product customers receive. Additional images are bonus concept/detail reference images and do not represent extra products or selectable variations.&lt;/p&gt;&lt;p&gt;&lt;em&gt;Image Note: &lt;/em&gt;&lt;/p&gt;</t>
+          <t>&lt;h2&gt;Dark Study Smoky Jade Ethereal Archway Soul 5x7 Acrylic Block Shelf Decor Gift&lt;/h2&gt;&lt;p&gt;This listing is part of a focused search-intent experiment for dark study room decor. It is written for buyers decorating quiet shelves, meditation corners, gothic study desks, collector rooms, and deep-work apartments, not for generic wall-art browsing.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 5x7 vertical acrylic photo block, produced on demand through Printify.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Visual Mood:&lt;/strong&gt; Quiet Luxury Apartment.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Design Language:&lt;/strong&gt; refractive depth, smoky jade color, internal glow, and premium desk-object presence.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Search Lane:&lt;/strong&gt; gothic shelf decor, moody desk display, occult library art, dark study room decor, collector shelf object, smoky jade relic.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; This is a single printed acrylic display block. The main artwork is the product customers receive; any additional gallery images are concept/detail references.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Acrylic-Grimdark-0033. Prior title: Dark Study Smoky Jade Ethereal Archway Soul Lantern Artifact 5x7 Acrylic Block&lt;/small&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="G218" t="inlineStr">
@@ -22678,6 +22838,31 @@
       </c>
       <c r="AC218" s="1" t="n">
         <v>46149.0791625</v>
+      </c>
+      <c r="AH218" t="inlineStr">
+        <is>
+          <t>MULTI_TRACK_SYNCED_PRINTIFY_PUBLISH</t>
+        </is>
+      </c>
+      <c r="AK218" t="inlineStr">
+        <is>
+          <t>2026-05-07 02:48:12 -0400</t>
+        </is>
+      </c>
+      <c r="AL218" t="inlineStr">
+        <is>
+          <t>A_LOW_COMPETITION_NICHE</t>
+        </is>
+      </c>
+      <c r="AM218" t="inlineStr">
+        <is>
+          <t>dark study room decor</t>
+        </is>
+      </c>
+      <c r="AN218" t="inlineStr">
+        <is>
+          <t>quiet_luxury_apartment</t>
+        </is>
       </c>
     </row>
     <row r="219">
@@ -23199,12 +23384,12 @@
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t>Quiet Luxury Desk Relic Rose Quartz Chapel Soul Lantern 5x7 Acrylic Block Decor</t>
+          <t>Collector Shelf Smoky Jade Quiet Luxury 5x7 Acrylic Block Shelf Decor Gift Wall</t>
         </is>
       </c>
       <c r="F223" t="inlineStr">
         <is>
-          <t>&lt;h2&gt;Quiet Luxury Desk Relic Rose Quartz Chapel Soul Lantern 5x7 Acrylic Block Decor&lt;/h2&gt;&lt;p&gt;This is part of a fast A/B traffic test built around higher-intent buyer scenes: quiet luxury apartment shelves, gothic study desks, collector corners, and deep-work rooms. The style leans into smoky jade glow, acrylic depth, refractive light, and gallery-object presence, avoiding generic mass-market wording.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 5x7 vertical acrylic photo block, produced on demand through Printify.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Visual Lane:&lt;/strong&gt; A Quiet Luxury Desk Object&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Grimdark with Quiet Jade / Deep Work positioning.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the physical product customers receive. Additional gallery images are concept, detail, or collection-reference views and are not extra products or selectable variations.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Acrylic-Grimdark-0038&lt;/small&gt;&lt;/p&gt;</t>
+          <t>&lt;h2&gt;Collector Shelf Smoky Jade Quiet Luxury 5x7 Acrylic Block Shelf Decor Gift Wall&lt;/h2&gt;&lt;p&gt;This listing is part of a focused search-intent experiment for collector shelf object. It is written for buyers decorating quiet shelves, meditation corners, gothic study desks, collector rooms, and deep-work apartments, not for generic wall-art browsing.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 5x7 vertical acrylic photo block, produced on demand through Printify.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Visual Mood:&lt;/strong&gt; Reading Nook Warm Lamp.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Design Language:&lt;/strong&gt; refractive depth, smoky jade color, internal glow, and premium desk-object presence.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Search Lane:&lt;/strong&gt; gothic shelf decor, moody desk display, occult library art, dark study room decor, collector shelf object, smoky jade relic.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; This is a single printed acrylic display block. The main artwork is the product customers receive; any additional gallery images are concept/detail references.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Acrylic-Grimdark-0038. Prior title: Collector Shelf Smoky Jade Quiet Luxury Relic Rose Quartz 5x7 Acrylic Block&lt;/small&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="G223" t="inlineStr">
@@ -23263,7 +23448,7 @@
         </is>
       </c>
       <c r="R223" s="1" t="n">
-        <v>46149.08978430011</v>
+        <v>46149.08978430556</v>
       </c>
       <c r="S223" t="inlineStr">
         <is>
@@ -23281,11 +23466,11 @@
         </is>
       </c>
       <c r="V223" s="1" t="n">
-        <v>46149.09008196864</v>
+        <v>46149.0900819676</v>
       </c>
       <c r="AH223" t="inlineStr">
         <is>
-          <t>SEO_STRIKE_SYNCED_PRINTIFY_DRAFT</t>
+          <t>MULTI_TRACK_SYNCED_PRINTIFY_PUBLISH</t>
         </is>
       </c>
       <c r="AI223" t="inlineStr">
@@ -23296,6 +23481,26 @@
       <c r="AJ223" t="inlineStr">
         <is>
           <t>A_QUIET_LUXURY_DESK_OBJECT</t>
+        </is>
+      </c>
+      <c r="AK223" t="inlineStr">
+        <is>
+          <t>2026-05-07 02:48:12 -0400</t>
+        </is>
+      </c>
+      <c r="AL223" t="inlineStr">
+        <is>
+          <t>A_LOW_COMPETITION_NICHE</t>
+        </is>
+      </c>
+      <c r="AM223" t="inlineStr">
+        <is>
+          <t>collector shelf object</t>
+        </is>
+      </c>
+      <c r="AN223" t="inlineStr">
+        <is>
+          <t>reading_nook_warm_lamp</t>
         </is>
       </c>
     </row>
@@ -23386,7 +23591,7 @@
         </is>
       </c>
       <c r="R224" s="1" t="n">
-        <v>46149.09025860706</v>
+        <v>46149.09025861111</v>
       </c>
       <c r="S224" t="inlineStr">
         <is>
@@ -23404,7 +23609,7 @@
         </is>
       </c>
       <c r="V224" s="1" t="n">
-        <v>46149.09070339654</v>
+        <v>46149.0907033912</v>
       </c>
       <c r="AH224" t="inlineStr">
         <is>
@@ -23509,7 +23714,7 @@
         </is>
       </c>
       <c r="R225" s="1" t="n">
-        <v>46149.09086501994</v>
+        <v>46149.09086502315</v>
       </c>
       <c r="S225" t="inlineStr">
         <is>
@@ -23527,7 +23732,7 @@
         </is>
       </c>
       <c r="V225" s="1" t="n">
-        <v>46149.09116347688</v>
+        <v>46149.09116347222</v>
       </c>
       <c r="AH225" t="inlineStr">
         <is>
@@ -23692,12 +23897,12 @@
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>Dark Academia Archivist Gateway Poster 12x18 Vintage Study Room Decor Wall Gift</t>
+          <t>Reading Nook Smoky Jade Wall Art Archivist 12x18 Matte Poster Apartment Decor</t>
         </is>
       </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Step into the quiet majesty of the &lt;strong&gt;Archivist's Gateway of Catalogued Eternity&lt;/strong&gt;, a poster that transforms your study into a sanctuary of systematic wisdom. This mentor-grade artwork captures a moonstone and imperial jade archway leading to an eternal classification chamber, with brass indices and ink-wash clouds swirling around ancient calfskin pages. The dark academia aesthetic is perfect for those who revere organized knowledge and timeless beauty.&lt;/p&gt;&lt;p&gt;Printed on premium matte paper, this 12x18 poster brings cinematic chiaroscuro lighting and jade archival luminescence to your wall. Use it above a reading desk, in a home library, or as a focal point in a student's room to inspire deep focus and intellectual curiosity. The ultra-detailed moonstone cataloguing patterns and brass archival mechanisms reward close inspection, making it a collectible piece for book lovers and scholars alike.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 12x18 poster, ready to frame&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; Premium matte paper with archival-grade inks&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Size:&lt;/strong&gt; 12 inches by 18 inches (30.5 x 45.7 cm)&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Dark Academia, Mentor-Grade – moonstone, imperial jade, ancient calfskin, burnished brass, ink-wash nebula&lt;/li&gt;&lt;li&gt;&lt;strong&gt;DNA Profile:&lt;/strong&gt; Archivist's gateway, catalogued eternity, classification chamber, brass indices, jade archival luminescence, systematic wisdom, vintage study aesthetic&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Use Cases:&lt;/strong&gt; Study desk decor, home library accent, student room inspiration, vintage intellectual gift, book lover's wall art&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the actual product customers receive. Additional images are bonus concept/detail reference images and do not represent extra products or selectable variations.&lt;/p&gt;&lt;p&gt;&lt;em&gt;Image Note: &lt;/em&gt;&lt;/p&gt;</t>
+          <t>&lt;h2&gt;Reading Nook Smoky Jade Wall Art Archivist 12x18 Matte Poster Apartment Decor&lt;/h2&gt;&lt;p&gt;This listing is part of a focused search-intent experiment for dark academia reading nook. It is written for buyers decorating reading nooks, home libraries, dorm study walls, meditation rooms, and quiet apartment corners, not for generic wall-art browsing.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 12x18 matte poster, produced on demand through Printify.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Visual Mood:&lt;/strong&gt; Quiet Luxury Apartment.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Design Language:&lt;/strong&gt; matte paper mood, cinematic depth, smoky jade tones, and calm visual focus.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Search Lane:&lt;/strong&gt; dark academia reading nook, home library wall art, book nook decor, study room poster, scholar desk decor, dorm library print.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; This is a single printed poster. The main artwork is the product customers receive; any additional gallery images are concept/detail references.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Poster-Academia-0019. Prior title: Reading Nook Smoky Jade Wall Art Archivist Gateway Vintage 12x18 Matte Poster&lt;/small&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="G227" t="inlineStr">
@@ -23791,6 +23996,31 @@
       </c>
       <c r="AC227" s="1" t="n">
         <v>46149.07923866898</v>
+      </c>
+      <c r="AH227" t="inlineStr">
+        <is>
+          <t>MULTI_TRACK_SYNCED_PRINTIFY_PUBLISH</t>
+        </is>
+      </c>
+      <c r="AK227" t="inlineStr">
+        <is>
+          <t>2026-05-07 02:48:12 -0400</t>
+        </is>
+      </c>
+      <c r="AL227" t="inlineStr">
+        <is>
+          <t>A_LOW_COMPETITION_NICHE</t>
+        </is>
+      </c>
+      <c r="AM227" t="inlineStr">
+        <is>
+          <t>dark academia reading nook</t>
+        </is>
+      </c>
+      <c r="AN227" t="inlineStr">
+        <is>
+          <t>quiet_luxury_apartment</t>
+        </is>
       </c>
     </row>
     <row r="228">
@@ -28717,12 +28947,12 @@
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t>Mechanical Encyclopedia Sphere Dark Academia Aesthetic 12x18 Poster Study Room</t>
+          <t>Reading Nook Smoky Jade Wall Art Mechanical 12x18 Matte Poster Apartment Decor</t>
         </is>
       </c>
       <c r="F268" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;This poster presents the Mechanical Encyclopedia Sphere, a dark academia masterpiece that transforms a corroded iron vessel into an archive of forgotten engineering. The cracked technical glass and kintsugi repair seams, glowing with golden light, encase gravity-defying ancient books and blueprint manuscripts, while toxic jade bioluminescence casts an emerald glow across the scene. It is an immersive environment for the intellectual soul.&lt;/p&gt;&lt;p&gt;Printed on premium semi-gloss poster paper, this 12x18 inch piece is ideal for a study desk, library wall, or vintage-inspired workspace. The ultra-detailed corrosion and glass fracture patterns reward close inspection, making it a conversation starter for book lovers and industrial design enthusiasts. Use it to evoke a mood of scholarly mystery in your home or office.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 12x18 inch poster (unframed)&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; Premium semi-gloss poster paper (200 gsm)&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Size:&lt;/strong&gt; 12 x 18 inches (30.48 x 45.72 cm)&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Dark Academia, Mentor-Grade, Industrial Design&lt;/li&gt;&lt;li&gt;&lt;strong&gt;DNA Profile:&lt;/strong&gt; Corroded iron, cracked glass, kintsugi gold, toxic jade bioluminescence, ancient calfskin, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments with intentional negative space&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Use Cases:&lt;/strong&gt; Study room decor, library wall art, vintage intellectual gift for students or engineers, dark academia bedroom accent, office inspiration&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the actual product customers receive. Additional images are bonus concept/detail reference images and do not represent extra products or selectable variations.&lt;/p&gt;&lt;p&gt;&lt;em&gt;Image Note:&lt;/em&gt; </t>
+          <t>&lt;h2&gt;Reading Nook Smoky Jade Wall Art Mechanical 12x18 Matte Poster Apartment Decor&lt;/h2&gt;&lt;p&gt;This listing is part of a focused search-intent experiment for dark academia reading nook. It is written for buyers decorating reading nooks, home libraries, dorm study walls, meditation rooms, and quiet apartment corners, not for generic wall-art browsing.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 12x18 matte poster, produced on demand through Printify.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Visual Mood:&lt;/strong&gt; Reading Nook Warm Lamp.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Design Language:&lt;/strong&gt; matte paper mood, cinematic depth, smoky jade tones, and calm visual focus.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Search Lane:&lt;/strong&gt; dark academia reading nook, home library wall art, book nook decor, study room poster, scholar desk decor, dorm library print.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; This is a single printed poster. The main artwork is the product customers receive; any additional gallery images are concept/detail references.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Poster-Academia-0036. Prior title: Reading Nook Smoky Jade Wall Art Mechanical Encyclopedia Sphere 12x18 Matte&lt;/small&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="G268" t="inlineStr">
@@ -28816,6 +29046,31 @@
       </c>
       <c r="AC268" s="1" t="n">
         <v>46149.07974864583</v>
+      </c>
+      <c r="AH268" t="inlineStr">
+        <is>
+          <t>MULTI_TRACK_SYNCED_PRINTIFY_PUBLISH</t>
+        </is>
+      </c>
+      <c r="AK268" t="inlineStr">
+        <is>
+          <t>2026-05-07 02:48:12 -0400</t>
+        </is>
+      </c>
+      <c r="AL268" t="inlineStr">
+        <is>
+          <t>A_LOW_COMPETITION_NICHE</t>
+        </is>
+      </c>
+      <c r="AM268" t="inlineStr">
+        <is>
+          <t>dark academia reading nook</t>
+        </is>
+      </c>
+      <c r="AN268" t="inlineStr">
+        <is>
+          <t>reading_nook_warm_lamp</t>
+        </is>
       </c>
     </row>
     <row r="269">

</xml_diff>

<commit_message>
Verify cover gate replacement path
</commit_message>
<xml_diff>
--- a/Database/eBay_listing.xlsx
+++ b/Database/eBay_listing.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN283"/>
+  <dimension ref="A1:AN284"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -940,7 +940,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -14394,7 +14394,7 @@
       </c>
       <c r="O151" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="P151" t="inlineStr">
@@ -14629,7 +14629,7 @@
       </c>
       <c r="O153" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="P153" t="inlineStr">
@@ -14759,7 +14759,7 @@
       </c>
       <c r="O154" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="P154" t="inlineStr">
@@ -14864,7 +14864,7 @@
       </c>
       <c r="O155" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="P155" t="inlineStr">
@@ -14994,7 +14994,7 @@
       </c>
       <c r="O156" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="P156" t="inlineStr">
@@ -15124,7 +15124,7 @@
       </c>
       <c r="O157" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="P157" t="inlineStr">
@@ -15229,7 +15229,7 @@
       </c>
       <c r="O158" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="P158" t="inlineStr">
@@ -15334,7 +15334,7 @@
       </c>
       <c r="O159" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="P159" t="inlineStr">
@@ -15464,7 +15464,7 @@
       </c>
       <c r="O160" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="P160" t="inlineStr">
@@ -15594,7 +15594,7 @@
       </c>
       <c r="O161" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="P161" t="inlineStr">
@@ -15724,7 +15724,7 @@
       </c>
       <c r="O162" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="P162" t="inlineStr">
@@ -15854,7 +15854,7 @@
       </c>
       <c r="O163" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="P163" t="inlineStr">
@@ -15984,7 +15984,7 @@
       </c>
       <c r="O164" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="P164" t="inlineStr">
@@ -16089,7 +16089,7 @@
       </c>
       <c r="O165" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="P165" t="inlineStr">
@@ -16219,7 +16219,7 @@
       </c>
       <c r="O166" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="P166" t="inlineStr">
@@ -16349,7 +16349,7 @@
       </c>
       <c r="O167" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="P167" t="inlineStr">
@@ -16479,7 +16479,7 @@
       </c>
       <c r="O168" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="P168" t="inlineStr">
@@ -16584,7 +16584,7 @@
       </c>
       <c r="O169" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="P169" t="inlineStr">
@@ -16714,7 +16714,7 @@
       </c>
       <c r="O170" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="P170" t="inlineStr">
@@ -16844,7 +16844,7 @@
       </c>
       <c r="O171" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="P171" t="inlineStr">
@@ -17056,7 +17056,7 @@
       </c>
       <c r="O173" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="P173" t="inlineStr">
@@ -17186,7 +17186,7 @@
       </c>
       <c r="O174" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="P174" t="inlineStr">
@@ -17336,7 +17336,7 @@
       </c>
       <c r="O175" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="P175" t="inlineStr">
@@ -17466,7 +17466,7 @@
       </c>
       <c r="O176" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="P176" t="inlineStr">
@@ -17596,7 +17596,7 @@
       </c>
       <c r="O177" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="P177" t="inlineStr">
@@ -31013,6 +31013,134 @@
       </c>
       <c r="V283" s="1" t="n">
         <v>46148.98066784722</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0055-FIX1</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0055-FIX1</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>Zen</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>Sticker</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>Quiet Desk Sticker Pack Azure Dragon Warrior 4pc 6x6 Kiss-Cut Vinyl Laptop Gift</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>&lt;h2&gt;Quiet Desk Sticker Pack Azure Dragon Warrior 4pc 6x6 Kiss-Cut Vinyl Laptop Gift&lt;/h2&gt;&lt;p&gt;A Quiet Jade collection piece built for laptops, journals, planners, bottles, reading notebooks, and study desk gifts. The visual direction leans into smoky jade tones, quiet luxury decor language, kintsugi detail, and deep-work atmosphere instead of generic mass-market wall art.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 6x6 kiss-cut vinyl sticker sheet with four coordinated designs.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; Durable kiss-cut vinyl sticker sheet produced on demand through Printify.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Zen collector aesthetic; smoky jade, wabi-sabi, scholar-room mood.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Best For:&lt;/strong&gt; apartment decor, reading nook styling, focused workspaces, collectors, and giftable room accents.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the physical product customers receive. Additional gallery images are concept, detail, or collection-reference views and are not extra products or selectable variations.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Search Themes:&lt;/strong&gt; Azure Dragon Warrior, Smoky Jade, Quiet Luxury Decor, Deep Work Visuals, Reading Nook Decor, Wabi Sabi Decor, Scholar Room, Apartment Decor, Jade Art, Kintsugi Aesthetic, Collector Gift, Meditation Decor, Calm Desk Art&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Sticker-Zen-0055; Subject: Azure Dragon Warrior&lt;/small&gt;&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>$11.99</t>
+        </is>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>Warrior Azure dragon with Translucent Imperial Jade armor, Kintsugi Gold Veins repairs, Bioluminescent Glow eyes, and Internal Crystalline Structures weapons, , , , , 3D relief effect, sharp focus</t>
+        </is>
+      </c>
+      <c r="I284" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0055_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="J284" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0055_Ready_for_Steaming\Cover_Mockup.png</t>
+        </is>
+      </c>
+      <c r="K284" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0055_Ready_for_Steaming\Sticker-Zen-0055_U1_Grid.png</t>
+        </is>
+      </c>
+      <c r="L284" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0055_Ready_for_Steaming\Sticker-Zen-0055_U2_Grid.png</t>
+        </is>
+      </c>
+      <c r="M284" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0055_Ready_for_Steaming\Sticker-Zen-0055_U3_Grid.png</t>
+        </is>
+      </c>
+      <c r="N284" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0055_Ready_for_Steaming\Sticker-Zen-0055_U4_Grid.png</t>
+        </is>
+      </c>
+      <c r="O284" t="inlineStr">
+        <is>
+          <t>Printify_Published_Mockups3</t>
+        </is>
+      </c>
+      <c r="P284" t="inlineStr">
+        <is>
+          <t>2026-05-07 11:16:22 -0400</t>
+        </is>
+      </c>
+      <c r="Q284" t="inlineStr">
+        <is>
+          <t>69fcad74346e75ac9f07d550</t>
+        </is>
+      </c>
+      <c r="R284" s="1" t="n">
+        <v>46149.47507757742</v>
+      </c>
+      <c r="S284" t="inlineStr">
+        <is>
+          <t>406910984204</t>
+        </is>
+      </c>
+      <c r="T284" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406910984204</t>
+        </is>
+      </c>
+      <c r="U284" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V284" s="1" t="n">
+        <v>46149.4753887167</v>
+      </c>
+      <c r="AD284" t="inlineStr">
+        <is>
+          <t>2026-05-07 00:46:18 -0400</t>
+        </is>
+      </c>
+      <c r="AE284" t="inlineStr">
+        <is>
+          <t>Operation Quiet Jade</t>
+        </is>
+      </c>
+      <c r="AF284" t="inlineStr">
+        <is>
+          <t>Azure Dragon Warrior, Smoky Jade, Quiet Luxury Decor, Deep Work Visuals, Reading Nook Decor, Wabi Sabi Decor, Scholar Room, Apartment Decor, Jade Art, Kintsugi Aesthetic, Collector Gift, Meditation Decor, Calm Desk Art</t>
+        </is>
+      </c>
+      <c r="AG284" t="inlineStr">
+        <is>
+          <t>Sticker kept review-friendly; not part of high-ticket price lift.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Close sticker cover replacements
</commit_message>
<xml_diff>
--- a/Database/eBay_listing.xlsx
+++ b/Database/eBay_listing.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN284"/>
+  <dimension ref="A1:AN287"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6160,7 +6160,7 @@
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Retired_Replaced</t>
         </is>
       </c>
       <c r="P59" t="inlineStr">
@@ -6190,6 +6190,14 @@
       </c>
       <c r="V59" s="1" t="n">
         <v>46148.85754021991</v>
+      </c>
+      <c r="W59" s="1" t="n">
+        <v>46149.49644304398</v>
+      </c>
+      <c r="X59" t="inlineStr">
+        <is>
+          <t>ENDED_CONFIRMED_SELLER_HUB; Seller Hub success banner detected.; printify_external_detached</t>
+        </is>
       </c>
       <c r="AD59" t="inlineStr">
         <is>
@@ -6290,7 +6298,7 @@
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Retired_Replaced</t>
         </is>
       </c>
       <c r="P60" t="inlineStr">
@@ -6320,6 +6328,14 @@
       </c>
       <c r="V60" s="1" t="n">
         <v>46148.85755953703</v>
+      </c>
+      <c r="W60" s="1" t="n">
+        <v>46149.50266826389</v>
+      </c>
+      <c r="X60" t="inlineStr">
+        <is>
+          <t>ENDED_CONFIRMED_SELLER_HUB; Seller Hub success banner detected.; printify_external_detached</t>
+        </is>
       </c>
       <c r="AD60" t="inlineStr">
         <is>
@@ -6420,7 +6436,7 @@
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Retired_Replaced</t>
         </is>
       </c>
       <c r="P61" t="inlineStr">
@@ -6450,6 +6466,14 @@
       </c>
       <c r="V61" s="1" t="n">
         <v>46148.85758619213</v>
+      </c>
+      <c r="W61" s="1" t="n">
+        <v>46149.51885146759</v>
+      </c>
+      <c r="X61" t="inlineStr">
+        <is>
+          <t>ENDED_CONFIRMED_SELLER_HUB; Seller Hub success banner detected.; printify_external_detached</t>
+        </is>
       </c>
       <c r="AD61" t="inlineStr">
         <is>
@@ -31102,7 +31126,7 @@
         </is>
       </c>
       <c r="R284" s="1" t="n">
-        <v>46149.47507757742</v>
+        <v>46149.47507758102</v>
       </c>
       <c r="S284" t="inlineStr">
         <is>
@@ -31120,7 +31144,7 @@
         </is>
       </c>
       <c r="V284" s="1" t="n">
-        <v>46149.4753887167</v>
+        <v>46149.47538871528</v>
       </c>
       <c r="AD284" t="inlineStr">
         <is>
@@ -31138,6 +31162,388 @@
         </is>
       </c>
       <c r="AG284" t="inlineStr">
+        <is>
+          <t>Sticker kept review-friendly; not part of high-ticket price lift.</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0056-FIX1</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0056-FIX1</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>Zen</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>Sticker</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>Reading Nook Vinyl Set Dragon Cherry Blossom 4pc 6x6 Kiss-Cut Vinyl Laptop Gift</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>&lt;h2&gt;Reading Nook Vinyl Set Dragon Cherry Blossom 4pc 6x6 Kiss-Cut Vinyl Laptop Gift&lt;/h2&gt;&lt;p&gt;A Quiet Jade collection piece built for laptops, journals, planners, bottles, reading notebooks, and study desk gifts. The visual direction leans into smoky jade tones, quiet luxury decor language, kintsugi detail, and deep-work atmosphere instead of generic mass-market wall art.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 6x6 kiss-cut vinyl sticker sheet with four coordinated designs.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; Durable kiss-cut vinyl sticker sheet produced on demand through Printify.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Zen collector aesthetic; smoky jade, wabi-sabi, scholar-room mood.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Best For:&lt;/strong&gt; apartment decor, reading nook styling, focused workspaces, collectors, and giftable room accents.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the physical product customers receive. Additional gallery images are concept, detail, or collection-reference views and are not extra products or selectable variations.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Search Themes:&lt;/strong&gt; Dragon Cherry Blossom, Smoky Jade, Quiet Luxury Decor, Deep Work Visuals, Reading Nook Decor, Wabi Sabi Decor, Scholar Room, Apartment Decor, Jade Art, Kintsugi Aesthetic, Collector Gift, Meditation Decor, Calm Desk Art&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Sticker-Zen-0056; Subject: Dragon Cherry Blossom&lt;/small&gt;&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>$11.99</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>Zen dragon with Translucent Imperial Jade scales surrounded by cherry blossoms, Kintsugi Gold Veins branches, Bioluminescent Glow petals, and Internal Crystalline Structures dewdrops, , , , , 3D relief effect, sharp focus</t>
+        </is>
+      </c>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0056_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="J285" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0056_Ready_for_Steaming\Cover_Mockup.png</t>
+        </is>
+      </c>
+      <c r="K285" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0056_Ready_for_Steaming\Sticker-Zen-0056_U1_Grid.png</t>
+        </is>
+      </c>
+      <c r="L285" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0056_Ready_for_Steaming\Sticker-Zen-0056_U2_Grid.png</t>
+        </is>
+      </c>
+      <c r="M285" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0056_Ready_for_Steaming\Sticker-Zen-0056_U3_Grid.png</t>
+        </is>
+      </c>
+      <c r="N285" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0056_Ready_for_Steaming\Sticker-Zen-0056_U4_Grid.png</t>
+        </is>
+      </c>
+      <c r="O285" t="inlineStr">
+        <is>
+          <t>Printify_Published_Mockups3</t>
+        </is>
+      </c>
+      <c r="P285" t="inlineStr">
+        <is>
+          <t>2026-05-07 11:57:21 -0400</t>
+        </is>
+      </c>
+      <c r="Q285" t="inlineStr">
+        <is>
+          <t>69fcb688d0e6f406f20a3d2a</t>
+        </is>
+      </c>
+      <c r="R285" s="1" t="n">
+        <v>46149.50093743056</v>
+      </c>
+      <c r="S285" t="inlineStr">
+        <is>
+          <t>406911030956</t>
+        </is>
+      </c>
+      <c r="T285" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406911030956</t>
+        </is>
+      </c>
+      <c r="U285" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V285" s="1" t="n">
+        <v>46149.50125799768</v>
+      </c>
+      <c r="AD285" t="inlineStr">
+        <is>
+          <t>2026-05-07 00:46:18 -0400</t>
+        </is>
+      </c>
+      <c r="AE285" t="inlineStr">
+        <is>
+          <t>Operation Quiet Jade</t>
+        </is>
+      </c>
+      <c r="AF285" t="inlineStr">
+        <is>
+          <t>Dragon Cherry Blossom, Smoky Jade, Quiet Luxury Decor, Deep Work Visuals, Reading Nook Decor, Wabi Sabi Decor, Scholar Room, Apartment Decor, Jade Art, Kintsugi Aesthetic, Collector Gift, Meditation Decor, Calm Desk Art</t>
+        </is>
+      </c>
+      <c r="AG285" t="inlineStr">
+        <is>
+          <t>Sticker kept review-friendly; not part of high-ticket price lift.</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0057-FIX1</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0057-FIX1</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>Zen</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>Sticker</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>Wabi Sabi Journal Decals Moonlit Dragon 4pc 6x6 Kiss-Cut Vinyl Laptop Journal</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>&lt;h2&gt;Wabi Sabi Journal Decals Moonlit Dragon 4pc 6x6 Kiss-Cut Vinyl Laptop Journal&lt;/h2&gt;&lt;p&gt;A Quiet Jade collection piece built for laptops, journals, planners, bottles, reading notebooks, and study desk gifts. The visual direction leans into smoky jade tones, quiet luxury decor language, kintsugi detail, and deep-work atmosphere instead of generic mass-market wall art.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 6x6 kiss-cut vinyl sticker sheet with four coordinated designs.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; Durable kiss-cut vinyl sticker sheet produced on demand through Printify.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Zen collector aesthetic; smoky jade, wabi-sabi, scholar-room mood.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Best For:&lt;/strong&gt; apartment decor, reading nook styling, focused workspaces, collectors, and giftable room accents.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the physical product customers receive. Additional gallery images are concept, detail, or collection-reference views and are not extra products or selectable variations.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Search Themes:&lt;/strong&gt; Moonlit Dragon, Smoky Jade, Quiet Luxury Decor, Deep Work Visuals, Reading Nook Decor, Wabi Sabi Decor, Scholar Room, Apartment Decor, Jade Art, Kintsugi Aesthetic, Collector Gift, Meditation Decor, Calm Desk Art&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Sticker-Zen-0057; Subject: Moonlit Dragon&lt;/small&gt;&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>$11.99</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>Zen dragon under moonlight with Translucent Imperial Jade reflecting moonbeams, Kintsugi Gold Veins constellations, Bioluminescent Glow moonlight, and Internal Crystalline Structures stars, , , , , 3D relief effect, sharp focus</t>
+        </is>
+      </c>
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0057_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="J286" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0057_Ready_for_Steaming\Cover_Mockup.png</t>
+        </is>
+      </c>
+      <c r="K286" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0057_Ready_for_Steaming\Sticker-Zen-0057_U1_Grid.png</t>
+        </is>
+      </c>
+      <c r="L286" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0057_Ready_for_Steaming\Sticker-Zen-0057_U2_Grid.png</t>
+        </is>
+      </c>
+      <c r="M286" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0057_Ready_for_Steaming\Sticker-Zen-0057_U3_Grid.png</t>
+        </is>
+      </c>
+      <c r="N286" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0057_Ready_for_Steaming\Sticker-Zen-0057_U4_Grid.png</t>
+        </is>
+      </c>
+      <c r="O286" t="inlineStr">
+        <is>
+          <t>Printify_Published</t>
+        </is>
+      </c>
+      <c r="P286" t="inlineStr">
+        <is>
+          <t>2026-05-07 12:05:47 -0400</t>
+        </is>
+      </c>
+      <c r="Q286" t="inlineStr">
+        <is>
+          <t>69fcb8762007fddea00e4ebe</t>
+        </is>
+      </c>
+      <c r="R286" s="1" t="n">
+        <v>46149.5054065625</v>
+      </c>
+      <c r="S286" t="inlineStr">
+        <is>
+          <t>406911046712</t>
+        </is>
+      </c>
+      <c r="T286" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406911046712</t>
+        </is>
+      </c>
+      <c r="U286" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V286" s="1" t="n">
+        <v>46149.51745751157</v>
+      </c>
+      <c r="Y286" s="1" t="n">
+        <v>46149.50771107639</v>
+      </c>
+      <c r="Z286" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA286" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB286" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406911046712 handle=https://www.ebay.com/itm/406911046712</t>
+        </is>
+      </c>
+      <c r="AC286" s="1" t="n">
+        <v>46149.51745751157</v>
+      </c>
+      <c r="AD286" t="inlineStr">
+        <is>
+          <t>2026-05-07 00:46:18 -0400</t>
+        </is>
+      </c>
+      <c r="AE286" t="inlineStr">
+        <is>
+          <t>Operation Quiet Jade</t>
+        </is>
+      </c>
+      <c r="AF286" t="inlineStr">
+        <is>
+          <t>Moonlit Dragon, Smoky Jade, Quiet Luxury Decor, Deep Work Visuals, Reading Nook Decor, Wabi Sabi Decor, Scholar Room, Apartment Decor, Jade Art, Kintsugi Aesthetic, Collector Gift, Meditation Decor, Calm Desk Art</t>
+        </is>
+      </c>
+      <c r="AG286" t="inlineStr">
+        <is>
+          <t>Sticker kept review-friendly; not part of high-ticket price lift.</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0058-FIX1</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0058-FIX1</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>Zen</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>Sticker</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>Smoky Jade Sticker Set Dragon Calligraphy Serene Clean 4pc 6x6 Kiss-Cut Vinyl</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>&lt;h2&gt;Smoky Jade Sticker Set Dragon Calligraphy Serene Clean 4pc 6x6 Kiss-Cut Vinyl&lt;/h2&gt;&lt;p&gt;A Quiet Jade collection piece built for laptops, journals, planners, bottles, reading notebooks, and study desk gifts. The visual direction leans into smoky jade tones, quiet luxury decor language, kintsugi detail, and deep-work atmosphere instead of generic mass-market wall art.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 6x6 kiss-cut vinyl sticker sheet with four coordinated designs.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; Durable kiss-cut vinyl sticker sheet produced on demand through Printify.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Zen collector aesthetic; smoky jade, wabi-sabi, scholar-room mood.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Best For:&lt;/strong&gt; apartment decor, reading nook styling, focused workspaces, collectors, and giftable room accents.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the physical product customers receive. Additional gallery images are concept, detail, or collection-reference views and are not extra products or selectable variations.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Search Themes:&lt;/strong&gt; Dragon Calligraphy Serene Clean, Smoky Jade, Quiet Luxury Decor, Deep Work Visuals, Reading Nook Decor, Wabi Sabi Decor, Scholar Room, Apartment Decor, Jade Art, Kintsugi Aesthetic, Collector Gift, Meditation Decor, Calm Desk Art&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Sticker-Zen-0058; Subject: Dragon Calligraphy Serene Clean&lt;/small&gt;&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>$11.99</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>Zen dragon formed from Japanese calligraphy strokes using Translucent Imperial Jade ink, Kintsugi Gold Veins brushwork, Bioluminescent Glow highlights, and Internal Crystalline Structures ink splatters, , , , , 3D relief effect, sharp focus</t>
+        </is>
+      </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0058_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="J287" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0058_Ready_for_Steaming\Cover_Mockup.png</t>
+        </is>
+      </c>
+      <c r="K287" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0058_Ready_for_Steaming\Sticker-Zen-0058_U1_Grid.png</t>
+        </is>
+      </c>
+      <c r="L287" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0058_Ready_for_Steaming\Sticker-Zen-0058_U2_Grid.png</t>
+        </is>
+      </c>
+      <c r="M287" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0058_Ready_for_Steaming\Sticker-Zen-0058_U3_Grid.png</t>
+        </is>
+      </c>
+      <c r="N287" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0058_Ready_for_Steaming\Sticker-Zen-0058_U4_Grid.png</t>
+        </is>
+      </c>
+      <c r="O287" t="inlineStr">
+        <is>
+          <t>Printify_UI_Failed</t>
+        </is>
+      </c>
+      <c r="P287" t="inlineStr">
+        <is>
+          <t>2026-05-07 12:15:28 -0400</t>
+        </is>
+      </c>
+      <c r="Q287" t="inlineStr">
+        <is>
+          <t>69fcbabcbb3409c48f0e342c</t>
+        </is>
+      </c>
+      <c r="AD287" t="inlineStr">
+        <is>
+          <t>2026-05-07 00:46:18 -0400</t>
+        </is>
+      </c>
+      <c r="AE287" t="inlineStr">
+        <is>
+          <t>Operation Quiet Jade</t>
+        </is>
+      </c>
+      <c r="AF287" t="inlineStr">
+        <is>
+          <t>Dragon Calligraphy Serene Clean, Smoky Jade, Quiet Luxury Decor, Deep Work Visuals, Reading Nook Decor, Wabi Sabi Decor, Scholar Room, Apartment Decor, Jade Art, Kintsugi Aesthetic, Collector Gift, Meditation Decor, Calm Desk Art</t>
+        </is>
+      </c>
+      <c r="AG287" t="inlineStr">
         <is>
           <t>Sticker kept review-friendly; not part of high-ticket price lift.</t>
         </is>

</xml_diff>

<commit_message>
Advance cover replacement queue
</commit_message>
<xml_diff>
--- a/Database/eBay_listing.xlsx
+++ b/Database/eBay_listing.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN287"/>
+  <dimension ref="A1:AN288"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6468,7 +6468,7 @@
         <v>46148.85758619213</v>
       </c>
       <c r="W61" s="1" t="n">
-        <v>46149.51885146759</v>
+        <v>46149.5188514699</v>
       </c>
       <c r="X61" t="inlineStr">
         <is>
@@ -6574,7 +6574,7 @@
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Retired_Replaced</t>
         </is>
       </c>
       <c r="P62" t="inlineStr">
@@ -6604,6 +6604,14 @@
       </c>
       <c r="V62" s="1" t="n">
         <v>46148.85760666666</v>
+      </c>
+      <c r="W62" s="1" t="n">
+        <v>46149.52602256944</v>
+      </c>
+      <c r="X62" t="inlineStr">
+        <is>
+          <t>ENDED_CONFIRMED_SELLER_HUB; Seller Hub success banner detected.; printify_external_detached</t>
+        </is>
       </c>
       <c r="AD62" t="inlineStr">
         <is>
@@ -6704,7 +6712,7 @@
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Retired_Replaced</t>
         </is>
       </c>
       <c r="P63" t="inlineStr">
@@ -6734,6 +6742,14 @@
       </c>
       <c r="V63" s="1" t="n">
         <v>46148.85762224537</v>
+      </c>
+      <c r="W63" s="1" t="n">
+        <v>46149.53241861867</v>
+      </c>
+      <c r="X63" t="inlineStr">
+        <is>
+          <t>ENDED_CONFIRMED_SELLER_HUB; Seller Hub success banner detected.; printify_external_detached</t>
+        </is>
       </c>
       <c r="AD63" t="inlineStr">
         <is>
@@ -31515,7 +31531,7 @@
       </c>
       <c r="O287" t="inlineStr">
         <is>
-          <t>Printify_UI_Failed</t>
+          <t>Printify_Published</t>
         </is>
       </c>
       <c r="P287" t="inlineStr">
@@ -31528,6 +31544,46 @@
           <t>69fcbabcbb3409c48f0e342c</t>
         </is>
       </c>
+      <c r="R287" s="1" t="n">
+        <v>46149.52264045139</v>
+      </c>
+      <c r="S287" t="inlineStr">
+        <is>
+          <t>406911102240</t>
+        </is>
+      </c>
+      <c r="T287" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406911102240</t>
+        </is>
+      </c>
+      <c r="U287" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V287" s="1" t="n">
+        <v>46149.5236897338</v>
+      </c>
+      <c r="Y287" s="1" t="n">
+        <v>46149.5236897338</v>
+      </c>
+      <c r="Z287" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA287" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB287" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406911102240 handle=https://www.ebay.com/itm/406911102240</t>
+        </is>
+      </c>
+      <c r="AC287" s="1" t="n">
+        <v>46149.5236897338</v>
+      </c>
       <c r="AD287" t="inlineStr">
         <is>
           <t>2026-05-07 00:46:18 -0400</t>
@@ -31544,6 +31600,153 @@
         </is>
       </c>
       <c r="AG287" t="inlineStr">
+        <is>
+          <t>Sticker kept review-friendly; not part of high-ticket price lift.</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0060-FIX1</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0060-FIX1</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>Zen</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>Sticker</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>Reading Nook Vinyl Set Translucent Jade Dragon Serene Clean 4pc 6x6 Kiss-Cut</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>&lt;h2&gt;Reading Nook Vinyl Set Translucent Jade Dragon Serene Clean 4pc 6x6 Kiss-Cut&lt;/h2&gt;&lt;p&gt;A Quiet Jade collection piece built for laptops, journals, planners, bottles, reading notebooks, and study desk gifts. The visual direction leans into smoky jade tones, quiet luxury decor language, kintsugi detail, and deep-work atmosphere instead of generic mass-market wall art.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 6x6 kiss-cut vinyl sticker sheet with four coordinated designs.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; Durable kiss-cut vinyl sticker sheet produced on demand through Printify.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Zen collector aesthetic; smoky jade, wabi-sabi, scholar-room mood.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Best For:&lt;/strong&gt; apartment decor, reading nook styling, focused workspaces, collectors, and giftable room accents.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the physical product customers receive. Additional gallery images are concept, detail, or collection-reference views and are not extra products or selectable variations.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Search Themes:&lt;/strong&gt; Translucent Jade Dragon Serene Clean, Smoky Jade, Quiet Luxury Decor, Deep Work Visuals, Reading Nook Decor, Wabi Sabi Decor, Scholar Room, Apartment Decor, Jade Art, Kintsugi Aesthetic, Collector Gift, Meditation Decor, Calm Desk Art&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Sticker-Zen-0060; Subject: Translucent Jade Dragon Serene Clean&lt;/small&gt;&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>$11.99</t>
+        </is>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>A detailed sticker design of a Zen dragon, Translucent Imperial Jade material, Kintsugi Gold Veins, Bioluminescent Glow, Internal Crystalline Structures, , , , , 3D relief effect, sharp focus</t>
+        </is>
+      </c>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0060_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="J288" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0060_Ready_for_Steaming\Cover_Mockup.png</t>
+        </is>
+      </c>
+      <c r="K288" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0060_Ready_for_Steaming\Sticker-Zen-0060_U1_Grid.png</t>
+        </is>
+      </c>
+      <c r="L288" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0060_Ready_for_Steaming\Sticker-Zen-0060_U2_Grid.png</t>
+        </is>
+      </c>
+      <c r="M288" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0060_Ready_for_Steaming\Sticker-Zen-0060_U3_Grid.png</t>
+        </is>
+      </c>
+      <c r="N288" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0060_Ready_for_Steaming\Sticker-Zen-0060_U4_Grid.png</t>
+        </is>
+      </c>
+      <c r="O288" t="inlineStr">
+        <is>
+          <t>Printify_Published</t>
+        </is>
+      </c>
+      <c r="P288" t="inlineStr">
+        <is>
+          <t>2026-05-07 12:38:46 -0400</t>
+        </is>
+      </c>
+      <c r="Q288" t="inlineStr">
+        <is>
+          <t>69fcc02e6a069c45c0013c52</t>
+        </is>
+      </c>
+      <c r="R288" s="1" t="n">
+        <v>46149.52965991898</v>
+      </c>
+      <c r="S288" t="inlineStr">
+        <is>
+          <t>406911120974</t>
+        </is>
+      </c>
+      <c r="T288" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406911120974</t>
+        </is>
+      </c>
+      <c r="U288" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V288" s="1" t="n">
+        <v>46149.53064886574</v>
+      </c>
+      <c r="Y288" s="1" t="n">
+        <v>46149.53064886574</v>
+      </c>
+      <c r="Z288" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA288" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB288" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406911120974 handle=https://www.ebay.com/itm/406911120974</t>
+        </is>
+      </c>
+      <c r="AC288" s="1" t="n">
+        <v>46149.53064886574</v>
+      </c>
+      <c r="AD288" t="inlineStr">
+        <is>
+          <t>2026-05-07 00:46:18 -0400</t>
+        </is>
+      </c>
+      <c r="AE288" t="inlineStr">
+        <is>
+          <t>Operation Quiet Jade</t>
+        </is>
+      </c>
+      <c r="AF288" t="inlineStr">
+        <is>
+          <t>Translucent Jade Dragon Serene Clean, Smoky Jade, Quiet Luxury Decor, Deep Work Visuals, Reading Nook Decor, Wabi Sabi Decor, Scholar Room, Apartment Decor, Jade Art, Kintsugi Aesthetic, Collector Gift, Meditation Decor, Calm Desk Art</t>
+        </is>
+      </c>
+      <c r="AG288" t="inlineStr">
         <is>
           <t>Sticker kept review-friendly; not part of high-ticket price lift.</t>
         </is>

</xml_diff>

<commit_message>
Close cover replacement 0061
</commit_message>
<xml_diff>
--- a/Database/eBay_listing.xlsx
+++ b/Database/eBay_listing.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN288"/>
+  <dimension ref="A1:AN289"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6744,7 +6744,7 @@
         <v>46148.85762224537</v>
       </c>
       <c r="W63" s="1" t="n">
-        <v>46149.53241861867</v>
+        <v>46149.53241862269</v>
       </c>
       <c r="X63" t="inlineStr">
         <is>
@@ -6850,12 +6850,12 @@
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Retired_Replaced</t>
         </is>
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>4/29/2026  1:28:53 PM</t>
+          <t>5/7/2026  4:07:15 PM</t>
         </is>
       </c>
       <c r="Q64" t="inlineStr">
@@ -6880,6 +6880,14 @@
       </c>
       <c r="V64" s="1" t="n">
         <v>46148.8576396875</v>
+      </c>
+      <c r="W64" s="1" t="n">
+        <v>46149.68053679106</v>
+      </c>
+      <c r="X64" t="inlineStr">
+        <is>
+          <t>ENDED_CONFIRMED_SELLER_HUB; Seller Hub success banner detected.; printify_external_detached</t>
+        </is>
       </c>
       <c r="AD64" t="inlineStr">
         <is>
@@ -31747,6 +31755,134 @@
         </is>
       </c>
       <c r="AG288" t="inlineStr">
+        <is>
+          <t>Sticker kept review-friendly; not part of high-ticket price lift.</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0061-FIX1</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0061-FIX1</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>Zen</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>Sticker</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>Wabi Sabi Journal Decals Kintsugi Gold Dragon Serene Calm 4pc 6x6 Kiss-Cut Gift</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>&lt;h2&gt;Wabi Sabi Journal Decals Kintsugi Gold Dragon Serene Calm 4pc 6x6 Kiss-Cut Gift&lt;/h2&gt;&lt;p&gt;A Quiet Jade collection piece built for laptops, journals, planners, bottles, reading notebooks, and study desk gifts. The visual direction leans into smoky jade tones, quiet luxury decor language, kintsugi detail, and deep-work atmosphere instead of generic mass-market wall art.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 6x6 kiss-cut vinyl sticker sheet with four coordinated designs.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; Durable kiss-cut vinyl sticker sheet produced on demand through Printify.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Zen collector aesthetic; smoky jade, wabi-sabi, scholar-room mood.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Best For:&lt;/strong&gt; apartment decor, reading nook styling, focused workspaces, collectors, and giftable room accents.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the physical product customers receive. Additional gallery images are concept, detail, or collection-reference views and are not extra products or selectable variations.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Search Themes:&lt;/strong&gt; Kintsugi Gold Dragon Serene Calm, Smoky Jade, Quiet Luxury Decor, Deep Work Visuals, Reading Nook Decor, Wabi Sabi Decor, Scholar Room, Apartment Decor, Jade Art, Kintsugi Aesthetic, Collector Gift, Meditation Decor, Calm Desk Art&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Sticker-Zen-0061; Subject: Kintsugi Gold Dragon Serene Calm&lt;/small&gt;&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>$11.99</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>A Zen dragon sticker with Kintsugi Gold Veins repairing Translucent Imperial Jade, Bioluminescent Glow from cracks, Internal Crystalline Structures visible, , , , , 3D relief effect, sharp focus</t>
+        </is>
+      </c>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0061_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="J289" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0061_Ready_for_Steaming\Cover_Mockup.png</t>
+        </is>
+      </c>
+      <c r="K289" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0061_Ready_for_Steaming\Sticker-Zen-0061_U1_Grid.png</t>
+        </is>
+      </c>
+      <c r="L289" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0061_Ready_for_Steaming\Sticker-Zen-0061_U2_Grid.png</t>
+        </is>
+      </c>
+      <c r="M289" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0061_Ready_for_Steaming\Sticker-Zen-0061_U3_Grid.png</t>
+        </is>
+      </c>
+      <c r="N289" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0061_Ready_for_Steaming\Sticker-Zen-0061_U4_Grid.png</t>
+        </is>
+      </c>
+      <c r="O289" t="inlineStr">
+        <is>
+          <t>Printify_Published_Mockups3</t>
+        </is>
+      </c>
+      <c r="P289" t="inlineStr">
+        <is>
+          <t>2026-05-07 16:14:41 -0400</t>
+        </is>
+      </c>
+      <c r="Q289" t="inlineStr">
+        <is>
+          <t>69fcf2ccf2b2884ff107c609</t>
+        </is>
+      </c>
+      <c r="R289" s="1" t="n">
+        <v>46149.67832842593</v>
+      </c>
+      <c r="S289" t="inlineStr">
+        <is>
+          <t>406911452547</t>
+        </is>
+      </c>
+      <c r="T289" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406911452547</t>
+        </is>
+      </c>
+      <c r="U289" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V289" s="1" t="n">
+        <v>46149.67892783564</v>
+      </c>
+      <c r="AD289" t="inlineStr">
+        <is>
+          <t>2026-05-07 00:46:18 -0400</t>
+        </is>
+      </c>
+      <c r="AE289" t="inlineStr">
+        <is>
+          <t>Operation Quiet Jade</t>
+        </is>
+      </c>
+      <c r="AF289" t="inlineStr">
+        <is>
+          <t>Kintsugi Gold Dragon Serene Calm, Smoky Jade, Quiet Luxury Decor, Deep Work Visuals, Reading Nook Decor, Wabi Sabi Decor, Scholar Room, Apartment Decor, Jade Art, Kintsugi Aesthetic, Collector Gift, Meditation Decor, Calm Desk Art</t>
+        </is>
+      </c>
+      <c r="AG289" t="inlineStr">
         <is>
           <t>Sticker kept review-friendly; not part of high-ticket price lift.</t>
         </is>

</xml_diff>

<commit_message>
Close cover replacements 0062 0063
</commit_message>
<xml_diff>
--- a/Database/eBay_listing.xlsx
+++ b/Database/eBay_listing.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN289"/>
+  <dimension ref="A1:AN291"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6882,7 +6882,7 @@
         <v>46148.8576396875</v>
       </c>
       <c r="W64" s="1" t="n">
-        <v>46149.68053679106</v>
+        <v>46149.68053679398</v>
       </c>
       <c r="X64" t="inlineStr">
         <is>
@@ -6988,7 +6988,7 @@
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Retired_Replaced</t>
         </is>
       </c>
       <c r="P65" t="inlineStr">
@@ -7018,6 +7018,14 @@
       </c>
       <c r="V65" s="1" t="n">
         <v>46148.85765802083</v>
+      </c>
+      <c r="W65" s="1" t="n">
+        <v>46149.7010079051</v>
+      </c>
+      <c r="X65" t="inlineStr">
+        <is>
+          <t>ENDED_CONFIRMED_SELLER_HUB; Seller Hub success banner detected.; printify_external_detached</t>
+        </is>
       </c>
       <c r="AD65" t="inlineStr">
         <is>
@@ -7118,7 +7126,7 @@
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Retired_Replaced</t>
         </is>
       </c>
       <c r="P66" t="inlineStr">
@@ -7148,6 +7156,14 @@
       </c>
       <c r="V66" s="1" t="n">
         <v>46148.85767342593</v>
+      </c>
+      <c r="W66" s="1" t="n">
+        <v>46149.7045780371</v>
+      </c>
+      <c r="X66" t="inlineStr">
+        <is>
+          <t>ENDED_CONFIRMED_SELLER_HUB; Seller Hub success banner detected.; printify_external_detached</t>
+        </is>
       </c>
     </row>
     <row r="67">
@@ -31886,6 +31902,242 @@
         <is>
           <t>Sticker kept review-friendly; not part of high-ticket price lift.</t>
         </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0062-FIX1</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0062-FIX1</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>Zen</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>Sticker</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>Smoky Jade Sticker Set Bioluminescent Dragon 4pc 6x6 Kiss-Cut Vinyl Laptop Gift</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>&lt;h2&gt;Smoky Jade Sticker Set Bioluminescent Dragon 4pc 6x6 Kiss-Cut Vinyl Laptop Gift&lt;/h2&gt;&lt;p&gt;A Quiet Jade collection piece built for laptops, journals, planners, bottles, reading notebooks, and study desk gifts. The visual direction leans into smoky jade tones, quiet luxury decor language, kintsugi detail, and deep-work atmosphere instead of generic mass-market wall art.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 6x6 kiss-cut vinyl sticker sheet with four coordinated designs.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; Durable kiss-cut vinyl sticker sheet produced on demand through Printify.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Zen collector aesthetic; smoky jade, wabi-sabi, scholar-room mood.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Best For:&lt;/strong&gt; apartment decor, reading nook styling, focused workspaces, collectors, and giftable room accents.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the physical product customers receive. Additional gallery images are concept, detail, or collection-reference views and are not extra products or selectable variations.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Search Themes:&lt;/strong&gt; Bioluminescent Dragon, Smoky Jade, Quiet Luxury Decor, Deep Work Visuals, Reading Nook Decor, Wabi Sabi Decor, Scholar Room, Apartment Decor, Jade Art, Kintsugi Aesthetic, Collector Gift, Meditation Decor, Calm Desk Art&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Sticker-Zen-0062; Subject: Bioluminescent Dragon&lt;/small&gt;&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>$11.99</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>A glowing Zen dragon sticker with Bioluminescent Glow illuminating Translucent Imperial Jade body, Kintsugi Gold Veins, Internal Crystalline Structures glowing from within, , , , , 3D relief effect, sharp focus</t>
+        </is>
+      </c>
+      <c r="I290" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0062_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="J290" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0062_Ready_for_Steaming\Cover_Mockup.png</t>
+        </is>
+      </c>
+      <c r="K290" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0062_Ready_for_Steaming\Sticker-Zen-0062_U1_Grid.png</t>
+        </is>
+      </c>
+      <c r="L290" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0062_Ready_for_Steaming\Sticker-Zen-0062_U2_Grid.png</t>
+        </is>
+      </c>
+      <c r="M290" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0062_Ready_for_Steaming\Sticker-Zen-0062_U3_Grid.png</t>
+        </is>
+      </c>
+      <c r="N290" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0062_Ready_for_Steaming\Sticker-Zen-0062_U4_Grid.png</t>
+        </is>
+      </c>
+      <c r="O290" t="inlineStr">
+        <is>
+          <t>Printify_Published_Mockups3</t>
+        </is>
+      </c>
+      <c r="P290" t="inlineStr">
+        <is>
+          <t>2026-05-07 16:46:14 -0400</t>
+        </is>
+      </c>
+      <c r="Q290" t="inlineStr">
+        <is>
+          <t>69fcfa3363b7f727e7012b1a</t>
+        </is>
+      </c>
+      <c r="R290" s="1" t="n">
+        <v>46149.69972608797</v>
+      </c>
+      <c r="S290" t="inlineStr">
+        <is>
+          <t>406911488570</t>
+        </is>
+      </c>
+      <c r="T290" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406911488570</t>
+        </is>
+      </c>
+      <c r="U290" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V290" s="1" t="n">
+        <v>46149.70002454861</v>
+      </c>
+      <c r="AD290" t="inlineStr">
+        <is>
+          <t>2026-05-07 00:46:18 -0400</t>
+        </is>
+      </c>
+      <c r="AE290" t="inlineStr">
+        <is>
+          <t>Operation Quiet Jade</t>
+        </is>
+      </c>
+      <c r="AF290" t="inlineStr">
+        <is>
+          <t>Bioluminescent Dragon, Smoky Jade, Quiet Luxury Decor, Deep Work Visuals, Reading Nook Decor, Wabi Sabi Decor, Scholar Room, Apartment Decor, Jade Art, Kintsugi Aesthetic, Collector Gift, Meditation Decor, Calm Desk Art</t>
+        </is>
+      </c>
+      <c r="AG290" t="inlineStr">
+        <is>
+          <t>Sticker kept review-friendly; not part of high-ticket price lift.</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0063-FIX1</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0063-FIX1</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>Zen</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>Sticker</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>Crystalline Dragon Core 4pc 6x6 Kiss-Cut Sticker Zen Aesthetic Laptop Journal</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>&lt;h2&gt;Crystalline Dragon Core Sticker Kiss-Cut Sticker&lt;/h2&gt;&lt;p&gt;Bring calm and balance into your daily routine with this Crystalline Dragon Core Sticker zen aesthetic kiss-cut sticker.&lt;/p&gt;&lt;p&gt;Designed for study rooms, creative workspaces, shelves, gallery walls, and collectible aesthetic decor, this sticker blends niche aesthetic appeal with collectible mentor-grade artwork.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 6x6 kiss-cut sheet with 4 individual sticker designs.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; Durable kiss-cut vinyl sticker sheet with waterproof finish.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Size:&lt;/strong&gt; 6x6 kiss-cut sheet with four coordinated designs.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Zen Mentor-Grade; Zen aesthetic.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;DNA Profile:&lt;/strong&gt; A Zen dragon sticker focusing on Internal Crystalline Structures within Translucent Imperial Jade, Kintsugi Gold Veins as circuitry, Bioluminescent Glow from crystal formations, , , , , 3D relief effect, sharp focus&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Best For:&lt;/strong&gt; mindfulness lovers, minimalists, journal keepers, yoga enthusiasts, and peaceful room setups.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;SEO Keywords:&lt;/strong&gt; crystal core, geometric dragon, sacred geometry, mineral art, crystal healing, energy centers, chakra dragon, metaphysical, gemstone art, spiritual science&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the actual product customers receive. Additional images are bonus concept/detail reference images and do not represent extra products or selectable variations.&lt;/p&gt;&lt;p&gt;Complete the collection with matching Alchemy pieces.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Sticker-Zen-0063&lt;/small&gt;&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>$11.99</t>
+        </is>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>A Zen dragon sticker focusing on Internal Crystalline Structures within Translucent Imperial Jade, Kintsugi Gold Veins as circuitry, Bioluminescent Glow from crystal formations, , , , , 3D relief effect, sharp focus</t>
+        </is>
+      </c>
+      <c r="I291" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0063_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="J291" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0063_Ready_for_Steaming\Cover_Mockup.png</t>
+        </is>
+      </c>
+      <c r="K291" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0063_Ready_for_Steaming\Sticker-Zen-0063_U1_Grid.png</t>
+        </is>
+      </c>
+      <c r="L291" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0063_Ready_for_Steaming\Sticker-Zen-0063_U2_Grid.png</t>
+        </is>
+      </c>
+      <c r="M291" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0063_Ready_for_Steaming\Sticker-Zen-0063_U3_Grid.png</t>
+        </is>
+      </c>
+      <c r="N291" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0063_Ready_for_Steaming\Sticker-Zen-0063_U4_Grid.png</t>
+        </is>
+      </c>
+      <c r="O291" t="inlineStr">
+        <is>
+          <t>Printify_Published_Mockups3</t>
+        </is>
+      </c>
+      <c r="P291" t="inlineStr">
+        <is>
+          <t>2026-05-07 16:50:31 -0400</t>
+        </is>
+      </c>
+      <c r="Q291" t="inlineStr">
+        <is>
+          <t>69fcfb2d111bf518b6078098</t>
+        </is>
+      </c>
+      <c r="R291" s="1" t="n">
+        <v>46149.70332143518</v>
+      </c>
+      <c r="S291" t="inlineStr">
+        <is>
+          <t>406911494155</t>
+        </is>
+      </c>
+      <c r="T291" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406911494155</t>
+        </is>
+      </c>
+      <c r="U291" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V291" s="1" t="n">
+        <v>46149.70362003472</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Close cover replacement 0066
</commit_message>
<xml_diff>
--- a/Database/eBay_listing.xlsx
+++ b/Database/eBay_listing.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN291"/>
+  <dimension ref="A1:AN292"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7158,7 +7158,7 @@
         <v>46148.85767342593</v>
       </c>
       <c r="W66" s="1" t="n">
-        <v>46149.7045780371</v>
+        <v>46149.7045780324</v>
       </c>
       <c r="X66" t="inlineStr">
         <is>
@@ -7239,7 +7239,7 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Retired_Replaced</t>
         </is>
       </c>
       <c r="P67" t="inlineStr">
@@ -7269,6 +7269,14 @@
       </c>
       <c r="V67" s="1" t="n">
         <v>46148.85769063657</v>
+      </c>
+      <c r="W67" s="1" t="n">
+        <v>46149.70952028736</v>
+      </c>
+      <c r="X67" t="inlineStr">
+        <is>
+          <t>ENDED_CONFIRMED_SELLER_HUB; Seller Hub success banner detected.; printify_external_detached</t>
+        </is>
       </c>
     </row>
     <row r="68">
@@ -32138,6 +32146,114 @@
       </c>
       <c r="V291" s="1" t="n">
         <v>46149.70362003472</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0066-FIX1</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0066-FIX1</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>Zen</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>Sticker</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>Golden Vein Circuitry Dragon 4pc 6x6 Kiss-Cut Sticker Zen Aesthetic Laptop Gift</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>&lt;h2&gt;Golden Vein Circuitry Dragon Sticker Kiss-Cut Sticker&lt;/h2&gt;&lt;p&gt;Bring calm and balance into your daily routine with this Golden Vein Circuitry Dragon Sticker zen aesthetic kiss-cut sticker.&lt;/p&gt;&lt;p&gt;Designed for study rooms, creative workspaces, shelves, gallery walls, and collectible aesthetic decor, this sticker blends niche aesthetic appeal with collectible mentor-grade artwork.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 6x6 kiss-cut sheet with 4 individual sticker designs.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; Durable kiss-cut vinyl sticker sheet with waterproof finish.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Size:&lt;/strong&gt; 6x6 kiss-cut sheet with four coordinated designs.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Zen Mentor-Grade; Zen aesthetic.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;DNA Profile:&lt;/strong&gt; A cyber-Zen dragon sticker with Kintsugi Gold Veins as glowing circuitry on Translucent Imperial Jade, Bioluminescent Glow at connection nodes, Internal Crystalline Structures as processing cores, , , , , 3D relief effect, sharp focus&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Best For:&lt;/strong&gt; mindfulness lovers, minimalists, journal keepers, yoga enthusiasts, and peaceful room setups.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;SEO Keywords:&lt;/strong&gt; cyber dragon, tech spirituality, circuit board art, glitch art, digital zen, future Buddhism, neon circuits, cyberpunk, techwear, gamer culture&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the actual product customers receive. Additional images are bonus concept/detail reference images and do not represent extra products or selectable variations.&lt;/p&gt;&lt;p&gt;Complete the collection with matching Alchemy pieces.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Sticker-Zen-0066&lt;/small&gt;&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>$11.99</t>
+        </is>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>A cyber-Zen dragon sticker with Kintsugi Gold Veins as glowing circuitry on Translucent Imperial Jade, Bioluminescent Glow at connection nodes, Internal Crystalline Structures as processing cores, , , , , 3D relief effect, sharp focus</t>
+        </is>
+      </c>
+      <c r="I292" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0066_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="J292" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0066_Ready_for_Steaming\Cover_Mockup.png</t>
+        </is>
+      </c>
+      <c r="K292" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0066_Ready_for_Steaming\Sticker-Zen-0066_U1_Grid.png</t>
+        </is>
+      </c>
+      <c r="L292" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0066_Ready_for_Steaming\Sticker-Zen-0066_U2_Grid.png</t>
+        </is>
+      </c>
+      <c r="M292" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0066_Ready_for_Steaming\Sticker-Zen-0066_U3_Grid.png</t>
+        </is>
+      </c>
+      <c r="N292" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0066_Ready_for_Steaming\Sticker-Zen-0066_U4_Grid.png</t>
+        </is>
+      </c>
+      <c r="O292" t="inlineStr">
+        <is>
+          <t>Printify_Published_Mockups3</t>
+        </is>
+      </c>
+      <c r="P292" t="inlineStr">
+        <is>
+          <t>2026-05-07 16:58:26 -0400</t>
+        </is>
+      </c>
+      <c r="Q292" t="inlineStr">
+        <is>
+          <t>69fcfd2914568b768c07abd9</t>
+        </is>
+      </c>
+      <c r="R292" s="1" t="n">
+        <v>46149.70837517361</v>
+      </c>
+      <c r="S292" t="inlineStr">
+        <is>
+          <t>406911509730</t>
+        </is>
+      </c>
+      <c r="T292" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406911509730</t>
+        </is>
+      </c>
+      <c r="U292" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V292" s="1" t="n">
+        <v>46149.70867581019</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Close cover replacement 0069
</commit_message>
<xml_diff>
--- a/Database/eBay_listing.xlsx
+++ b/Database/eBay_listing.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN292"/>
+  <dimension ref="A1:AN293"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7271,7 +7271,7 @@
         <v>46148.85769063657</v>
       </c>
       <c r="W67" s="1" t="n">
-        <v>46149.70952028736</v>
+        <v>46149.70952028935</v>
       </c>
       <c r="X67" t="inlineStr">
         <is>
@@ -7570,7 +7570,7 @@
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Retired_Replaced</t>
         </is>
       </c>
       <c r="P70" t="inlineStr">
@@ -7600,6 +7600,14 @@
       </c>
       <c r="V70" s="1" t="n">
         <v>46148.85774657407</v>
+      </c>
+      <c r="W70" s="1" t="n">
+        <v>46149.71563981934</v>
+      </c>
+      <c r="X70" t="inlineStr">
+        <is>
+          <t>ENDED_CONFIRMED_SELLER_HUB; Seller Hub success banner detected.; printify_external_detached</t>
+        </is>
       </c>
     </row>
     <row r="71">
@@ -32254,6 +32262,114 @@
       </c>
       <c r="V292" s="1" t="n">
         <v>46149.70867581019</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0069-FIX1</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0069-FIX1</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>Zen</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>Sticker</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>Minimal Zen Dragon Guardian 4pc 6x6 Sticker Sheet Serene Mindful Clean Decor</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>&lt;h2&gt;Zen Dragon Guardian Sticker - Kiss-Cut Sticker&lt;/h2&gt;&lt;p&gt;A polished Zen aesthetic piece for students, remote workers, yoga lovers, and anyone building a serene everyday space. Designed for peaceful desks, journals, and small rituals, this Zen Dragon Guardian Sticker kiss-cut sticker carries a clean Zen mood.&lt;/p&gt;&lt;p&gt;The design works well across journal spreads, library shelves, dorm rooms, studio desks, and cozy personal collections, while the title, material notes, and DNA profile stay specific for easy comparison.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 6x6 kiss-cut sheet with 4 individual sticker designs.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; Durable kiss-cut vinyl sticker sheet with waterproof finish.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Size:&lt;/strong&gt; 6x6 kiss-cut sheet with four coordinated designs.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Zen Mentor-Grade; Zen aesthetic.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;DNA Profile:&lt;/strong&gt; A protective Zen dragon sticker in guardian pose with Translucent Imperial Jade scales, Kintsugi Gold Veins as armor seams, Bioluminescent Glow from eyes, Internal Crystalline Structures as power source, , , , , 3D relief effect, sharp focus&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Best For:&lt;/strong&gt; students, remote workers, yoga lovers, and anyone building a serene everyday space.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;SEO Keywords:&lt;/strong&gt; guardian dragon, protective symbol, armor art, spiritual protection, warrior zen, defensive art, talisman, amulet, good luck charm, safety symbol&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the actual product customers receive. Additional images are bonus concept/detail reference images and do not represent extra products or selectable variations.&lt;/p&gt;&lt;p&gt;Saved under the reference SKU below for easy collector matching.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Sticker-Zen-0069&lt;/small&gt;&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>$11.99</t>
+        </is>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>A protective Zen dragon sticker in guardian pose with Translucent Imperial Jade scales, Kintsugi Gold Veins as armor seams, Bioluminescent Glow from eyes, Internal Crystalline Structures as power source, , , , , 3D relief effect, sharp focus</t>
+        </is>
+      </c>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0069_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="J293" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0069_Ready_for_Steaming\Cover_Mockup.png</t>
+        </is>
+      </c>
+      <c r="K293" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0069_Ready_for_Steaming\Sticker-Zen-0069_U1_Grid.png</t>
+        </is>
+      </c>
+      <c r="L293" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0069_Ready_for_Steaming\Sticker-Zen-0069_U2_Grid.png</t>
+        </is>
+      </c>
+      <c r="M293" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0069_Ready_for_Steaming\Sticker-Zen-0069_U3_Grid.png</t>
+        </is>
+      </c>
+      <c r="N293" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0069_Ready_for_Steaming\Sticker-Zen-0069_U4_Grid.png</t>
+        </is>
+      </c>
+      <c r="O293" t="inlineStr">
+        <is>
+          <t>Printify_Published_Mockups3</t>
+        </is>
+      </c>
+      <c r="P293" t="inlineStr">
+        <is>
+          <t>2026-05-07 17:05:41 -0400</t>
+        </is>
+      </c>
+      <c r="Q293" t="inlineStr">
+        <is>
+          <t>69fcff15cd220b844e0f655c</t>
+        </is>
+      </c>
+      <c r="R293" s="1" t="n">
+        <v>46149.71467765046</v>
+      </c>
+      <c r="S293" t="inlineStr">
+        <is>
+          <t>406911531255</t>
+        </is>
+      </c>
+      <c r="T293" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406911531255</t>
+        </is>
+      </c>
+      <c r="U293" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V293" s="1" t="n">
+        <v>46149.71497859954</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Close cover replacements 0070 0071
</commit_message>
<xml_diff>
--- a/Database/eBay_listing.xlsx
+++ b/Database/eBay_listing.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN293"/>
+  <dimension ref="A1:AN295"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7602,7 +7602,7 @@
         <v>46148.85774657407</v>
       </c>
       <c r="W70" s="1" t="n">
-        <v>46149.71563981934</v>
+        <v>46149.71563981481</v>
       </c>
       <c r="X70" t="inlineStr">
         <is>
@@ -7683,7 +7683,7 @@
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Retired_Replaced</t>
         </is>
       </c>
       <c r="P71" t="inlineStr">
@@ -7713,6 +7713,14 @@
       </c>
       <c r="V71" s="1" t="n">
         <v>46148.85776375</v>
+      </c>
+      <c r="W71" s="1" t="n">
+        <v>46149.71832703704</v>
+      </c>
+      <c r="X71" t="inlineStr">
+        <is>
+          <t>ENDED_CONFIRMED_SELLER_HUB; Seller Hub success banner detected.; printify_external_detached</t>
+        </is>
       </c>
     </row>
     <row r="72">
@@ -7788,7 +7796,7 @@
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Retired_Replaced</t>
         </is>
       </c>
       <c r="P72" t="inlineStr">
@@ -7818,6 +7826,14 @@
       </c>
       <c r="V72" s="1" t="n">
         <v>46148.85778013889</v>
+      </c>
+      <c r="W72" s="1" t="n">
+        <v>46149.72013065044</v>
+      </c>
+      <c r="X72" t="inlineStr">
+        <is>
+          <t>ENDED_CONFIRMED_SELLER_HUB; Seller Hub success banner detected.; printify_external_detached</t>
+        </is>
       </c>
     </row>
     <row r="73">
@@ -32370,6 +32386,222 @@
       </c>
       <c r="V293" s="1" t="n">
         <v>46149.71497859954</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0070-FIX1</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0070-FIX1</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>Zen</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>Sticker</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>Minimal Zen Jade Phoenix Ascension 4pc 6x6 Sticker Sheet Serene Mindful Clean</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>&lt;h2&gt;Jade Phoenix Ascension - Kiss-Cut Sticker&lt;/h2&gt;&lt;p&gt;A polished Zen aesthetic piece for students, remote workers, yoga lovers, and anyone building a serene everyday space. Designed for peaceful desks, journals, and small rituals, this Jade Phoenix Ascension kiss-cut sticker carries a clean Zen mood.&lt;/p&gt;&lt;p&gt;The design works well across journal spreads, library shelves, dorm rooms, studio desks, and cozy personal collections, while the title, material notes, and DNA profile stay specific for easy comparison.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 6x6 kiss-cut sheet with 4 individual sticker designs.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; Durable kiss-cut vinyl sticker sheet with waterproof finish.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Size:&lt;/strong&gt; 6x6 kiss-cut sheet with four coordinated designs.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Zen Mentor-Grade; Zen aesthetic.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;DNA Profile:&lt;/strong&gt; A majestic phoenix rising from translucent moonstone flames, wings spread with imperial jade feather inlays, floating Daoist Fulu talisman fragments orbiting the bird, ink-wash nebula trailing behind, ethereal bioluminescence emanating from wing tips, zen-mythic aesthetic, , , , , , person, text, watermark&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Best For:&lt;/strong&gt; students, remote workers, yoga lovers, and anyone building a serene everyday space.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;SEO Keywords:&lt;/strong&gt; phoenix sticker, jade phoenix, moonstone art, spiritual bird, zen phoenix, celestial creature, mythic phoenix, translucent wings, Daoist talisman, bioluminescent design&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the actual product customers receive. Additional images are bonus concept/detail reference images and do not represent extra products or selectable variations.&lt;/p&gt;&lt;p&gt;Saved under the reference SKU below for easy collector matching.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Sticker-Zen-0070&lt;/small&gt;&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>$11.99</t>
+        </is>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>A majestic phoenix rising from translucent moonstone flames, wings spread with imperial jade feather inlays, floating Daoist Fulu talisman fragments orbiting the bird, ink-wash nebula trailing behind, ethereal bioluminescence emanating from wing tips, zen-mythic aesthetic, , , , , , person, text, watermark</t>
+        </is>
+      </c>
+      <c r="I294" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0070_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="J294" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0070_Ready_for_Steaming\Cover_Mockup.png</t>
+        </is>
+      </c>
+      <c r="K294" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0070_Ready_for_Steaming\Sticker-Zen-0070_U1_Grid.png</t>
+        </is>
+      </c>
+      <c r="L294" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0070_Ready_for_Steaming\Sticker-Zen-0070_U2_Grid.png</t>
+        </is>
+      </c>
+      <c r="M294" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0070_Ready_for_Steaming\Sticker-Zen-0070_U3_Grid.png</t>
+        </is>
+      </c>
+      <c r="N294" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0070_Ready_for_Steaming\Sticker-Zen-0070_U4_Grid.png</t>
+        </is>
+      </c>
+      <c r="O294" t="inlineStr">
+        <is>
+          <t>Printify_Published_Mockups3</t>
+        </is>
+      </c>
+      <c r="P294" t="inlineStr">
+        <is>
+          <t>2026-05-07 17:12:09 -0400</t>
+        </is>
+      </c>
+      <c r="Q294" t="inlineStr">
+        <is>
+          <t>69fd002f096d6b4f0000a934</t>
+        </is>
+      </c>
+      <c r="R294" s="1" t="n">
+        <v>46149.71738046296</v>
+      </c>
+      <c r="S294" t="inlineStr">
+        <is>
+          <t>406911541926</t>
+        </is>
+      </c>
+      <c r="T294" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406911541926</t>
+        </is>
+      </c>
+      <c r="U294" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V294" s="1" t="n">
+        <v>46149.71768587963</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0071-FIX1</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>Sticker-Zen-0071-FIX1</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>Zen</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>Sticker</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>Zen Aesthetic Lotus Lantern Vessel 4pc 6x6 Kiss-Cut Sticker Laptop Journal Gift</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>&lt;h2&gt;Lotus Lantern Vessel Kiss-Cut Sticker&lt;/h2&gt;&lt;p&gt;Bring calm and balance into your daily routine with this Lotus Lantern Vessel zen aesthetic kiss-cut sticker.&lt;/p&gt;&lt;p&gt;Designed for study rooms, creative workspaces, shelves, gallery walls, and collectible aesthetic decor, this sticker blends niche aesthetic appeal with collectible mentor-grade artwork.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 6x6 kiss-cut sheet with 4 individual sticker designs.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; Durable kiss-cut vinyl sticker sheet with waterproof finish.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Size:&lt;/strong&gt; 6x6 kiss-cut sheet with four coordinated designs.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Zen Mentor-Grade; Zen aesthetic.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;DNA Profile:&lt;/strong&gt; An ornate lotus-shaped lantern vessel crafted from translucent moonstone petals and imperial jade stem, ink-wash nebula wisps flowing from interior chamber, floating Daoist Fulu talisman fragments circling the base, ethereal bioluminescence glowing within, zen-mythic aesthetic, , , , , , person, text, watermark&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Best For:&lt;/strong&gt; mindfulness lovers, minimalists, journal keepers, yoga enthusiasts, and peaceful room setups.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;SEO Keywords:&lt;/strong&gt; lotus lantern, jade vessel, moonstone container, spiritual lamp, zen lantern, celestial vessel, ritual lantern, translucent lotus, Daoist artifact, bioluminescent glow&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the actual product customers receive. Additional images are bonus concept/detail reference images and do not represent extra products or selectable variations.&lt;/p&gt;&lt;p&gt;Complete the collection with matching Alchemy pieces.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Sticker-Zen-0071&lt;/small&gt;&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>$11.99</t>
+        </is>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>An ornate lotus-shaped lantern vessel crafted from translucent moonstone petals and imperial jade stem, ink-wash nebula wisps flowing from interior chamber, floating Daoist Fulu talisman fragments circling the base, ethereal bioluminescence glowing within, zen-mythic aesthetic, , , , , , person, text, watermark</t>
+        </is>
+      </c>
+      <c r="I295" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0071_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="J295" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0071_Ready_for_Steaming\Cover_Mockup.png</t>
+        </is>
+      </c>
+      <c r="K295" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0071_Ready_for_Steaming\Sticker-Zen-0071_U1_Grid.png</t>
+        </is>
+      </c>
+      <c r="L295" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0071_Ready_for_Steaming\Sticker-Zen-0071_U2_Grid.png</t>
+        </is>
+      </c>
+      <c r="M295" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0071_Ready_for_Steaming\Sticker-Zen-0071_U3_Grid.png</t>
+        </is>
+      </c>
+      <c r="N295" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Sticker\Kiss-Cut\MASTER_Sticker-Zen-0071_Ready_for_Steaming\Sticker-Zen-0071_U4_Grid.png</t>
+        </is>
+      </c>
+      <c r="O295" t="inlineStr">
+        <is>
+          <t>Printify_Published_Mockups3</t>
+        </is>
+      </c>
+      <c r="P295" t="inlineStr">
+        <is>
+          <t>2026-05-07 17:14:44 -0400</t>
+        </is>
+      </c>
+      <c r="Q295" t="inlineStr">
+        <is>
+          <t>69fd00ca9f7703138202688c</t>
+        </is>
+      </c>
+      <c r="R295" s="1" t="n">
+        <v>46149.71918982639</v>
+      </c>
+      <c r="S295" t="inlineStr">
+        <is>
+          <t>406911551031</t>
+        </is>
+      </c>
+      <c r="T295" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406911551031</t>
+        </is>
+      </c>
+      <c r="U295" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V295" s="1" t="n">
+        <v>46149.71949134259</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Promote non-sticker cover review replacements
</commit_message>
<xml_diff>
--- a/Database/eBay_listing.xlsx
+++ b/Database/eBay_listing.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN295"/>
+  <dimension ref="A1:AN296"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7828,7 +7828,7 @@
         <v>46148.85778013889</v>
       </c>
       <c r="W72" s="1" t="n">
-        <v>46149.72013065044</v>
+        <v>46149.72013064815</v>
       </c>
       <c r="X72" t="inlineStr">
         <is>
@@ -14960,7 +14960,7 @@
       </c>
       <c r="O155" t="inlineStr">
         <is>
-          <t>Printify_PrimaryFix_Needed</t>
+          <t>Retired_Replaced</t>
         </is>
       </c>
       <c r="P155" t="inlineStr">
@@ -14990,6 +14990,14 @@
       </c>
       <c r="V155" s="1" t="n">
         <v>46148.85789751157</v>
+      </c>
+      <c r="W155" s="1" t="n">
+        <v>46149.72674940436</v>
+      </c>
+      <c r="X155" t="inlineStr">
+        <is>
+          <t>ENDED_CONFIRMED_SELLER_HUB; Seller Hub success banner detected.; printify_external_detached</t>
+        </is>
       </c>
       <c r="AD155" t="inlineStr">
         <is>
@@ -32602,6 +32610,134 @@
       </c>
       <c r="V295" s="1" t="n">
         <v>46149.71949134259</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0081-FIX1</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0081-FIX1</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>Grimdark</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>Acrylic</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>Smoky Jade Desk Object Plague Doctor Raven Skull Alchemy 5x7 Acrylic Photo Gift</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>&lt;h2&gt;Smoky Jade Desk Object Plague Doctor Raven Skull Alchemy 5x7 Acrylic Photo Gift&lt;/h2&gt;&lt;p&gt;A Quiet Jade collection piece built for desks, bookshelves, altar corners, office focus spaces, and collector displays. The visual direction leans into smoky jade tones, quiet luxury decor language, kintsugi detail, and deep-work atmosphere instead of generic mass-market wall art.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 5x7 vertical acrylic photo block.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; Acrylic block display with depth, gloss, and light-reflective finish.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Grimdark collector aesthetic; smoky jade, wabi-sabi, scholar-room mood.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Best For:&lt;/strong&gt; apartment decor, reading nook styling, focused workspaces, collectors, and giftable room accents.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the physical product customers receive. Additional gallery images are concept, detail, or collection-reference views and are not extra products or selectable variations.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Search Themes:&lt;/strong&gt; Plague Doctor Raven Skull Alchemy, Smoky Jade, Quiet Luxury Decor, Deep Work Visuals, Reading Nook Decor, Wabi Sabi Decor, Scholar Room, Apartment Decor, Jade Art, Kintsugi Aesthetic, Collector Gift, Gothic Study Decor, Alchemy Decor&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Acrylic-Grimdark-0081; Subject: Plague Doctor Raven Skull Alchemy&lt;/small&gt;&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>$89.99</t>
+        </is>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>Plague doctor raven skull, elongated brass beak apparatus, corroded iron rivets, kintsugi gold veins sealing bone fractures, toxic amber bioluminescent vapor seeping from eye sockets, grimdark industrial aesthetic, aged bone, corroded iron, oxidized brass, kintsugi gold, toxic amber bioluminescence, micro-engraved surface relief, handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments, intentional negative space, cinematic rim lighting, soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, premium vertical acrylic photo block composition, 3D depth, refractive light, internal glow, ray tracing, gallery collectible art object</t>
+        </is>
+      </c>
+      <c r="I296" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0081_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="J296" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0081_Ready_for_Steaming\Cover_Mockup.png</t>
+        </is>
+      </c>
+      <c r="K296" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0081_Ready_for_Steaming\Gallery_U1.png</t>
+        </is>
+      </c>
+      <c r="L296" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0081_Ready_for_Steaming\Gallery_U2.png</t>
+        </is>
+      </c>
+      <c r="M296" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0081_Ready_for_Steaming\Gallery_U3.png</t>
+        </is>
+      </c>
+      <c r="N296" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0081_Ready_for_Steaming\Gallery_U4.png</t>
+        </is>
+      </c>
+      <c r="O296" t="inlineStr">
+        <is>
+          <t>Printify_Published_Mockups4</t>
+        </is>
+      </c>
+      <c r="P296" t="inlineStr">
+        <is>
+          <t>2026-05-07 17:23:44 -0400</t>
+        </is>
+      </c>
+      <c r="Q296" t="inlineStr">
+        <is>
+          <t>69fd02f3d70cf705c50f4d27</t>
+        </is>
+      </c>
+      <c r="R296" s="1" t="n">
+        <v>46149.72578068287</v>
+      </c>
+      <c r="S296" t="inlineStr">
+        <is>
+          <t>406911568594</t>
+        </is>
+      </c>
+      <c r="T296" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406911568594</t>
+        </is>
+      </c>
+      <c r="U296" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V296" s="1" t="n">
+        <v>46149.72608443287</v>
+      </c>
+      <c r="AD296" t="inlineStr">
+        <is>
+          <t>2026-05-07 00:46:18 -0400</t>
+        </is>
+      </c>
+      <c r="AE296" t="inlineStr">
+        <is>
+          <t>Operation Quiet Jade</t>
+        </is>
+      </c>
+      <c r="AF296" t="inlineStr">
+        <is>
+          <t>Plague Doctor Raven Skull Alchemy, Smoky Jade, Quiet Luxury Decor, Deep Work Visuals, Reading Nook Decor, Wabi Sabi Decor, Scholar Room, Apartment Decor, Jade Art, Kintsugi Aesthetic, Collector Gift, Gothic Study Decor, Alchemy Decor</t>
+        </is>
+      </c>
+      <c r="AG296" t="inlineStr">
+        <is>
+          <t>Acrylic kept premium; $29.99-$34.99 would violate cost+shipping guardrail.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Close acrylic cover replacement 0001
</commit_message>
<xml_diff>
--- a/Database/eBay_listing.xlsx
+++ b/Database/eBay_listing.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN296"/>
+  <dimension ref="A1:AN297"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14992,7 +14992,7 @@
         <v>46148.85789751157</v>
       </c>
       <c r="W155" s="1" t="n">
-        <v>46149.72674940436</v>
+        <v>46149.72674940973</v>
       </c>
       <c r="X155" t="inlineStr">
         <is>
@@ -15098,7 +15098,7 @@
       </c>
       <c r="O156" t="inlineStr">
         <is>
-          <t>Printify_PrimaryFix_Needed</t>
+          <t>Retired_Replaced</t>
         </is>
       </c>
       <c r="P156" t="inlineStr">
@@ -15128,6 +15128,14 @@
       </c>
       <c r="V156" s="1" t="n">
         <v>46148.85791638889</v>
+      </c>
+      <c r="W156" s="1" t="n">
+        <v>46149.73156060472</v>
+      </c>
+      <c r="X156" t="inlineStr">
+        <is>
+          <t>ENDED_CONFIRMED_SELLER_HUB; Seller Hub success banner detected.; printify_external_detached</t>
+        </is>
       </c>
       <c r="AD156" t="inlineStr">
         <is>
@@ -32735,6 +32743,134 @@
         </is>
       </c>
       <c r="AG296" t="inlineStr">
+        <is>
+          <t>Acrylic kept premium; $29.99-$34.99 would violate cost+shipping guardrail.</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>Acrylic-Zen-0001-FIX1</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>Acrylic-Zen-0001-FIX1</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>Zen</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>Acrylic</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>Smoky Jade Desk Object Mechanical Crane Calm Origami Sculpture 5x7 Acrylic Gift</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>&lt;h2&gt;Smoky Jade Desk Object Mechanical Crane Calm Origami Sculpture 5x7 Acrylic Gift&lt;/h2&gt;&lt;p&gt;A Quiet Jade collection piece built for desks, bookshelves, altar corners, office focus spaces, and collector displays. The visual direction leans into smoky jade tones, quiet luxury decor language, kintsugi detail, and deep-work atmosphere instead of generic mass-market wall art.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 5x7 vertical acrylic photo block.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; Acrylic block display with depth, gloss, and light-reflective finish.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Zen collector aesthetic; smoky jade, wabi-sabi, scholar-room mood.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Best For:&lt;/strong&gt; apartment decor, reading nook styling, focused workspaces, collectors, and giftable room accents.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the physical product customers receive. Additional gallery images are concept, detail, or collection-reference views and are not extra products or selectable variations.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Search Themes:&lt;/strong&gt; Mechanical Crane Calm Origami Sculpture, Smoky Jade, Quiet Luxury Decor, Deep Work Visuals, Reading Nook Decor, Wabi Sabi Decor, Scholar Room, Apartment Decor, Jade Art, Kintsugi Aesthetic, Collector Gift, Meditation Decor, Calm Desk Art&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Acrylic-Zen-0001; Subject: Mechanical Crane Calm Origami Sculpture&lt;/small&gt;&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>$89.99</t>
+        </is>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>Mechanical crane, origami sculpture, moonstone wings, jade clockwork, aquamarine crystals, zen cyberpunk, bioluminescent art, floating fragments, celestial mist, translucent depth, museum grade lighting</t>
+        </is>
+      </c>
+      <c r="I297" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Zen-0001_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="J297" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Zen-0001_Ready_for_Steaming\Cover_Mockup.png</t>
+        </is>
+      </c>
+      <c r="K297" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Zen-0001_Ready_for_Steaming\Gallery_U1.png</t>
+        </is>
+      </c>
+      <c r="L297" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Zen-0001_Ready_for_Steaming\Gallery_U2.png</t>
+        </is>
+      </c>
+      <c r="M297" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Zen-0001_Ready_for_Steaming\Gallery_U3.png</t>
+        </is>
+      </c>
+      <c r="N297" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Zen-0001_Ready_for_Steaming\Gallery_U4.png</t>
+        </is>
+      </c>
+      <c r="O297" t="inlineStr">
+        <is>
+          <t>Printify_Published_Mockups4</t>
+        </is>
+      </c>
+      <c r="P297" t="inlineStr">
+        <is>
+          <t>2026-05-07 17:28:27 -0400</t>
+        </is>
+      </c>
+      <c r="Q297" t="inlineStr">
+        <is>
+          <t>69fd040f6873b551670941bd</t>
+        </is>
+      </c>
+      <c r="R297" s="1" t="n">
+        <v>46149.73057622685</v>
+      </c>
+      <c r="S297" t="inlineStr">
+        <is>
+          <t>406911574121</t>
+        </is>
+      </c>
+      <c r="T297" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406911574121</t>
+        </is>
+      </c>
+      <c r="U297" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V297" s="1" t="n">
+        <v>46149.73087425926</v>
+      </c>
+      <c r="AD297" t="inlineStr">
+        <is>
+          <t>2026-05-07 00:46:18 -0400</t>
+        </is>
+      </c>
+      <c r="AE297" t="inlineStr">
+        <is>
+          <t>Operation Quiet Jade</t>
+        </is>
+      </c>
+      <c r="AF297" t="inlineStr">
+        <is>
+          <t>Mechanical Crane Calm Origami Sculpture, Smoky Jade, Quiet Luxury Decor, Deep Work Visuals, Reading Nook Decor, Wabi Sabi Decor, Scholar Room, Apartment Decor, Jade Art, Kintsugi Aesthetic, Collector Gift, Meditation Decor, Calm Desk Art</t>
+        </is>
+      </c>
+      <c r="AG297" t="inlineStr">
         <is>
           <t>Acrylic kept premium; $29.99-$34.99 would violate cost+shipping guardrail.</t>
         </is>

</xml_diff>

<commit_message>
Close poster cover replacement 0001
</commit_message>
<xml_diff>
--- a/Database/eBay_listing.xlsx
+++ b/Database/eBay_listing.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN297"/>
+  <dimension ref="A1:AN298"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14490,7 +14490,7 @@
       </c>
       <c r="O151" t="inlineStr">
         <is>
-          <t>Printify_PrimaryFix_Needed</t>
+          <t>Retired_Replaced</t>
         </is>
       </c>
       <c r="P151" t="inlineStr">
@@ -14520,6 +14520,14 @@
       </c>
       <c r="V151" s="1" t="n">
         <v>46148.85780189815</v>
+      </c>
+      <c r="W151" s="1" t="n">
+        <v>46149.74256543438</v>
+      </c>
+      <c r="X151" t="inlineStr">
+        <is>
+          <t>ENDED_CONFIRMED_SELLER_HUB; Seller Hub success banner detected.; printify_external_detached</t>
+        </is>
       </c>
     </row>
     <row r="152">
@@ -15130,7 +15138,7 @@
         <v>46148.85791638889</v>
       </c>
       <c r="W156" s="1" t="n">
-        <v>46149.73156060472</v>
+        <v>46149.73156060185</v>
       </c>
       <c r="X156" t="inlineStr">
         <is>
@@ -32874,6 +32882,133 @@
         <is>
           <t>Acrylic kept premium; $29.99-$34.99 would violate cost+shipping guardrail.</t>
         </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0001-FIX1</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0001-FIX1</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>Academia</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>Poster</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>Celestial Gateway Dark Academia Poster 12x18 Study Decor Moonstone Architecture</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Step into the Astral Archive with this mentor-grade poster, a celestial gateway of moonstone and imperial jade rising before a floating library of ancient manuscripts. This 12x18 print captures the essence of dark academia, blending brass clockwork, ink-wash cosmos clouds, and bioluminescent glow for a timeless study companion.&lt;/p&gt;&lt;p&gt;Perfect for adorning your study desk, library wall, or reading nook, this poster transforms any space into a portal of temporal wisdom. The ultra-detailed moonstone crystalline texture and burnished brass accents evoke a vintage intellectual mood, ideal for book lovers and students seeking minimalist elegance.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 12x18 poster, ready to frame&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; Premium matte paper, archival quality&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Size:&lt;/strong&gt; 12 inches by 18 inches&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Academia Mentor-Grade, dark academia aesthetic&lt;/li&gt;&lt;li&gt;&lt;strong&gt;DNA Profile:&lt;/strong&gt; Celestial gateway, moonstone architecture, imperial jade portal, floating library, ancient manuscripts, brass clockwork, mystical knowledge, temporal wisdom, ethereal lighting, bioluminescent glow&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Use Cases:&lt;/strong&gt; Study room decor, library wall art, gift for scholars, vintage intellectual display&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the actual product customers receive. Additional images are bonus concept/detail reference images and do not represent extra products or selectable variations.&lt;/p&gt;&lt;p&gt;&lt;em&gt;Image Note: &lt;/em&gt;&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>$34.99</t>
+        </is>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>Celestial gateway, moonstone architecture, imperial jade portal, floating library, ancient manuscripts, brass clockwork, mystical knowledge, temporal wisdom, ethereal lighting, bioluminescent glow</t>
+        </is>
+      </c>
+      <c r="I298" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0001_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="J298" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0001_Ready_for_Steaming\Cover_Mockup.png</t>
+        </is>
+      </c>
+      <c r="K298" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0001_Ready_for_Steaming\Gallery_U1.png</t>
+        </is>
+      </c>
+      <c r="L298" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0001_Ready_for_Steaming\Gallery_U2.png</t>
+        </is>
+      </c>
+      <c r="M298" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0001_Ready_for_Steaming\Gallery_U3.png</t>
+        </is>
+      </c>
+      <c r="N298" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0001_Ready_for_Steaming\Gallery_U4.png</t>
+        </is>
+      </c>
+      <c r="O298" t="inlineStr">
+        <is>
+          <t>Printify_Published</t>
+        </is>
+      </c>
+      <c r="P298" t="inlineStr">
+        <is>
+          <t>2026-05-07 17:36:44 -0400</t>
+        </is>
+      </c>
+      <c r="Q298" t="inlineStr">
+        <is>
+          <t>69fd05fcd70cf705c50f4ef9</t>
+        </is>
+      </c>
+      <c r="R298" s="1" t="n">
+        <v>46149.74042334491</v>
+      </c>
+      <c r="S298" t="inlineStr">
+        <is>
+          <t>406911589289</t>
+        </is>
+      </c>
+      <c r="T298" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406911589289</t>
+        </is>
+      </c>
+      <c r="U298" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V298" s="1" t="n">
+        <v>46149.7418525463</v>
+      </c>
+      <c r="Y298" s="1" t="n">
+        <v>46149.7418525463</v>
+      </c>
+      <c r="Z298" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA298" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB298" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406911589289 handle=https://www.ebay.com/itm/406911589289</t>
+        </is>
+      </c>
+      <c r="AC298" s="1" t="n">
+        <v>46149.7418525463</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Close poster cover replacement 0003
</commit_message>
<xml_diff>
--- a/Database/eBay_listing.xlsx
+++ b/Database/eBay_listing.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN298"/>
+  <dimension ref="A1:AN299"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14522,7 +14522,7 @@
         <v>46148.85780189815</v>
       </c>
       <c r="W151" s="1" t="n">
-        <v>46149.74256543438</v>
+        <v>46149.74256543982</v>
       </c>
       <c r="X151" t="inlineStr">
         <is>
@@ -14733,7 +14733,7 @@
       </c>
       <c r="O153" t="inlineStr">
         <is>
-          <t>Printify_PrimaryFix_Needed</t>
+          <t>Retired_Replaced</t>
         </is>
       </c>
       <c r="P153" t="inlineStr">
@@ -14763,6 +14763,14 @@
       </c>
       <c r="V153" s="1" t="n">
         <v>46148.8578553125</v>
+      </c>
+      <c r="W153" s="1" t="n">
+        <v>46149.74747569766</v>
+      </c>
+      <c r="X153" t="inlineStr">
+        <is>
+          <t>ENDED_CONFIRMED_SELLER_HUB; Seller Hub success banner detected.; printify_external_detached</t>
+        </is>
       </c>
       <c r="AD153" t="inlineStr">
         <is>
@@ -33009,6 +33017,153 @@
       </c>
       <c r="AC298" s="1" t="n">
         <v>46149.7418525463</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0003-FIX1</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0003-FIX1</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>Academia</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>Poster</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>Reading Nook Wall Decor Serpentine Portal of Alchemical Texts 12x18 Matte Gift</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>&lt;h2&gt;Reading Nook Wall Decor Serpentine Portal of Alchemical Texts 12x18 Matte Gift&lt;/h2&gt;&lt;p&gt;A Quiet Jade collection piece built for quiet apartments, reading nooks, deep-work offices, study rooms, and gallery walls. The visual direction leans into smoky jade tones, quiet luxury decor language, kintsugi detail, and deep-work atmosphere instead of generic mass-market wall art.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 12x18 premium matte vertical poster.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; Premium matte paper wall art produced on demand through Printify.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Academia collector aesthetic; smoky jade, wabi-sabi, scholar-room mood.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Best For:&lt;/strong&gt; apartment decor, reading nook styling, focused workspaces, collectors, and giftable room accents.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the physical product customers receive. Additional gallery images are concept, detail, or collection-reference views and are not extra products or selectable variations.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Search Themes:&lt;/strong&gt; Serpentine Portal of Alchemical Texts, Smoky Jade, Quiet Luxury Decor, Deep Work Visuals, Reading Nook Decor, Wabi Sabi Decor, Scholar Room, Apartment Decor, Jade Art, Kintsugi Aesthetic, Collector Gift, Dark Study Decor, Library Wall Art&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Poster-Academia-0003; Subject: Serpentine Portal of Alchemical Texts&lt;/small&gt;&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>$34.99</t>
+        </is>
+      </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>A serpentine gateway crafted from iridescent moonstone and imperial jade standing before a levitating archive chamber, ancient leather volumes cascading through the portal vortex, nebulous ink-wash clouds merging with aged paper dust, floating brass talisman pieces with engraved hermetic symbols, cinematic chiaroscuro lighting with jade phosphorescence, dark academia aesthetic, ultra-detailed moonstone iridescence and brass gear mechanisms, hyper-detailed mentor-grade artifact design, primary material system: Moonstone, Imperial Jade, Ancient Calfskin, Burnished Brass, Ink-wash Nebula, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, full frame, cinematic lighting, edge-to-edge composition, immersive environment, --ar 9:16 --v 6.1 --style raw --no skin, person, text, watermark</t>
+        </is>
+      </c>
+      <c r="I299" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0003_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="J299" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0003_Ready_for_Steaming\Cover_Mockup.png</t>
+        </is>
+      </c>
+      <c r="K299" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0003_Ready_for_Steaming\Gallery_U1.png</t>
+        </is>
+      </c>
+      <c r="L299" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0003_Ready_for_Steaming\Gallery_U2.png</t>
+        </is>
+      </c>
+      <c r="M299" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0003_Ready_for_Steaming\Gallery_U3.png</t>
+        </is>
+      </c>
+      <c r="N299" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0003_Ready_for_Steaming\Gallery_U4.png</t>
+        </is>
+      </c>
+      <c r="O299" t="inlineStr">
+        <is>
+          <t>Printify_Published</t>
+        </is>
+      </c>
+      <c r="P299" t="inlineStr">
+        <is>
+          <t>2026-05-07 17:51:09 -0400</t>
+        </is>
+      </c>
+      <c r="Q299" t="inlineStr">
+        <is>
+          <t>69fd095c9f77031382026de2</t>
+        </is>
+      </c>
+      <c r="R299" s="1" t="n">
+        <v>46149.74574953704</v>
+      </c>
+      <c r="S299" t="inlineStr">
+        <is>
+          <t>406911598735</t>
+        </is>
+      </c>
+      <c r="T299" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406911598735</t>
+        </is>
+      </c>
+      <c r="U299" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V299" s="1" t="n">
+        <v>46149.74666180556</v>
+      </c>
+      <c r="Y299" s="1" t="n">
+        <v>46149.74666180556</v>
+      </c>
+      <c r="Z299" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA299" t="inlineStr">
+        <is>
+          <t>FORCE_ASSOCIATE</t>
+        </is>
+      </c>
+      <c r="AB299" t="inlineStr">
+        <is>
+          <t>Printify product external.id=406911598735 handle=https://www.ebay.com/itm/406911598735</t>
+        </is>
+      </c>
+      <c r="AC299" s="1" t="n">
+        <v>46149.74666180556</v>
+      </c>
+      <c r="AD299" t="inlineStr">
+        <is>
+          <t>2026-05-07 00:46:18 -0400</t>
+        </is>
+      </c>
+      <c r="AE299" t="inlineStr">
+        <is>
+          <t>Operation Quiet Jade</t>
+        </is>
+      </c>
+      <c r="AF299" t="inlineStr">
+        <is>
+          <t>Serpentine Portal of Alchemical Texts, Smoky Jade, Quiet Luxury Decor, Deep Work Visuals, Reading Nook Decor, Wabi Sabi Decor, Scholar Room, Apartment Decor, Jade Art, Kintsugi Aesthetic, Collector Gift, Dark Study Decor, Library Wall Art</t>
+        </is>
+      </c>
+      <c r="AG299" t="inlineStr">
+        <is>
+          <t>Poster value-pivot target $34.99; above cost+shipping+fees guardrail.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Tighten sticker publish gallery gate
</commit_message>
<xml_diff>
--- a/Database/eBay_listing.xlsx
+++ b/Database/eBay_listing.xlsx
@@ -7909,7 +7909,7 @@
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>Printify_UI_Mockups5</t>
+          <t>Printify_Published_Mockups5</t>
         </is>
       </c>
       <c r="P73" t="inlineStr">
@@ -7921,6 +7921,27 @@
         <is>
           <t>69f26281feceb0d66c042ce7</t>
         </is>
+      </c>
+      <c r="R73" s="1" t="n">
+        <v>46149.90896847222</v>
+      </c>
+      <c r="S73" t="inlineStr">
+        <is>
+          <t>406911942577</t>
+        </is>
+      </c>
+      <c r="T73" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406911942577</t>
+        </is>
+      </c>
+      <c r="U73" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V73" s="1" t="n">
+        <v>46149.90897497685</v>
       </c>
       <c r="AH73" t="inlineStr">
         <is>
@@ -8011,7 +8032,7 @@
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>Printify_UI_Mockups5</t>
+          <t>Printify_Published_Mockups5</t>
         </is>
       </c>
       <c r="P74" t="inlineStr">
@@ -8023,6 +8044,27 @@
         <is>
           <t>69f262db5269e3325904b893</t>
         </is>
+      </c>
+      <c r="R74" s="1" t="n">
+        <v>46149.91137163734</v>
+      </c>
+      <c r="S74" t="inlineStr">
+        <is>
+          <t>406911955913</t>
+        </is>
+      </c>
+      <c r="T74" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406911955913</t>
+        </is>
+      </c>
+      <c r="U74" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V74" s="1" t="n">
+        <v>46149.91138125821</v>
       </c>
       <c r="AH74" t="inlineStr">
         <is>
@@ -8113,7 +8155,7 @@
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>Printify_UI_Mockups5</t>
+          <t>Printify_Published_Mockups5</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
@@ -8125,6 +8167,27 @@
         <is>
           <t>69f263729b469f716d0e7409</t>
         </is>
+      </c>
+      <c r="R75" s="1" t="n">
+        <v>46149.91389873351</v>
+      </c>
+      <c r="S75" t="inlineStr">
+        <is>
+          <t>406911953636</t>
+        </is>
+      </c>
+      <c r="T75" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406911953636</t>
+        </is>
+      </c>
+      <c r="U75" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V75" s="1" t="n">
+        <v>46149.91390609904</v>
       </c>
       <c r="AH75" t="inlineStr">
         <is>
@@ -33274,7 +33337,7 @@
         <v>46149.88308030093</v>
       </c>
       <c r="W300" s="1" t="n">
-        <v>46149.90281554782</v>
+        <v>46149.90281554398</v>
       </c>
       <c r="X300" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Prototype sticker mixed gallery guard
</commit_message>
<xml_diff>
--- a/Database/eBay_listing.xlsx
+++ b/Database/eBay_listing.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN300"/>
+  <dimension ref="A1:AO300"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -620,6 +620,11 @@
           <t>Multi_Track_Mockup_Mood</t>
         </is>
       </c>
+      <c r="AO1" t="inlineStr">
+        <is>
+          <t>QA_Note</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -8046,7 +8051,7 @@
         </is>
       </c>
       <c r="R74" s="1" t="n">
-        <v>46149.91137163734</v>
+        <v>46149.91137163195</v>
       </c>
       <c r="S74" t="inlineStr">
         <is>
@@ -8064,7 +8069,7 @@
         </is>
       </c>
       <c r="V74" s="1" t="n">
-        <v>46149.91138125821</v>
+        <v>46149.91138126158</v>
       </c>
       <c r="AH74" t="inlineStr">
         <is>
@@ -8169,7 +8174,7 @@
         </is>
       </c>
       <c r="R75" s="1" t="n">
-        <v>46149.91389873351</v>
+        <v>46149.91389873843</v>
       </c>
       <c r="S75" t="inlineStr">
         <is>
@@ -8187,7 +8192,7 @@
         </is>
       </c>
       <c r="V75" s="1" t="n">
-        <v>46149.91390609904</v>
+        <v>46149.91390609954</v>
       </c>
       <c r="AH75" t="inlineStr">
         <is>
@@ -8278,13 +8283,11 @@
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>Printify_UI_Mockups5</t>
-        </is>
-      </c>
-      <c r="P76" t="inlineStr">
-        <is>
-          <t>4/29/2026  1:28:54 PM</t>
-        </is>
+          <t>Printify_StickerMixedGallery_Hold</t>
+        </is>
+      </c>
+      <c r="P76" s="1" t="n">
+        <v>46149.94308292386</v>
       </c>
       <c r="Q76" t="inlineStr">
         <is>
@@ -8304,6 +8307,11 @@
       <c r="AJ76" t="inlineStr">
         <is>
           <t>B_BOOK_NOOK_LAPTOP_DECALS</t>
+        </is>
+      </c>
+      <c r="AO76" t="inlineStr">
+        <is>
+          <t>Cover-only mixed gallery probe failed API verification: Printify still selected 5 custom gallery images, no official mockups. Do not publish until mixed Cover + official mockup path is fixed.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Verify sticker mixed cover gallery path
</commit_message>
<xml_diff>
--- a/Database/eBay_listing.xlsx
+++ b/Database/eBay_listing.xlsx
@@ -8283,17 +8283,38 @@
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>Printify_StickerMixedGallery_Hold</t>
+          <t>Printify_Published_Mockups4</t>
         </is>
       </c>
       <c r="P76" s="1" t="n">
-        <v>46149.94308292386</v>
+        <v>46149.9474558912</v>
       </c>
       <c r="Q76" t="inlineStr">
         <is>
           <t>69f26426671cc7c7960b3f3d</t>
         </is>
       </c>
+      <c r="R76" s="1" t="n">
+        <v>46149.94883718868</v>
+      </c>
+      <c r="S76" t="inlineStr">
+        <is>
+          <t>406912077790</t>
+        </is>
+      </c>
+      <c r="T76" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406912077790</t>
+        </is>
+      </c>
+      <c r="U76" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V76" s="1" t="n">
+        <v>46149.94917833775</v>
+      </c>
       <c r="AH76" t="inlineStr">
         <is>
           <t>SEO_STRIKE_SYNCED_PRINTIFY_DRAFT</t>
@@ -8311,7 +8332,7 @@
       </c>
       <c r="AO76" t="inlineStr">
         <is>
-          <t>Cover-only mixed gallery probe failed API verification: Printify still selected 5 custom gallery images, no official mockups. Do not publish until mixed Cover + official mockup path is fixed.</t>
+          <t>Sticker mixed gallery verified by Printify API: 3 official mockups + 1 custom cover, selected=4, unique=4. Publish only after dry-run and post-publish live gallery audit.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add hash-verified sticker cover selection
</commit_message>
<xml_diff>
--- a/Database/eBay_listing.xlsx
+++ b/Database/eBay_listing.xlsx
@@ -8295,7 +8295,7 @@
         </is>
       </c>
       <c r="R76" s="1" t="n">
-        <v>46149.94883718868</v>
+        <v>46149.9488371875</v>
       </c>
       <c r="S76" t="inlineStr">
         <is>
@@ -8313,7 +8313,7 @@
         </is>
       </c>
       <c r="V76" s="1" t="n">
-        <v>46149.94917833775</v>
+        <v>46149.94917833334</v>
       </c>
       <c r="AH76" t="inlineStr">
         <is>
@@ -8409,13 +8409,11 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>Printify_UI_Mockups5</t>
-        </is>
-      </c>
-      <c r="P77" t="inlineStr">
-        <is>
-          <t>4/29/2026  1:28:54 PM</t>
-        </is>
+          <t>Printify_StickerMixedGallery_Hold</t>
+        </is>
+      </c>
+      <c r="P77" s="1" t="n">
+        <v>46149.95420189814</v>
       </c>
       <c r="Q77" t="inlineStr">
         <is>
@@ -8435,6 +8433,11 @@
       <c r="AJ77" t="inlineStr">
         <is>
           <t>A_DEEP_WORK_STICKER_SET</t>
+        </is>
+      </c>
+      <c r="AO77" t="inlineStr">
+        <is>
+          <t>Mixed gallery selector over-selected custom images: API showed 3 official + 4 custom. Publish scheduler blocked. Retry only after selector is hardened.</t>
         </is>
       </c>
     </row>
@@ -8757,7 +8760,7 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>Printify_UI_Mockups5</t>
+          <t>Retired_Replaced</t>
         </is>
       </c>
       <c r="P81" t="inlineStr">
@@ -8768,6 +8771,35 @@
       <c r="Q81" t="inlineStr">
         <is>
           <t>69f26782c326d7da170c1498</t>
+        </is>
+      </c>
+      <c r="R81" s="1" t="n">
+        <v>46149.95453435185</v>
+      </c>
+      <c r="S81" t="inlineStr">
+        <is>
+          <t>406912094146</t>
+        </is>
+      </c>
+      <c r="T81" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406912094146</t>
+        </is>
+      </c>
+      <c r="U81" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="V81" s="1" t="n">
+        <v>46149.95484488426</v>
+      </c>
+      <c r="W81" s="1" t="n">
+        <v>46149.95751690179</v>
+      </c>
+      <c r="X81" t="inlineStr">
+        <is>
+          <t>ENDED_CONFIRMED_SELLER_HUB; Seller Hub success banner detected.; printify_external_detached</t>
         </is>
       </c>
       <c r="AH81" t="inlineStr">

</xml_diff>

<commit_message>
Advance eBay traffic experiments and gallery risk reporting
</commit_message>
<xml_diff>
--- a/Database/eBay_listing.xlsx
+++ b/Database/eBay_listing.xlsx
@@ -2805,7 +2805,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
@@ -7914,7 +7914,7 @@
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="P73" t="inlineStr">
@@ -8037,7 +8037,7 @@
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="P74" t="inlineStr">
@@ -8160,7 +8160,7 @@
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
@@ -8283,7 +8283,7 @@
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups4</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="P76" s="1" t="n">
@@ -8981,8 +8981,6 @@
           <t>5/7/2026  11:50:52 PM</t>
         </is>
       </c>
-      <c r="Q83" t="inlineStr"/>
-      <c r="S83" t="inlineStr"/>
       <c r="AH83" t="inlineStr">
         <is>
           <t>SEO_STRIKE_SYNCED_PRINTIFY_DRAFT</t>
@@ -9072,7 +9070,7 @@
       </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t>Printify_UI_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="P84" t="inlineStr">
@@ -9241,7 +9239,7 @@
       </c>
       <c r="O86" t="inlineStr">
         <is>
-          <t>Printify_UI_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="P86" t="inlineStr">
@@ -9328,7 +9326,7 @@
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>Printify_UI_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="P87" t="inlineStr">
@@ -9415,7 +9413,7 @@
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t>Printify_UI_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="P88" t="inlineStr">
@@ -9502,7 +9500,7 @@
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>Printify_UI_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="P89" t="inlineStr">
@@ -9671,7 +9669,7 @@
       </c>
       <c r="O91" t="inlineStr">
         <is>
-          <t>Printify_UI_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="P91" t="inlineStr">
@@ -9758,7 +9756,7 @@
       </c>
       <c r="O92" t="inlineStr">
         <is>
-          <t>Printify_UI_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="P92" t="inlineStr">
@@ -9845,7 +9843,7 @@
       </c>
       <c r="O93" t="inlineStr">
         <is>
-          <t>Printify_UI_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="P93" t="inlineStr">
@@ -9932,7 +9930,7 @@
       </c>
       <c r="O94" t="inlineStr">
         <is>
-          <t>Printify_UI_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="P94" t="inlineStr">
@@ -14724,7 +14722,7 @@
       </c>
       <c r="O152" t="inlineStr">
         <is>
-          <t>Printify_Published_Mockups5</t>
+          <t>Printify_PrimaryFix_Needed</t>
         </is>
       </c>
       <c r="P152" t="inlineStr">
@@ -16053,12 +16051,12 @@
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>Deep Work Desk Visual Pagoda Fragment Relic Print Floating 5x7 Acrylic Photo</t>
+          <t>Meditation Room Jade Relic Deep Work Visual Pagoda 5x7 Acrylic Block Shelf Gift</t>
         </is>
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>&lt;h2&gt;Deep Work Desk Visual Pagoda Fragment Relic Print Floating 5x7 Acrylic Photo&lt;/h2&gt;&lt;p&gt;A Quiet Jade collection piece built for desks, bookshelves, altar corners, office focus spaces, and collector displays. The visual direction leans into smoky jade tones, quiet luxury decor language, kintsugi detail, and deep-work atmosphere instead of generic mass-market wall art.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 5x7 vertical acrylic photo block.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; Acrylic block display with depth, gloss, and light-reflective finish.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Zen collector aesthetic; smoky jade, wabi-sabi, scholar-room mood.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Best For:&lt;/strong&gt; apartment decor, reading nook styling, focused workspaces, collectors, and giftable room accents.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the physical product customers receive. Additional gallery images are concept, detail, or collection-reference views and are not extra products or selectable variations.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Search Themes:&lt;/strong&gt; Pagoda Fragment Relic Print Floating, Smoky Jade, Quiet Luxury Decor, Deep Work Visuals, Reading Nook Decor, Wabi Sabi Decor, Scholar Room, Apartment Decor, Jade Art, Kintsugi Aesthetic, Collector Gift, Meditation Decor, Calm Desk Art&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Acrylic-Zen-0003; Subject: Pagoda Fragment Relic Print Floating&lt;/small&gt;&lt;/p&gt;</t>
+          <t>&lt;h2&gt;Meditation Room Jade Relic Deep Work Visual Pagoda 5x7 Acrylic Block Shelf Gift&lt;/h2&gt;&lt;p&gt;This listing is part of a focused search-intent experiment for reading nook decor. It is written for buyers decorating quiet shelves, meditation corners, gothic study desks, collector rooms, and deep-work apartments, not for generic wall-art browsing.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 5x7 vertical acrylic photo block, produced on demand through Printify.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Visual Mood:&lt;/strong&gt; Reading Nook Warm Lamp.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Design Language:&lt;/strong&gt; refractive depth, smoky jade color, internal glow, and premium desk-object presence.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Search Lane:&lt;/strong&gt; reading nook decor, meditation room wall art, tea room accent, quiet corner decor, dorm desk calm art, deep work visual.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; This is a single printed acrylic display block. The main artwork is the product customers receive; any additional gallery images are concept/detail references.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Acrylic-Zen-0003. Prior title: Deep Work Desk Visual Pagoda Fragment Relic Print Floating 5x7 Acrylic Photo&lt;/small&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="G163" t="inlineStr">
@@ -16156,7 +16154,27 @@
       </c>
       <c r="AH163" t="inlineStr">
         <is>
-          <t>QUIET_JADE_SYNCED_PRINTIFY_PUBLISH</t>
+          <t>MULTI_TRACK_SYNCED_PRINTIFY_PUBLISH</t>
+        </is>
+      </c>
+      <c r="AK163" t="inlineStr">
+        <is>
+          <t>2026-05-08 08:17:21 -0400</t>
+        </is>
+      </c>
+      <c r="AL163" t="inlineStr">
+        <is>
+          <t>A_LOW_COMPETITION_NICHE</t>
+        </is>
+      </c>
+      <c r="AM163" t="inlineStr">
+        <is>
+          <t>reading nook decor</t>
+        </is>
+      </c>
+      <c r="AN163" t="inlineStr">
+        <is>
+          <t>reading_nook_warm_lamp</t>
         </is>
       </c>
     </row>
@@ -16783,12 +16801,12 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>Gallery Desk Art Incense Vessel Constellation for Meditation 5x7 Acrylic Photo</t>
+          <t>Meditation Room Jade Relic Incense Vessel Constellation 5x7 Acrylic Block Decor</t>
         </is>
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>&lt;h2&gt;Gallery Desk Art Incense Vessel Constellation for Meditation 5x7 Acrylic Photo&lt;/h2&gt;&lt;p&gt;A Quiet Jade collection piece built for desks, bookshelves, altar corners, office focus spaces, and collector displays. The visual direction leans into smoky jade tones, quiet luxury decor language, kintsugi detail, and deep-work atmosphere instead of generic mass-market wall art.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 5x7 vertical acrylic photo block.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; Acrylic block display with depth, gloss, and light-reflective finish.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Zen collector aesthetic; smoky jade, wabi-sabi, scholar-room mood.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Best For:&lt;/strong&gt; apartment decor, reading nook styling, focused workspaces, collectors, and giftable room accents.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the physical product customers receive. Additional gallery images are concept, detail, or collection-reference views and are not extra products or selectable variations.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Search Themes:&lt;/strong&gt; Incense Vessel Constellation for Meditat, Smoky Jade, Quiet Luxury Decor, Deep Work Visuals, Reading Nook Decor, Wabi Sabi Decor, Scholar Room, Apartment Decor, Jade Art, Kintsugi Aesthetic, Collector Gift, Meditation Decor, Calm Desk Art&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Acrylic-Zen-0005; Subject: Incense Vessel Constellation for Meditation&lt;/small&gt;&lt;/p&gt;</t>
+          <t>&lt;h2&gt;Meditation Room Jade Relic Incense Vessel Constellation 5x7 Acrylic Block Decor&lt;/h2&gt;&lt;p&gt;This listing is part of a focused search-intent experiment for tea room accent. It is written for buyers decorating quiet shelves, meditation corners, gothic study desks, collector rooms, and deep-work apartments, not for generic wall-art browsing.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 5x7 vertical acrylic photo block, produced on demand through Printify.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Visual Mood:&lt;/strong&gt; Reading Nook Warm Lamp.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Design Language:&lt;/strong&gt; refractive depth, smoky jade color, internal glow, and premium desk-object presence.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Search Lane:&lt;/strong&gt; reading nook decor, meditation room wall art, tea room accent, quiet corner decor, dorm desk calm art, deep work visual.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; This is a single printed acrylic display block. The main artwork is the product customers receive; any additional gallery images are concept/detail references.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Acrylic-Zen-0005. Prior title: Gallery Desk Art Incense Vessel Constellation for Meditation 5x7 Acrylic Photo&lt;/small&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="G169" t="inlineStr">
@@ -16886,7 +16904,27 @@
       </c>
       <c r="AH169" t="inlineStr">
         <is>
-          <t>QUIET_JADE_SYNCED_PRINTIFY_PUBLISH</t>
+          <t>MULTI_TRACK_SYNCED_PRINTIFY_PUBLISH</t>
+        </is>
+      </c>
+      <c r="AK169" t="inlineStr">
+        <is>
+          <t>2026-05-08 08:17:21 -0400</t>
+        </is>
+      </c>
+      <c r="AL169" t="inlineStr">
+        <is>
+          <t>A_LOW_COMPETITION_NICHE</t>
+        </is>
+      </c>
+      <c r="AM169" t="inlineStr">
+        <is>
+          <t>tea room accent</t>
+        </is>
+      </c>
+      <c r="AN169" t="inlineStr">
+        <is>
+          <t>reading_nook_warm_lamp</t>
         </is>
       </c>
     </row>
@@ -18485,12 +18523,12 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>Deep Work Desk Visual Lantern Soul Cage Crimson Flame 5x7 Acrylic Photo Block</t>
+          <t>Dark Study Smoky Jade Deep Work Visual Lantern 5x7 Acrylic Block Shelf Decor</t>
         </is>
       </c>
       <c r="F182" t="inlineStr">
         <is>
-          <t>&lt;h2&gt;Deep Work Desk Visual Lantern Soul Cage Crimson Flame 5x7 Acrylic Photo Block&lt;/h2&gt;&lt;p&gt;A Quiet Jade collection piece built for desks, bookshelves, altar corners, office focus spaces, and collector displays. The visual direction leans into smoky jade tones, quiet luxury decor language, kintsugi detail, and deep-work atmosphere instead of generic mass-market wall art.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 5x7 vertical acrylic photo block.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; Acrylic block display with depth, gloss, and light-reflective finish.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Grimdark collector aesthetic; smoky jade, wabi-sabi, scholar-room mood.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Best For:&lt;/strong&gt; apartment decor, reading nook styling, focused workspaces, collectors, and giftable room accents.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the physical product customers receive. Additional gallery images are concept, detail, or collection-reference views and are not extra products or selectable variations.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Search Themes:&lt;/strong&gt; Lantern Soul Cage Crimson Flame, Smoky Jade, Quiet Luxury Decor, Deep Work Visuals, Reading Nook Decor, Wabi Sabi Decor, Scholar Room, Apartment Decor, Jade Art, Kintsugi Aesthetic, Collector Gift, Gothic Study Decor, Alchemy Decor&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Acrylic-Grimdark-0001; Subject: Lantern Soul Cage Crimson Flame&lt;/small&gt;&lt;/p&gt;</t>
+          <t>&lt;h2&gt;Dark Study Smoky Jade Deep Work Visual Lantern 5x7 Acrylic Block Shelf Decor&lt;/h2&gt;&lt;p&gt;This listing is part of a focused search-intent experiment for dark study room decor. It is written for buyers decorating quiet shelves, meditation corners, gothic study desks, collector rooms, and deep-work apartments, not for generic wall-art browsing.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 5x7 vertical acrylic photo block, produced on demand through Printify.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Visual Mood:&lt;/strong&gt; Reading Nook Warm Lamp.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Design Language:&lt;/strong&gt; refractive depth, smoky jade color, internal glow, and premium desk-object presence.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Search Lane:&lt;/strong&gt; gothic shelf decor, moody desk display, occult library art, dark study room decor, collector shelf object, smoky jade relic.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; This is a single printed acrylic display block. The main artwork is the product customers receive; any additional gallery images are concept/detail references.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Acrylic-Grimdark-0001. Prior title: Deep Work Desk Visual Lantern Soul Cage Crimson Flame 5x7 Acrylic Photo Block&lt;/small&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="G182" t="inlineStr">
@@ -18588,7 +18626,27 @@
       </c>
       <c r="AH182" t="inlineStr">
         <is>
-          <t>QUIET_JADE_SYNCED_PRINTIFY_PUBLISH</t>
+          <t>MULTI_TRACK_SYNCED_PRINTIFY_PUBLISH</t>
+        </is>
+      </c>
+      <c r="AK182" t="inlineStr">
+        <is>
+          <t>2026-05-08 08:17:21 -0400</t>
+        </is>
+      </c>
+      <c r="AL182" t="inlineStr">
+        <is>
+          <t>A_LOW_COMPETITION_NICHE</t>
+        </is>
+      </c>
+      <c r="AM182" t="inlineStr">
+        <is>
+          <t>dark study room decor</t>
+        </is>
+      </c>
+      <c r="AN182" t="inlineStr">
+        <is>
+          <t>reading_nook_warm_lamp</t>
         </is>
       </c>
     </row>
@@ -19235,12 +19293,12 @@
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>Gothic Grimdark Lich Phylactery Lantern 5x7 Acrylic Print Dark Fantasy Home</t>
+          <t>Quiet Luxury Jade Relic Lich Phylactery Lantern Fantasy 5x7 Acrylic Block Decor</t>
         </is>
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t>&lt;p&gt;This 5x7 acrylic print captures the haunting beauty of a Lich's Phylactery Lantern, a grimdark artifact forged from wrought iron and ghostly topaz glass. The amber spirit flame swirls within, casting a bioluminescent glow through cracked refractive layers. A premium collectible for dark fantasy enthusiasts, it brings an aura of ancient magic and undead lore to any space.&lt;/p&gt;&lt;p&gt;Display this piece on a study desk, bookshelf, or altar to evoke the mood of a gothic ritual chamber. The high-contrast shadows and bone inlay details reward close inspection, while the museum-grade finish ensures lasting vibrancy. Ideal for fans of grimdark art, necromancer aesthetics, or dark academia decor.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 5x7 acrylic print, ready to hang or stand&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; High-gloss acrylic with UV-resistant ink&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Size:&lt;/strong&gt; 5x7 inches (12.7 x 17.8 cm)&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Grimdark Mentor-Grade, gothic artifact&lt;/li&gt;&lt;li&gt;&lt;strong&gt;DNA Profile:&lt;/strong&gt; Wrought iron, ghostly topaz glass, amber spirit flame, gothic filigree, bone inlay, refractive depth, bioluminescent light, micro-engraved surface relief, handcrafted edge bevels, layered translucent depth, subtle internal glow, kintsugi-like vein logic, floating accent fragments, cinematic rim lighting, soft museum-grade overhead fill&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Use Cases:&lt;/strong&gt; Dark fantasy home decor, gothic study accent, collector display, Halloween ambiance, occult-themed room, gift for grimdark fans&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the actual product customers receive. Additional images are bonus concept/detail reference images and do not represent extra products or selectable variations.&lt;/p&gt;&lt;p&gt;&lt;em&gt;Image Note: &lt;/em&gt;&lt;/p&gt;</t>
+          <t>&lt;h2&gt;Quiet Luxury Jade Relic Lich Phylactery Lantern Fantasy 5x7 Acrylic Block Decor&lt;/h2&gt;&lt;p&gt;This listing is part of a focused search-intent experiment for moody desk display. It is written for buyers decorating quiet shelves, meditation corners, gothic study desks, collector rooms, and deep-work apartments, not for generic wall-art browsing.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 5x7 vertical acrylic photo block, produced on demand through Printify.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Visual Mood:&lt;/strong&gt; Quiet Luxury Apartment.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Design Language:&lt;/strong&gt; refractive depth, smoky jade color, internal glow, and premium desk-object presence.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Search Lane:&lt;/strong&gt; gothic shelf decor, moody desk display, occult library art, dark study room decor, collector shelf object, smoky jade relic.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; This is a single printed acrylic display block. The main artwork is the product customers receive; any additional gallery images are concept/detail references.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Acrylic-Grimdark-0009. Prior title: Gothic Grimdark Lich Phylactery Lantern 5x7 Acrylic Print Dark Fantasy Home&lt;/small&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="G188" t="inlineStr">
@@ -19315,6 +19373,31 @@
       </c>
       <c r="V188" s="1" t="n">
         <v>46148.85851284722</v>
+      </c>
+      <c r="AH188" t="inlineStr">
+        <is>
+          <t>MULTI_TRACK_SYNCED_PRINTIFY_PUBLISH</t>
+        </is>
+      </c>
+      <c r="AK188" t="inlineStr">
+        <is>
+          <t>2026-05-08 08:17:21 -0400</t>
+        </is>
+      </c>
+      <c r="AL188" t="inlineStr">
+        <is>
+          <t>A_LOW_COMPETITION_NICHE</t>
+        </is>
+      </c>
+      <c r="AM188" t="inlineStr">
+        <is>
+          <t>moody desk display</t>
+        </is>
+      </c>
+      <c r="AN188" t="inlineStr">
+        <is>
+          <t>quiet_luxury_apartment</t>
+        </is>
       </c>
     </row>
     <row r="189">
@@ -21337,12 +21420,12 @@
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t>Grimdark Aesthetic Dreadlord Beacon Lantern 5x7 Acrylic Block Dark Decor Shelf</t>
+          <t>Collector Shelf Smoky Jade Dreadlord Beacon Lantern 5x7 Acrylic Block Shelf</t>
         </is>
       </c>
       <c r="F204" t="inlineStr">
         <is>
-          <t>&lt;p&gt;This Dreadlord's Dominion Beacon acrylic block captures a grimdark mentor-grade artifact in miniature form. The ornate wrought-iron lantern with demonic horns encloses a trapped scarlet spirit flame, its light refracting through cracked ghostly garnet glass. A perfect accent for a gothic study, altar shelf, or collector's cabinet.&lt;/p&gt;&lt;p&gt;Display this 5x7 block on a desk, bookshelf, or mantel to evoke a dark fantasy atmosphere. The high-contrast macro photography and cinematic rim lighting bring out the bioluminescent core and refined kintsugi-like vein logic. Use it as a paperweight, a decorative object, or a conversation starter for fans of grimdark lore.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 5x7 acrylic block print&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; Premium clear acrylic with UV-cured print&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Size:&lt;/strong&gt; 5x7 inches (12.7 x 17.8 cm)&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Grimdark Mentor-Grade&lt;/li&gt;&lt;li&gt;&lt;strong&gt;DNA Profile:&lt;/strong&gt; Wrought iron, ghostly garnet glass, scarlet spirit flame, gothic filigree, micro-engraved surface relief, layered translucent depth, internal bioluminescent glow&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Use Cases:&lt;/strong&gt; Gothic decor, dark fantasy collection, study shelf accent, altar display, gift for grimdark enthusiasts&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the actual product customers receive. Additional images are bonus concept/detail reference images and do not represent extra products or selectable variations.&lt;/p&gt;&lt;p&gt;&lt;em&gt;Image Note: &lt;/em&gt;&lt;/p&gt;</t>
+          <t>&lt;h2&gt;Collector Shelf Smoky Jade Dreadlord Beacon Lantern 5x7 Acrylic Block Shelf&lt;/h2&gt;&lt;p&gt;This listing is part of a focused search-intent experiment for gothic shelf decor. It is written for buyers decorating quiet shelves, meditation corners, gothic study desks, collector rooms, and deep-work apartments, not for generic wall-art browsing.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 5x7 vertical acrylic photo block, produced on demand through Printify.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Visual Mood:&lt;/strong&gt; Quiet Luxury Apartment.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Design Language:&lt;/strong&gt; refractive depth, smoky jade color, internal glow, and premium desk-object presence.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Search Lane:&lt;/strong&gt; gothic shelf decor, moody desk display, occult library art, dark study room decor, collector shelf object, smoky jade relic.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; This is a single printed acrylic display block. The main artwork is the product customers receive; any additional gallery images are concept/detail references.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Acrylic-Grimdark-0017. Prior title: Grimdark Aesthetic Dreadlord Beacon Lantern 5x7 Acrylic Block Dark Decor Shelf&lt;/small&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="G204" t="inlineStr">
@@ -21436,6 +21519,31 @@
       </c>
       <c r="AC204" s="1" t="n">
         <v>46149.07898653935</v>
+      </c>
+      <c r="AH204" t="inlineStr">
+        <is>
+          <t>MULTI_TRACK_SYNCED_PRINTIFY_PUBLISH</t>
+        </is>
+      </c>
+      <c r="AK204" t="inlineStr">
+        <is>
+          <t>2026-05-08 08:17:21 -0400</t>
+        </is>
+      </c>
+      <c r="AL204" t="inlineStr">
+        <is>
+          <t>A_LOW_COMPETITION_NICHE</t>
+        </is>
+      </c>
+      <c r="AM204" t="inlineStr">
+        <is>
+          <t>gothic shelf decor</t>
+        </is>
+      </c>
+      <c r="AN204" t="inlineStr">
+        <is>
+          <t>quiet_luxury_apartment</t>
+        </is>
       </c>
     </row>
     <row r="205">
@@ -21858,12 +21966,12 @@
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t>Violet Torment Lantern 5x7 Acrylic Grimdark Gothic Decor for Dark Fantasy Study</t>
+          <t>Dark Study Smoky Jade Violet Torment Lantern Fantasy 5x7 Acrylic Block Shelf</t>
         </is>
       </c>
       <c r="F208" t="inlineStr">
         <is>
-          <t>&lt;p&gt;This 5x7 acrylic print presents the Violet Torment Lantern, a grimdark artifact forged from blackened wrought iron with razor-sharp filigree and a violent violet spirit flame. The amethyst-tinted glass and internal bioluminescent glow create a corrupted, collector-grade aesthetic perfect for dark fantasy enthusiasts.&lt;/p&gt;&lt;p&gt;Ideal for a study desk, bookshelf, or gothic decor collection, this premium acrylic piece captures the translucent depth and oxidized iron details of the original design. The high-gloss surface and crisp silhouette ensure the lantern becomes a focal point in any room, from a minimalist workspace to a vintage-inspired library.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 5x7 acrylic print, ready to display (stand not included)&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; Premium acrylic with high-gloss finish, UV-resistant ink&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Size:&lt;/strong&gt; 5x7 inches (12.7 x 17.8 cm)&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Grimdark Mentor-Grade with violet spirit flame, blackened iron filigree, and layered translucent depth&lt;/li&gt;&lt;li&gt;&lt;strong&gt;DNA Profile:&lt;/strong&gt; Violet flame, amethyst gothic, corrupted spirit vessel, blackened iron filigree, dark fantasy artifact, grimdark collectible, translucent depth, premium lantern design, wrought iron craftsmanship, bioluminescent accent&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Use Cases:&lt;/strong&gt; Dark fantasy study decor, gothic bookshelf accent, collector gift for grimdark fans, vintage intellectual desk piece, minimalist room focal point&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the actual product customers receive. Additional images are bonus concept/detail reference images and do not represent extra products or selectable variations.&lt;/p&gt;&lt;p&gt;&lt;em&gt;Image Note: &lt;/em&gt;&lt;/p&gt;</t>
+          <t>&lt;h2&gt;Dark Study Smoky Jade Violet Torment Lantern Fantasy 5x7 Acrylic Block Shelf&lt;/h2&gt;&lt;p&gt;This listing is part of a focused search-intent experiment for dark study room decor. It is written for buyers decorating quiet shelves, meditation corners, gothic study desks, collector rooms, and deep-work apartments, not for generic wall-art browsing.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 5x7 vertical acrylic photo block, produced on demand through Printify.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Visual Mood:&lt;/strong&gt; Quiet Luxury Apartment.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Design Language:&lt;/strong&gt; refractive depth, smoky jade color, internal glow, and premium desk-object presence.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Search Lane:&lt;/strong&gt; gothic shelf decor, moody desk display, occult library art, dark study room decor, collector shelf object, smoky jade relic.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; This is a single printed acrylic display block. The main artwork is the product customers receive; any additional gallery images are concept/detail references.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Acrylic-Grimdark-0022. Prior title: Violet Torment Lantern 5x7 Acrylic Grimdark Gothic Decor for Dark Fantasy Study&lt;/small&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="G208" t="inlineStr">
@@ -21957,6 +22065,31 @@
       </c>
       <c r="AC208" s="1" t="n">
         <v>46149.079038125</v>
+      </c>
+      <c r="AH208" t="inlineStr">
+        <is>
+          <t>MULTI_TRACK_SYNCED_PRINTIFY_PUBLISH</t>
+        </is>
+      </c>
+      <c r="AK208" t="inlineStr">
+        <is>
+          <t>2026-05-08 08:17:21 -0400</t>
+        </is>
+      </c>
+      <c r="AL208" t="inlineStr">
+        <is>
+          <t>A_LOW_COMPETITION_NICHE</t>
+        </is>
+      </c>
+      <c r="AM208" t="inlineStr">
+        <is>
+          <t>dark study room decor</t>
+        </is>
+      </c>
+      <c r="AN208" t="inlineStr">
+        <is>
+          <t>quiet_luxury_apartment</t>
+        </is>
       </c>
     </row>
     <row r="209">
@@ -22580,7 +22713,7 @@
       </c>
       <c r="AH213" t="inlineStr">
         <is>
-          <t>MULTI_TRACK_PENDING_PRINTIFY_SYNC</t>
+          <t>MULTI_TRACK_SYNCED_PRINTIFY_PUBLISH</t>
         </is>
       </c>
       <c r="AK213" t="inlineStr">
@@ -22900,17 +23033,17 @@
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>Collector Shelf Smoky Jade Midnight Sanctuary 5x7 Acrylic Block Shelf Decor</t>
+          <t>Quiet Luxury Jade Relic Collector Smoky Midnight Sanctuary 5x7 Acrylic Block</t>
         </is>
       </c>
       <c r="F216" t="inlineStr">
         <is>
-          <t>&lt;h2&gt;Collector Shelf Smoky Jade Midnight Sanctuary 5x7 Acrylic Block Shelf Decor&lt;/h2&gt;&lt;p&gt;This listing is part of a focused search-intent experiment for collector gift. It is written for buyers decorating quiet shelves, meditation corners, gothic study desks, collector rooms, and deep-work apartments, not for generic wall-art browsing.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 5x7 vertical acrylic photo block, produced on demand through Printify.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Visual Mood:&lt;/strong&gt; Quiet Luxury Apartment.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Design Language:&lt;/strong&gt; refractive depth, smoky jade color, internal glow, and premium desk-object presence.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Search Lane:&lt;/strong&gt; acrylic photo block, desk display, shelf decor, collector gift, office decor, quiet jade, premium aesthetic, giftable decor.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; This is a single printed acrylic display block. The main artwork is the product customers receive; any additional gallery images are concept/detail references.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Acrylic-Grimdark-0031. Prior title: Collector Shelf Smoky Jade Midnight Sanctuary 5x7 Acrylic Block Shelf Decor&lt;/small&gt;&lt;/p&gt;</t>
+          <t>&lt;h2&gt;Quiet Luxury Jade Relic Collector Smoky Midnight Sanctuary 5x7 Acrylic Block&lt;/h2&gt;&lt;p&gt;This listing is part of a focused search-intent experiment for smoky jade relic. It is written for buyers decorating quiet shelves, meditation corners, gothic study desks, collector rooms, and deep-work apartments, not for generic wall-art browsing.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 5x7 vertical acrylic photo block, produced on demand through Printify.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Visual Mood:&lt;/strong&gt; Quiet Luxury Apartment.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Design Language:&lt;/strong&gt; refractive depth, smoky jade color, internal glow, and premium desk-object presence.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Search Lane:&lt;/strong&gt; gothic shelf decor, moody desk display, occult library art, dark study room decor, collector shelf object, smoky jade relic.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; This is a single printed acrylic display block. The main artwork is the product customers receive; any additional gallery images are concept/detail references.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Acrylic-Grimdark-0031. Prior title: Collector Shelf Smoky Jade Midnight Sanctuary 5x7 Acrylic Block Shelf Decor&lt;/small&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="G216" t="inlineStr">
         <is>
-          <t>$84.99</t>
+          <t>$89.99</t>
         </is>
       </c>
       <c r="H216" t="inlineStr">
@@ -23007,17 +23140,17 @@
       </c>
       <c r="AK216" t="inlineStr">
         <is>
-          <t>2026-05-07 07:37:28 -0400</t>
+          <t>2026-05-08 08:17:21 -0400</t>
         </is>
       </c>
       <c r="AL216" t="inlineStr">
         <is>
-          <t>B_HIGH_VOLUME_VALUE</t>
+          <t>A_LOW_COMPETITION_NICHE</t>
         </is>
       </c>
       <c r="AM216" t="inlineStr">
         <is>
-          <t>collector gift</t>
+          <t>smoky jade relic</t>
         </is>
       </c>
       <c r="AN216" t="inlineStr">
@@ -23049,12 +23182,12 @@
       </c>
       <c r="E217" t="inlineStr">
         <is>
-          <t>Grimdark Amber Monastery Soul Lantern 5x7 Acrylic Art Gothic Decor Golden Flame</t>
+          <t>Collector Shelf Smoky Jade Amber Monastery Soul Lantern 5x7 Acrylic Block Decor</t>
         </is>
       </c>
       <c r="F217" t="inlineStr">
         <is>
-          <t>&lt;p&gt;This Grimdark Mentor-Grade acrylic print captures the Amber Monastery Soul Lantern, an ethereal gothic artifact with a wrought iron monastery gate frame and swirling golden-orange spirit flame. The design features amber crystal inlays, floating talisman fragments, and ink-wash nebula patterns on imperial jade glass panels, all glowing with a soft amber luminescence. A refined kintsugi-like vein logic and micro-engraved surface relief create a hyper-detailed, high-end collectible aesthetic.&lt;/p&gt;&lt;p&gt;Printed on premium 5x7 acrylic, this piece delivers luminous depth and refractive light, making it ideal for a study desk, bookshelf, or dark academia-inspired wall display. The high-gloss surface and edge bevels enhance the visual impact, while the white background isolation ensures the artifact stands out in any room.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 5x7 acrylic print, ready to hang or display on a stand (stand not included)&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; High-gloss acrylic with UV-resistant inks&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Size:&lt;/strong&gt; 5x7 inches (12.7 x 17.8 cm)&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Grimdark Mentor-Grade, gothic collectible&lt;/li&gt;&lt;li&gt;&lt;strong&gt;DNA Profile:&lt;/strong&gt; Wrought Iron, Amber Crystal, Imperial Jade Glass, Talisman Fragments, Golden-Orange Flame&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Use Cases:&lt;/strong&gt; Gothic decor, study desk accent, collector display, gift for dark fantasy enthusiasts&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the actual product customers receive. Additional images are bonus concept/detail reference images and do not represent extra products or selectable variations.&lt;/p&gt;</t>
+          <t>&lt;h2&gt;Collector Shelf Smoky Jade Amber Monastery Soul Lantern 5x7 Acrylic Block Decor&lt;/h2&gt;&lt;p&gt;This listing is part of a focused search-intent experiment for collector shelf object. It is written for buyers decorating quiet shelves, meditation corners, gothic study desks, collector rooms, and deep-work apartments, not for generic wall-art browsing.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 5x7 vertical acrylic photo block, produced on demand through Printify.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Visual Mood:&lt;/strong&gt; Reading Nook Warm Lamp.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Design Language:&lt;/strong&gt; refractive depth, smoky jade color, internal glow, and premium desk-object presence.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Search Lane:&lt;/strong&gt; gothic shelf decor, moody desk display, occult library art, dark study room decor, collector shelf object, smoky jade relic.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; This is a single printed acrylic display block. The main artwork is the product customers receive; any additional gallery images are concept/detail references.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Acrylic-Grimdark-0032. Prior title: Grimdark Amber Monastery Soul Lantern 5x7 Acrylic Art Gothic Decor Golden Flame&lt;/small&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="G217" t="inlineStr">
@@ -23148,6 +23281,31 @@
       </c>
       <c r="AC217" s="1" t="n">
         <v>46149.07914980324</v>
+      </c>
+      <c r="AH217" t="inlineStr">
+        <is>
+          <t>MULTI_TRACK_SYNCED_PRINTIFY_PUBLISH</t>
+        </is>
+      </c>
+      <c r="AK217" t="inlineStr">
+        <is>
+          <t>2026-05-08 08:17:21 -0400</t>
+        </is>
+      </c>
+      <c r="AL217" t="inlineStr">
+        <is>
+          <t>A_LOW_COMPETITION_NICHE</t>
+        </is>
+      </c>
+      <c r="AM217" t="inlineStr">
+        <is>
+          <t>collector shelf object</t>
+        </is>
+      </c>
+      <c r="AN217" t="inlineStr">
+        <is>
+          <t>reading_nook_warm_lamp</t>
+        </is>
       </c>
     </row>
     <row r="218">
@@ -23275,7 +23433,7 @@
       </c>
       <c r="AH218" t="inlineStr">
         <is>
-          <t>MULTI_TRACK_PENDING_PRINTIFY_SYNC</t>
+          <t>MULTI_TRACK_SYNCED_PRINTIFY_PUBLISH</t>
         </is>
       </c>
       <c r="AK218" t="inlineStr">
@@ -23595,12 +23753,12 @@
       </c>
       <c r="E221" t="inlineStr">
         <is>
-          <t>Gothic Frost Cathedral Soul Lantern 5x7 Acrylic Display Grimdark Artifact Shelf</t>
+          <t>Quiet Luxury Jade Relic Frost Cathedral Soul Lantern 5x7 Acrylic Block Shelf</t>
         </is>
       </c>
       <c r="F221" t="inlineStr">
         <is>
-          <t>&lt;p&gt;This 5x7 acrylic print presents the &lt;strong&gt;Frost Cathedral Soul Lantern&lt;/strong&gt;, a gothic artifact that captures the grimdark mentor-grade aesthetic. The design features an ethereal lantern with a wrought-iron cathedral gate frame, aquamarine inlays, and an ice-blue spirit flame surrounded by floating talisman fragments. Ink-wash nebula patterns on imperial jade glass panels create a soft frost glow, evoking a sense of ancient mystery and refined darkness.&lt;/p&gt;&lt;p&gt;Perfect for display on a study desk, bookshelf, or altar, this acrylic piece brings a moody, collector-focused presence to any space. The high-gloss surface and edge-to-edge printing enhance the layered depth and internal bioluminescent glow, making it a standout addition to a gothic or dark academia interior.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 5x7 acrylic print with pre-installed hanging hardware (stand not included)&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; Premium acrylic with UV-resistant inks&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Size:&lt;/strong&gt; 5x7 inches (12.7 x 17.8 cm)&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Grimdark Mentor-Grade&lt;/li&gt;&lt;li&gt;&lt;strong&gt;DNA Profile:&lt;/strong&gt; Frost soul lantern, cathedral gate, aquamarine crystal, ice-blue flame, jade glass, wrought iron, talisman fragments, gothic artifact&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Use Cases:&lt;/strong&gt; Study desk decor, gothic altar piece, dark academia wall art, collector display, mentor-grade gift&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the actual product customers receive. Additional images are bonus concept/detail reference images and do not represent extra products or selectable variations.&lt;/p&gt;&lt;p&gt;&lt;em&gt;Image Note: &lt;/em&gt;&lt;/p&gt;</t>
+          <t>&lt;h2&gt;Quiet Luxury Jade Relic Frost Cathedral Soul Lantern 5x7 Acrylic Block Shelf&lt;/h2&gt;&lt;p&gt;This listing is part of a focused search-intent experiment for occult library art. It is written for buyers decorating quiet shelves, meditation corners, gothic study desks, collector rooms, and deep-work apartments, not for generic wall-art browsing.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 5x7 vertical acrylic photo block, produced on demand through Printify.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Visual Mood:&lt;/strong&gt; Quiet Luxury Apartment.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Design Language:&lt;/strong&gt; refractive depth, smoky jade color, internal glow, and premium desk-object presence.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Search Lane:&lt;/strong&gt; gothic shelf decor, moody desk display, occult library art, dark study room decor, collector shelf object, smoky jade relic.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; This is a single printed acrylic display block. The main artwork is the product customers receive; any additional gallery images are concept/detail references.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Acrylic-Grimdark-0036. Prior title: Gothic Frost Cathedral Soul Lantern 5x7 Acrylic Display Grimdark Artifact Shelf&lt;/small&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="G221" t="inlineStr">
@@ -23694,6 +23852,31 @@
       </c>
       <c r="AC221" s="1" t="n">
         <v>46149.07919978009</v>
+      </c>
+      <c r="AH221" t="inlineStr">
+        <is>
+          <t>MULTI_TRACK_SYNCED_PRINTIFY_PUBLISH</t>
+        </is>
+      </c>
+      <c r="AK221" t="inlineStr">
+        <is>
+          <t>2026-05-08 08:17:21 -0400</t>
+        </is>
+      </c>
+      <c r="AL221" t="inlineStr">
+        <is>
+          <t>A_LOW_COMPETITION_NICHE</t>
+        </is>
+      </c>
+      <c r="AM221" t="inlineStr">
+        <is>
+          <t>occult library art</t>
+        </is>
+      </c>
+      <c r="AN221" t="inlineStr">
+        <is>
+          <t>quiet_luxury_apartment</t>
+        </is>
       </c>
     </row>
     <row r="222">
@@ -23929,7 +24112,7 @@
       </c>
       <c r="AH223" t="inlineStr">
         <is>
-          <t>MULTI_TRACK_PENDING_PRINTIFY_SYNC</t>
+          <t>MULTI_TRACK_SYNCED_PRINTIFY_PUBLISH</t>
         </is>
       </c>
       <c r="AI223" t="inlineStr">
@@ -24478,7 +24661,7 @@
       </c>
       <c r="AH227" t="inlineStr">
         <is>
-          <t>MULTI_TRACK_PENDING_PRINTIFY_SYNC</t>
+          <t>MULTI_TRACK_SYNCED_PRINTIFY_PUBLISH</t>
         </is>
       </c>
       <c r="AK227" t="inlineStr">
@@ -24897,12 +25080,12 @@
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>Hermetic Knowledge Lantern Dark Academia Poster 12x18 Library Decor Wall Study</t>
+          <t>Dark Academia Reading Nook Art Hermetic Knowledge Lantern Library 12x18 Matte</t>
         </is>
       </c>
       <c r="F231" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Elevate your study or library with the Hermetic Knowledge Lantern, a dark academia poster that channels the mystique of alchemical discovery. This mentor-grade design features a corroded copper vessel with cracked glass panels, kintsugi gold seams, and toxic jade bioluminescence, capturing the essence of ancient hermetic texts in cinematic light.&lt;/p&gt;&lt;p&gt;Printed on premium semi-gloss paper, this 12x18 poster delivers rich color depth and fine detail, perfect for framing and display in a home office, reading nook, or academic workspace. The dramatic emerald glow and intricate corrosion patterns create an immersive focal point for any intellectual interior.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 12x18 poster (unframed)&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; Premium semi-gloss poster paper (200 gsm)&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Size:&lt;/strong&gt; 12 x 18 inches (30.5 x 45.7 cm)&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Dark Academia, Mentor-Grade&lt;/li&gt;&lt;li&gt;&lt;strong&gt;DNA Profile:&lt;/strong&gt; Corroded Copper, Cracked Glass, Kintsugi Gold, Toxic Jade, Ancient Parchment, brass clockwork, jade bioluminescence, alchemical dust, cinematic lighting&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Use Cases:&lt;/strong&gt; Study desk decor, library wall art, vintage collector gift, student room accent, alchemical aesthetic display&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; The main image shows the actual product customers receive. Additional images are bonus concept/detail reference images and do not represent extra products or selectable variations.&lt;/p&gt;&lt;p&gt;&lt;em&gt;Image Note: The main image shows the actual poster you will receive. Additional images are bonus concept and detail reference images; they do not represent extra products or selectable variations.&lt;/em&gt;&lt;/p&gt;</t>
+          <t>&lt;h2&gt;Dark Academia Reading Nook Art Hermetic Knowledge Lantern Library 12x18 Matte&lt;/h2&gt;&lt;p&gt;This listing is part of a focused search-intent experiment for home library wall art. It is written for buyers decorating reading nooks, home libraries, dorm study walls, meditation rooms, and quiet apartment corners, not for generic wall-art browsing.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; One 12x18 matte poster, produced on demand through Printify.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Visual Mood:&lt;/strong&gt; Reading Nook Warm Lamp.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Design Language:&lt;/strong&gt; matte paper mood, cinematic depth, smoky jade tones, and calm visual focus.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Search Lane:&lt;/strong&gt; dark academia reading nook, home library wall art, book nook decor, study room poster, scholar desk decor, dorm library print.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong&gt;Image Note:&lt;/strong&gt; This is a single printed poster. The main artwork is the product customers receive; any additional gallery images are concept/detail references.&lt;/p&gt;&lt;p&gt;&lt;small&gt;Reference SKU: Poster-Academia-0023. Prior title: Hermetic Knowledge Lantern Dark Academia Poster 12x18 Library Decor Wall Study&lt;/small&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="G231" t="inlineStr">
@@ -24996,6 +25179,31 @@
       </c>
       <c r="AC231" s="1" t="n">
         <v>46149.07928880787</v>
+      </c>
+      <c r="AH231" t="inlineStr">
+        <is>
+          <t>MULTI_TRACK_SYNCED_PRINTIFY_PUBLISH</t>
+        </is>
+      </c>
+      <c r="AK231" t="inlineStr">
+        <is>
+          <t>2026-05-08 08:17:21 -0400</t>
+        </is>
+      </c>
+      <c r="AL231" t="inlineStr">
+        <is>
+          <t>A_LOW_COMPETITION_NICHE</t>
+        </is>
+      </c>
+      <c r="AM231" t="inlineStr">
+        <is>
+          <t>home library wall art</t>
+        </is>
+      </c>
+      <c r="AN231" t="inlineStr">
+        <is>
+          <t>reading_nook_warm_lamp</t>
+        </is>
       </c>
     </row>
     <row r="232">
@@ -29528,7 +29736,7 @@
       </c>
       <c r="AH268" t="inlineStr">
         <is>
-          <t>MULTI_TRACK_PENDING_PRINTIFY_SYNC</t>
+          <t>MULTI_TRACK_SYNCED_PRINTIFY_PUBLISH</t>
         </is>
       </c>
       <c r="AK268" t="inlineStr">

</xml_diff>